<commit_message>
KRW: add the Date column from Kevin's spec
Kevin's requested table is Date, Year, Swap Rate, Zero Rate, Discount Factor,
Forward Rate - the Date column was the one thing missing. Added it as column A,
rolling quarterly off a curve-date input on Quotes!E2 (default 07/23/2026, his
email date). EDATE(curve date, 3*node) so 0.25y is three months out.

Confirmed the method already matches his three steps exactly: 3m zero -> 3m DF,
6m swap -> 6m DF by the par identity, then zero and forward off the DFs.

Verified after the column shift: every checked DF still matches the hand
bootstrap to 7 decimals, dates land on quarterly rolls, zero errors.

Simplification unchanged and worth stating to Kevin: dates are shown for the
column but the year fractions are still tau = 0.25 flat, not actual ACT/365 day
counts between those dates.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -18,10 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="168" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -117,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,6 +138,8 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -501,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -524,6 +528,14 @@
       </c>
       <c r="B2" s="3" t="n">
         <v>0.25</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>curve date</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="n">
+        <v>46226</v>
       </c>
     </row>
     <row r="4">
@@ -4301,2680 +4313,3166 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E122"/>
+  <dimension ref="A2:F122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Swap %</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>DF</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Zero %</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Future %</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6">
+      <c r="A3" s="15">
+        <f>EDATE(Quotes!$E$2,3*1)</f>
+        <v/>
+      </c>
+      <c r="B3" s="6">
         <f>Interpolation!A3</f>
         <v/>
       </c>
-      <c r="B3" s="12">
+      <c r="C3" s="12">
         <f>Interpolation!E3</f>
         <v/>
       </c>
-      <c r="C3" s="13">
-        <f>1/(1+B3*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D3" s="10">
-        <f>(1/C3-1)/A3</f>
+      <c r="D3" s="13">
+        <f>1/(1+C3*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E3" s="10">
-        <f>(1/C3-1)/Quotes!$B$2</f>
+        <f>(1/D3-1)/B3</f>
+        <v/>
+      </c>
+      <c r="F3" s="10">
+        <f>(1/D3-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="15">
+        <f>EDATE(Quotes!$E$2,3*2)</f>
+        <v/>
+      </c>
+      <c r="B4" s="6">
         <f>Interpolation!A4</f>
         <v/>
       </c>
-      <c r="B4" s="12">
+      <c r="C4" s="12">
         <f>Interpolation!E4</f>
         <v/>
       </c>
-      <c r="C4" s="13">
-        <f>(1-B4*Quotes!$B$2*SUM($C$3:C3))/(1+B4*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D4" s="10">
-        <f>(1/C4-1)/A4</f>
+      <c r="D4" s="13">
+        <f>(1-C4*Quotes!$B$2*SUM($D$3:D3))/(1+C4*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E4" s="10">
-        <f>(C3/C4-1)/Quotes!$B$2</f>
+        <f>(1/D4-1)/B4</f>
+        <v/>
+      </c>
+      <c r="F4" s="10">
+        <f>(D3/D4-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6">
+      <c r="A5" s="15">
+        <f>EDATE(Quotes!$E$2,3*3)</f>
+        <v/>
+      </c>
+      <c r="B5" s="6">
         <f>Interpolation!A5</f>
         <v/>
       </c>
-      <c r="B5" s="12">
+      <c r="C5" s="12">
         <f>Interpolation!E5</f>
         <v/>
       </c>
-      <c r="C5" s="13">
-        <f>(1-B5*Quotes!$B$2*SUM($C$3:C4))/(1+B5*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D5" s="10">
-        <f>(1/C5-1)/A5</f>
+      <c r="D5" s="13">
+        <f>(1-C5*Quotes!$B$2*SUM($D$3:D4))/(1+C5*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>(C4/C5-1)/Quotes!$B$2</f>
+        <f>(1/D5-1)/B5</f>
+        <v/>
+      </c>
+      <c r="F5" s="10">
+        <f>(D4/D5-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6">
+      <c r="A6" s="15">
+        <f>EDATE(Quotes!$E$2,3*4)</f>
+        <v/>
+      </c>
+      <c r="B6" s="6">
         <f>Interpolation!A6</f>
         <v/>
       </c>
-      <c r="B6" s="12">
+      <c r="C6" s="12">
         <f>Interpolation!E6</f>
         <v/>
       </c>
-      <c r="C6" s="13">
-        <f>(1-B6*Quotes!$B$2*SUM($C$3:C5))/(1+B6*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D6" s="10">
-        <f>(1/C6-1)/A6</f>
+      <c r="D6" s="13">
+        <f>(1-C6*Quotes!$B$2*SUM($D$3:D5))/(1+C6*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E6" s="10">
-        <f>(C5/C6-1)/Quotes!$B$2</f>
+        <f>(1/D6-1)/B6</f>
+        <v/>
+      </c>
+      <c r="F6" s="10">
+        <f>(D5/D6-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6">
+      <c r="A7" s="15">
+        <f>EDATE(Quotes!$E$2,3*5)</f>
+        <v/>
+      </c>
+      <c r="B7" s="6">
         <f>Interpolation!A7</f>
         <v/>
       </c>
-      <c r="B7" s="12">
+      <c r="C7" s="12">
         <f>Interpolation!E7</f>
         <v/>
       </c>
-      <c r="C7" s="13">
-        <f>(1-B7*Quotes!$B$2*SUM($C$3:C6))/(1+B7*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D7" s="10">
-        <f>(1/C7-1)/A7</f>
+      <c r="D7" s="13">
+        <f>(1-C7*Quotes!$B$2*SUM($D$3:D6))/(1+C7*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>(C6/C7-1)/Quotes!$B$2</f>
+        <f>(1/D7-1)/B7</f>
+        <v/>
+      </c>
+      <c r="F7" s="10">
+        <f>(D6/D7-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6">
+      <c r="A8" s="15">
+        <f>EDATE(Quotes!$E$2,3*6)</f>
+        <v/>
+      </c>
+      <c r="B8" s="6">
         <f>Interpolation!A8</f>
         <v/>
       </c>
-      <c r="B8" s="12">
+      <c r="C8" s="12">
         <f>Interpolation!E8</f>
         <v/>
       </c>
-      <c r="C8" s="13">
-        <f>(1-B8*Quotes!$B$2*SUM($C$3:C7))/(1+B8*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D8" s="10">
-        <f>(1/C8-1)/A8</f>
+      <c r="D8" s="13">
+        <f>(1-C8*Quotes!$B$2*SUM($D$3:D7))/(1+C8*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E8" s="10">
-        <f>(C7/C8-1)/Quotes!$B$2</f>
+        <f>(1/D8-1)/B8</f>
+        <v/>
+      </c>
+      <c r="F8" s="10">
+        <f>(D7/D8-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6">
+      <c r="A9" s="15">
+        <f>EDATE(Quotes!$E$2,3*7)</f>
+        <v/>
+      </c>
+      <c r="B9" s="6">
         <f>Interpolation!A9</f>
         <v/>
       </c>
-      <c r="B9" s="12">
+      <c r="C9" s="12">
         <f>Interpolation!E9</f>
         <v/>
       </c>
-      <c r="C9" s="13">
-        <f>(1-B9*Quotes!$B$2*SUM($C$3:C8))/(1+B9*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D9" s="10">
-        <f>(1/C9-1)/A9</f>
+      <c r="D9" s="13">
+        <f>(1-C9*Quotes!$B$2*SUM($D$3:D8))/(1+C9*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>(C8/C9-1)/Quotes!$B$2</f>
+        <f>(1/D9-1)/B9</f>
+        <v/>
+      </c>
+      <c r="F9" s="10">
+        <f>(D8/D9-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6">
+      <c r="A10" s="15">
+        <f>EDATE(Quotes!$E$2,3*8)</f>
+        <v/>
+      </c>
+      <c r="B10" s="6">
         <f>Interpolation!A10</f>
         <v/>
       </c>
-      <c r="B10" s="12">
+      <c r="C10" s="12">
         <f>Interpolation!E10</f>
         <v/>
       </c>
-      <c r="C10" s="13">
-        <f>(1-B10*Quotes!$B$2*SUM($C$3:C9))/(1+B10*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D10" s="10">
-        <f>(1/C10-1)/A10</f>
+      <c r="D10" s="13">
+        <f>(1-C10*Quotes!$B$2*SUM($D$3:D9))/(1+C10*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E10" s="10">
-        <f>(C9/C10-1)/Quotes!$B$2</f>
+        <f>(1/D10-1)/B10</f>
+        <v/>
+      </c>
+      <c r="F10" s="10">
+        <f>(D9/D10-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6">
+      <c r="A11" s="15">
+        <f>EDATE(Quotes!$E$2,3*9)</f>
+        <v/>
+      </c>
+      <c r="B11" s="6">
         <f>Interpolation!A11</f>
         <v/>
       </c>
-      <c r="B11" s="12">
+      <c r="C11" s="12">
         <f>Interpolation!E11</f>
         <v/>
       </c>
-      <c r="C11" s="13">
-        <f>(1-B11*Quotes!$B$2*SUM($C$3:C10))/(1+B11*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D11" s="10">
-        <f>(1/C11-1)/A11</f>
+      <c r="D11" s="13">
+        <f>(1-C11*Quotes!$B$2*SUM($D$3:D10))/(1+C11*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>(C10/C11-1)/Quotes!$B$2</f>
+        <f>(1/D11-1)/B11</f>
+        <v/>
+      </c>
+      <c r="F11" s="10">
+        <f>(D10/D11-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6">
+      <c r="A12" s="15">
+        <f>EDATE(Quotes!$E$2,3*10)</f>
+        <v/>
+      </c>
+      <c r="B12" s="6">
         <f>Interpolation!A12</f>
         <v/>
       </c>
-      <c r="B12" s="12">
+      <c r="C12" s="12">
         <f>Interpolation!E12</f>
         <v/>
       </c>
-      <c r="C12" s="13">
-        <f>(1-B12*Quotes!$B$2*SUM($C$3:C11))/(1+B12*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D12" s="10">
-        <f>(1/C12-1)/A12</f>
+      <c r="D12" s="13">
+        <f>(1-C12*Quotes!$B$2*SUM($D$3:D11))/(1+C12*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E12" s="10">
-        <f>(C11/C12-1)/Quotes!$B$2</f>
+        <f>(1/D12-1)/B12</f>
+        <v/>
+      </c>
+      <c r="F12" s="10">
+        <f>(D11/D12-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6">
+      <c r="A13" s="15">
+        <f>EDATE(Quotes!$E$2,3*11)</f>
+        <v/>
+      </c>
+      <c r="B13" s="6">
         <f>Interpolation!A13</f>
         <v/>
       </c>
-      <c r="B13" s="12">
+      <c r="C13" s="12">
         <f>Interpolation!E13</f>
         <v/>
       </c>
-      <c r="C13" s="13">
-        <f>(1-B13*Quotes!$B$2*SUM($C$3:C12))/(1+B13*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D13" s="10">
-        <f>(1/C13-1)/A13</f>
+      <c r="D13" s="13">
+        <f>(1-C13*Quotes!$B$2*SUM($D$3:D12))/(1+C13*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>(C12/C13-1)/Quotes!$B$2</f>
+        <f>(1/D13-1)/B13</f>
+        <v/>
+      </c>
+      <c r="F13" s="10">
+        <f>(D12/D13-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6">
+      <c r="A14" s="15">
+        <f>EDATE(Quotes!$E$2,3*12)</f>
+        <v/>
+      </c>
+      <c r="B14" s="6">
         <f>Interpolation!A14</f>
         <v/>
       </c>
-      <c r="B14" s="12">
+      <c r="C14" s="12">
         <f>Interpolation!E14</f>
         <v/>
       </c>
-      <c r="C14" s="13">
-        <f>(1-B14*Quotes!$B$2*SUM($C$3:C13))/(1+B14*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D14" s="10">
-        <f>(1/C14-1)/A14</f>
+      <c r="D14" s="13">
+        <f>(1-C14*Quotes!$B$2*SUM($D$3:D13))/(1+C14*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E14" s="10">
-        <f>(C13/C14-1)/Quotes!$B$2</f>
+        <f>(1/D14-1)/B14</f>
+        <v/>
+      </c>
+      <c r="F14" s="10">
+        <f>(D13/D14-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6">
+      <c r="A15" s="15">
+        <f>EDATE(Quotes!$E$2,3*13)</f>
+        <v/>
+      </c>
+      <c r="B15" s="6">
         <f>Interpolation!A15</f>
         <v/>
       </c>
-      <c r="B15" s="12">
+      <c r="C15" s="12">
         <f>Interpolation!E15</f>
         <v/>
       </c>
-      <c r="C15" s="13">
-        <f>(1-B15*Quotes!$B$2*SUM($C$3:C14))/(1+B15*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D15" s="10">
-        <f>(1/C15-1)/A15</f>
+      <c r="D15" s="13">
+        <f>(1-C15*Quotes!$B$2*SUM($D$3:D14))/(1+C15*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E15" s="10">
-        <f>(C14/C15-1)/Quotes!$B$2</f>
+        <f>(1/D15-1)/B15</f>
+        <v/>
+      </c>
+      <c r="F15" s="10">
+        <f>(D14/D15-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6">
+      <c r="A16" s="15">
+        <f>EDATE(Quotes!$E$2,3*14)</f>
+        <v/>
+      </c>
+      <c r="B16" s="6">
         <f>Interpolation!A16</f>
         <v/>
       </c>
-      <c r="B16" s="12">
+      <c r="C16" s="12">
         <f>Interpolation!E16</f>
         <v/>
       </c>
-      <c r="C16" s="13">
-        <f>(1-B16*Quotes!$B$2*SUM($C$3:C15))/(1+B16*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D16" s="10">
-        <f>(1/C16-1)/A16</f>
+      <c r="D16" s="13">
+        <f>(1-C16*Quotes!$B$2*SUM($D$3:D15))/(1+C16*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E16" s="10">
-        <f>(C15/C16-1)/Quotes!$B$2</f>
+        <f>(1/D16-1)/B16</f>
+        <v/>
+      </c>
+      <c r="F16" s="10">
+        <f>(D15/D16-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6">
+      <c r="A17" s="15">
+        <f>EDATE(Quotes!$E$2,3*15)</f>
+        <v/>
+      </c>
+      <c r="B17" s="6">
         <f>Interpolation!A17</f>
         <v/>
       </c>
-      <c r="B17" s="12">
+      <c r="C17" s="12">
         <f>Interpolation!E17</f>
         <v/>
       </c>
-      <c r="C17" s="13">
-        <f>(1-B17*Quotes!$B$2*SUM($C$3:C16))/(1+B17*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D17" s="10">
-        <f>(1/C17-1)/A17</f>
+      <c r="D17" s="13">
+        <f>(1-C17*Quotes!$B$2*SUM($D$3:D16))/(1+C17*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>(C16/C17-1)/Quotes!$B$2</f>
+        <f>(1/D17-1)/B17</f>
+        <v/>
+      </c>
+      <c r="F17" s="10">
+        <f>(D16/D17-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6">
+      <c r="A18" s="15">
+        <f>EDATE(Quotes!$E$2,3*16)</f>
+        <v/>
+      </c>
+      <c r="B18" s="6">
         <f>Interpolation!A18</f>
         <v/>
       </c>
-      <c r="B18" s="12">
+      <c r="C18" s="12">
         <f>Interpolation!E18</f>
         <v/>
       </c>
-      <c r="C18" s="13">
-        <f>(1-B18*Quotes!$B$2*SUM($C$3:C17))/(1+B18*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D18" s="10">
-        <f>(1/C18-1)/A18</f>
+      <c r="D18" s="13">
+        <f>(1-C18*Quotes!$B$2*SUM($D$3:D17))/(1+C18*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>(C17/C18-1)/Quotes!$B$2</f>
+        <f>(1/D18-1)/B18</f>
+        <v/>
+      </c>
+      <c r="F18" s="10">
+        <f>(D17/D18-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6">
+      <c r="A19" s="15">
+        <f>EDATE(Quotes!$E$2,3*17)</f>
+        <v/>
+      </c>
+      <c r="B19" s="6">
         <f>Interpolation!A19</f>
         <v/>
       </c>
-      <c r="B19" s="12">
+      <c r="C19" s="12">
         <f>Interpolation!E19</f>
         <v/>
       </c>
-      <c r="C19" s="13">
-        <f>(1-B19*Quotes!$B$2*SUM($C$3:C18))/(1+B19*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D19" s="10">
-        <f>(1/C19-1)/A19</f>
+      <c r="D19" s="13">
+        <f>(1-C19*Quotes!$B$2*SUM($D$3:D18))/(1+C19*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>(C18/C19-1)/Quotes!$B$2</f>
+        <f>(1/D19-1)/B19</f>
+        <v/>
+      </c>
+      <c r="F19" s="10">
+        <f>(D18/D19-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6">
+      <c r="A20" s="15">
+        <f>EDATE(Quotes!$E$2,3*18)</f>
+        <v/>
+      </c>
+      <c r="B20" s="6">
         <f>Interpolation!A20</f>
         <v/>
       </c>
-      <c r="B20" s="12">
+      <c r="C20" s="12">
         <f>Interpolation!E20</f>
         <v/>
       </c>
-      <c r="C20" s="13">
-        <f>(1-B20*Quotes!$B$2*SUM($C$3:C19))/(1+B20*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D20" s="10">
-        <f>(1/C20-1)/A20</f>
+      <c r="D20" s="13">
+        <f>(1-C20*Quotes!$B$2*SUM($D$3:D19))/(1+C20*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E20" s="10">
-        <f>(C19/C20-1)/Quotes!$B$2</f>
+        <f>(1/D20-1)/B20</f>
+        <v/>
+      </c>
+      <c r="F20" s="10">
+        <f>(D19/D20-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6">
+      <c r="A21" s="15">
+        <f>EDATE(Quotes!$E$2,3*19)</f>
+        <v/>
+      </c>
+      <c r="B21" s="6">
         <f>Interpolation!A21</f>
         <v/>
       </c>
-      <c r="B21" s="12">
+      <c r="C21" s="12">
         <f>Interpolation!E21</f>
         <v/>
       </c>
-      <c r="C21" s="13">
-        <f>(1-B21*Quotes!$B$2*SUM($C$3:C20))/(1+B21*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D21" s="10">
-        <f>(1/C21-1)/A21</f>
+      <c r="D21" s="13">
+        <f>(1-C21*Quotes!$B$2*SUM($D$3:D20))/(1+C21*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>(C20/C21-1)/Quotes!$B$2</f>
+        <f>(1/D21-1)/B21</f>
+        <v/>
+      </c>
+      <c r="F21" s="10">
+        <f>(D20/D21-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6">
+      <c r="A22" s="15">
+        <f>EDATE(Quotes!$E$2,3*20)</f>
+        <v/>
+      </c>
+      <c r="B22" s="6">
         <f>Interpolation!A22</f>
         <v/>
       </c>
-      <c r="B22" s="12">
+      <c r="C22" s="12">
         <f>Interpolation!E22</f>
         <v/>
       </c>
-      <c r="C22" s="13">
-        <f>(1-B22*Quotes!$B$2*SUM($C$3:C21))/(1+B22*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D22" s="10">
-        <f>(1/C22-1)/A22</f>
+      <c r="D22" s="13">
+        <f>(1-C22*Quotes!$B$2*SUM($D$3:D21))/(1+C22*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>(C21/C22-1)/Quotes!$B$2</f>
+        <f>(1/D22-1)/B22</f>
+        <v/>
+      </c>
+      <c r="F22" s="10">
+        <f>(D21/D22-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6">
+      <c r="A23" s="15">
+        <f>EDATE(Quotes!$E$2,3*21)</f>
+        <v/>
+      </c>
+      <c r="B23" s="6">
         <f>Interpolation!A23</f>
         <v/>
       </c>
-      <c r="B23" s="12">
+      <c r="C23" s="12">
         <f>Interpolation!E23</f>
         <v/>
       </c>
-      <c r="C23" s="13">
-        <f>(1-B23*Quotes!$B$2*SUM($C$3:C22))/(1+B23*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D23" s="10">
-        <f>(1/C23-1)/A23</f>
+      <c r="D23" s="13">
+        <f>(1-C23*Quotes!$B$2*SUM($D$3:D22))/(1+C23*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E23" s="10">
-        <f>(C22/C23-1)/Quotes!$B$2</f>
+        <f>(1/D23-1)/B23</f>
+        <v/>
+      </c>
+      <c r="F23" s="10">
+        <f>(D22/D23-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6">
+      <c r="A24" s="15">
+        <f>EDATE(Quotes!$E$2,3*22)</f>
+        <v/>
+      </c>
+      <c r="B24" s="6">
         <f>Interpolation!A24</f>
         <v/>
       </c>
-      <c r="B24" s="12">
+      <c r="C24" s="12">
         <f>Interpolation!E24</f>
         <v/>
       </c>
-      <c r="C24" s="13">
-        <f>(1-B24*Quotes!$B$2*SUM($C$3:C23))/(1+B24*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D24" s="10">
-        <f>(1/C24-1)/A24</f>
+      <c r="D24" s="13">
+        <f>(1-C24*Quotes!$B$2*SUM($D$3:D23))/(1+C24*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E24" s="10">
-        <f>(C23/C24-1)/Quotes!$B$2</f>
+        <f>(1/D24-1)/B24</f>
+        <v/>
+      </c>
+      <c r="F24" s="10">
+        <f>(D23/D24-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6">
+      <c r="A25" s="15">
+        <f>EDATE(Quotes!$E$2,3*23)</f>
+        <v/>
+      </c>
+      <c r="B25" s="6">
         <f>Interpolation!A25</f>
         <v/>
       </c>
-      <c r="B25" s="12">
+      <c r="C25" s="12">
         <f>Interpolation!E25</f>
         <v/>
       </c>
-      <c r="C25" s="13">
-        <f>(1-B25*Quotes!$B$2*SUM($C$3:C24))/(1+B25*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D25" s="10">
-        <f>(1/C25-1)/A25</f>
+      <c r="D25" s="13">
+        <f>(1-C25*Quotes!$B$2*SUM($D$3:D24))/(1+C25*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E25" s="10">
-        <f>(C24/C25-1)/Quotes!$B$2</f>
+        <f>(1/D25-1)/B25</f>
+        <v/>
+      </c>
+      <c r="F25" s="10">
+        <f>(D24/D25-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6">
+      <c r="A26" s="15">
+        <f>EDATE(Quotes!$E$2,3*24)</f>
+        <v/>
+      </c>
+      <c r="B26" s="6">
         <f>Interpolation!A26</f>
         <v/>
       </c>
-      <c r="B26" s="12">
+      <c r="C26" s="12">
         <f>Interpolation!E26</f>
         <v/>
       </c>
-      <c r="C26" s="13">
-        <f>(1-B26*Quotes!$B$2*SUM($C$3:C25))/(1+B26*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D26" s="10">
-        <f>(1/C26-1)/A26</f>
+      <c r="D26" s="13">
+        <f>(1-C26*Quotes!$B$2*SUM($D$3:D25))/(1+C26*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E26" s="10">
-        <f>(C25/C26-1)/Quotes!$B$2</f>
+        <f>(1/D26-1)/B26</f>
+        <v/>
+      </c>
+      <c r="F26" s="10">
+        <f>(D25/D26-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6">
+      <c r="A27" s="15">
+        <f>EDATE(Quotes!$E$2,3*25)</f>
+        <v/>
+      </c>
+      <c r="B27" s="6">
         <f>Interpolation!A27</f>
         <v/>
       </c>
-      <c r="B27" s="12">
+      <c r="C27" s="12">
         <f>Interpolation!E27</f>
         <v/>
       </c>
-      <c r="C27" s="13">
-        <f>(1-B27*Quotes!$B$2*SUM($C$3:C26))/(1+B27*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D27" s="10">
-        <f>(1/C27-1)/A27</f>
+      <c r="D27" s="13">
+        <f>(1-C27*Quotes!$B$2*SUM($D$3:D26))/(1+C27*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E27" s="10">
-        <f>(C26/C27-1)/Quotes!$B$2</f>
+        <f>(1/D27-1)/B27</f>
+        <v/>
+      </c>
+      <c r="F27" s="10">
+        <f>(D26/D27-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6">
+      <c r="A28" s="15">
+        <f>EDATE(Quotes!$E$2,3*26)</f>
+        <v/>
+      </c>
+      <c r="B28" s="6">
         <f>Interpolation!A28</f>
         <v/>
       </c>
-      <c r="B28" s="12">
+      <c r="C28" s="12">
         <f>Interpolation!E28</f>
         <v/>
       </c>
-      <c r="C28" s="13">
-        <f>(1-B28*Quotes!$B$2*SUM($C$3:C27))/(1+B28*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D28" s="10">
-        <f>(1/C28-1)/A28</f>
+      <c r="D28" s="13">
+        <f>(1-C28*Quotes!$B$2*SUM($D$3:D27))/(1+C28*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E28" s="10">
-        <f>(C27/C28-1)/Quotes!$B$2</f>
+        <f>(1/D28-1)/B28</f>
+        <v/>
+      </c>
+      <c r="F28" s="10">
+        <f>(D27/D28-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6">
+      <c r="A29" s="15">
+        <f>EDATE(Quotes!$E$2,3*27)</f>
+        <v/>
+      </c>
+      <c r="B29" s="6">
         <f>Interpolation!A29</f>
         <v/>
       </c>
-      <c r="B29" s="12">
+      <c r="C29" s="12">
         <f>Interpolation!E29</f>
         <v/>
       </c>
-      <c r="C29" s="13">
-        <f>(1-B29*Quotes!$B$2*SUM($C$3:C28))/(1+B29*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D29" s="10">
-        <f>(1/C29-1)/A29</f>
+      <c r="D29" s="13">
+        <f>(1-C29*Quotes!$B$2*SUM($D$3:D28))/(1+C29*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E29" s="10">
-        <f>(C28/C29-1)/Quotes!$B$2</f>
+        <f>(1/D29-1)/B29</f>
+        <v/>
+      </c>
+      <c r="F29" s="10">
+        <f>(D28/D29-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6">
+      <c r="A30" s="15">
+        <f>EDATE(Quotes!$E$2,3*28)</f>
+        <v/>
+      </c>
+      <c r="B30" s="6">
         <f>Interpolation!A30</f>
         <v/>
       </c>
-      <c r="B30" s="12">
+      <c r="C30" s="12">
         <f>Interpolation!E30</f>
         <v/>
       </c>
-      <c r="C30" s="13">
-        <f>(1-B30*Quotes!$B$2*SUM($C$3:C29))/(1+B30*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D30" s="10">
-        <f>(1/C30-1)/A30</f>
+      <c r="D30" s="13">
+        <f>(1-C30*Quotes!$B$2*SUM($D$3:D29))/(1+C30*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E30" s="10">
-        <f>(C29/C30-1)/Quotes!$B$2</f>
+        <f>(1/D30-1)/B30</f>
+        <v/>
+      </c>
+      <c r="F30" s="10">
+        <f>(D29/D30-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6">
+      <c r="A31" s="15">
+        <f>EDATE(Quotes!$E$2,3*29)</f>
+        <v/>
+      </c>
+      <c r="B31" s="6">
         <f>Interpolation!A31</f>
         <v/>
       </c>
-      <c r="B31" s="12">
+      <c r="C31" s="12">
         <f>Interpolation!E31</f>
         <v/>
       </c>
-      <c r="C31" s="13">
-        <f>(1-B31*Quotes!$B$2*SUM($C$3:C30))/(1+B31*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D31" s="10">
-        <f>(1/C31-1)/A31</f>
+      <c r="D31" s="13">
+        <f>(1-C31*Quotes!$B$2*SUM($D$3:D30))/(1+C31*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E31" s="10">
-        <f>(C30/C31-1)/Quotes!$B$2</f>
+        <f>(1/D31-1)/B31</f>
+        <v/>
+      </c>
+      <c r="F31" s="10">
+        <f>(D30/D31-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6">
+      <c r="A32" s="15">
+        <f>EDATE(Quotes!$E$2,3*30)</f>
+        <v/>
+      </c>
+      <c r="B32" s="6">
         <f>Interpolation!A32</f>
         <v/>
       </c>
-      <c r="B32" s="12">
+      <c r="C32" s="12">
         <f>Interpolation!E32</f>
         <v/>
       </c>
-      <c r="C32" s="13">
-        <f>(1-B32*Quotes!$B$2*SUM($C$3:C31))/(1+B32*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D32" s="10">
-        <f>(1/C32-1)/A32</f>
+      <c r="D32" s="13">
+        <f>(1-C32*Quotes!$B$2*SUM($D$3:D31))/(1+C32*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E32" s="10">
-        <f>(C31/C32-1)/Quotes!$B$2</f>
+        <f>(1/D32-1)/B32</f>
+        <v/>
+      </c>
+      <c r="F32" s="10">
+        <f>(D31/D32-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6">
+      <c r="A33" s="15">
+        <f>EDATE(Quotes!$E$2,3*31)</f>
+        <v/>
+      </c>
+      <c r="B33" s="6">
         <f>Interpolation!A33</f>
         <v/>
       </c>
-      <c r="B33" s="12">
+      <c r="C33" s="12">
         <f>Interpolation!E33</f>
         <v/>
       </c>
-      <c r="C33" s="13">
-        <f>(1-B33*Quotes!$B$2*SUM($C$3:C32))/(1+B33*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D33" s="10">
-        <f>(1/C33-1)/A33</f>
+      <c r="D33" s="13">
+        <f>(1-C33*Quotes!$B$2*SUM($D$3:D32))/(1+C33*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E33" s="10">
-        <f>(C32/C33-1)/Quotes!$B$2</f>
+        <f>(1/D33-1)/B33</f>
+        <v/>
+      </c>
+      <c r="F33" s="10">
+        <f>(D32/D33-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6">
+      <c r="A34" s="15">
+        <f>EDATE(Quotes!$E$2,3*32)</f>
+        <v/>
+      </c>
+      <c r="B34" s="6">
         <f>Interpolation!A34</f>
         <v/>
       </c>
-      <c r="B34" s="12">
+      <c r="C34" s="12">
         <f>Interpolation!E34</f>
         <v/>
       </c>
-      <c r="C34" s="13">
-        <f>(1-B34*Quotes!$B$2*SUM($C$3:C33))/(1+B34*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D34" s="10">
-        <f>(1/C34-1)/A34</f>
+      <c r="D34" s="13">
+        <f>(1-C34*Quotes!$B$2*SUM($D$3:D33))/(1+C34*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E34" s="10">
-        <f>(C33/C34-1)/Quotes!$B$2</f>
+        <f>(1/D34-1)/B34</f>
+        <v/>
+      </c>
+      <c r="F34" s="10">
+        <f>(D33/D34-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6">
+      <c r="A35" s="15">
+        <f>EDATE(Quotes!$E$2,3*33)</f>
+        <v/>
+      </c>
+      <c r="B35" s="6">
         <f>Interpolation!A35</f>
         <v/>
       </c>
-      <c r="B35" s="12">
+      <c r="C35" s="12">
         <f>Interpolation!E35</f>
         <v/>
       </c>
-      <c r="C35" s="13">
-        <f>(1-B35*Quotes!$B$2*SUM($C$3:C34))/(1+B35*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D35" s="10">
-        <f>(1/C35-1)/A35</f>
+      <c r="D35" s="13">
+        <f>(1-C35*Quotes!$B$2*SUM($D$3:D34))/(1+C35*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E35" s="10">
-        <f>(C34/C35-1)/Quotes!$B$2</f>
+        <f>(1/D35-1)/B35</f>
+        <v/>
+      </c>
+      <c r="F35" s="10">
+        <f>(D34/D35-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6">
+      <c r="A36" s="15">
+        <f>EDATE(Quotes!$E$2,3*34)</f>
+        <v/>
+      </c>
+      <c r="B36" s="6">
         <f>Interpolation!A36</f>
         <v/>
       </c>
-      <c r="B36" s="12">
+      <c r="C36" s="12">
         <f>Interpolation!E36</f>
         <v/>
       </c>
-      <c r="C36" s="13">
-        <f>(1-B36*Quotes!$B$2*SUM($C$3:C35))/(1+B36*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D36" s="10">
-        <f>(1/C36-1)/A36</f>
+      <c r="D36" s="13">
+        <f>(1-C36*Quotes!$B$2*SUM($D$3:D35))/(1+C36*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E36" s="10">
-        <f>(C35/C36-1)/Quotes!$B$2</f>
+        <f>(1/D36-1)/B36</f>
+        <v/>
+      </c>
+      <c r="F36" s="10">
+        <f>(D35/D36-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6">
+      <c r="A37" s="15">
+        <f>EDATE(Quotes!$E$2,3*35)</f>
+        <v/>
+      </c>
+      <c r="B37" s="6">
         <f>Interpolation!A37</f>
         <v/>
       </c>
-      <c r="B37" s="12">
+      <c r="C37" s="12">
         <f>Interpolation!E37</f>
         <v/>
       </c>
-      <c r="C37" s="13">
-        <f>(1-B37*Quotes!$B$2*SUM($C$3:C36))/(1+B37*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D37" s="10">
-        <f>(1/C37-1)/A37</f>
+      <c r="D37" s="13">
+        <f>(1-C37*Quotes!$B$2*SUM($D$3:D36))/(1+C37*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E37" s="10">
-        <f>(C36/C37-1)/Quotes!$B$2</f>
+        <f>(1/D37-1)/B37</f>
+        <v/>
+      </c>
+      <c r="F37" s="10">
+        <f>(D36/D37-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6">
+      <c r="A38" s="15">
+        <f>EDATE(Quotes!$E$2,3*36)</f>
+        <v/>
+      </c>
+      <c r="B38" s="6">
         <f>Interpolation!A38</f>
         <v/>
       </c>
-      <c r="B38" s="12">
+      <c r="C38" s="12">
         <f>Interpolation!E38</f>
         <v/>
       </c>
-      <c r="C38" s="13">
-        <f>(1-B38*Quotes!$B$2*SUM($C$3:C37))/(1+B38*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D38" s="10">
-        <f>(1/C38-1)/A38</f>
+      <c r="D38" s="13">
+        <f>(1-C38*Quotes!$B$2*SUM($D$3:D37))/(1+C38*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E38" s="10">
-        <f>(C37/C38-1)/Quotes!$B$2</f>
+        <f>(1/D38-1)/B38</f>
+        <v/>
+      </c>
+      <c r="F38" s="10">
+        <f>(D37/D38-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6">
+      <c r="A39" s="15">
+        <f>EDATE(Quotes!$E$2,3*37)</f>
+        <v/>
+      </c>
+      <c r="B39" s="6">
         <f>Interpolation!A39</f>
         <v/>
       </c>
-      <c r="B39" s="12">
+      <c r="C39" s="12">
         <f>Interpolation!E39</f>
         <v/>
       </c>
-      <c r="C39" s="13">
-        <f>(1-B39*Quotes!$B$2*SUM($C$3:C38))/(1+B39*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D39" s="10">
-        <f>(1/C39-1)/A39</f>
+      <c r="D39" s="13">
+        <f>(1-C39*Quotes!$B$2*SUM($D$3:D38))/(1+C39*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E39" s="10">
-        <f>(C38/C39-1)/Quotes!$B$2</f>
+        <f>(1/D39-1)/B39</f>
+        <v/>
+      </c>
+      <c r="F39" s="10">
+        <f>(D38/D39-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6">
+      <c r="A40" s="15">
+        <f>EDATE(Quotes!$E$2,3*38)</f>
+        <v/>
+      </c>
+      <c r="B40" s="6">
         <f>Interpolation!A40</f>
         <v/>
       </c>
-      <c r="B40" s="12">
+      <c r="C40" s="12">
         <f>Interpolation!E40</f>
         <v/>
       </c>
-      <c r="C40" s="13">
-        <f>(1-B40*Quotes!$B$2*SUM($C$3:C39))/(1+B40*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D40" s="10">
-        <f>(1/C40-1)/A40</f>
+      <c r="D40" s="13">
+        <f>(1-C40*Quotes!$B$2*SUM($D$3:D39))/(1+C40*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E40" s="10">
-        <f>(C39/C40-1)/Quotes!$B$2</f>
+        <f>(1/D40-1)/B40</f>
+        <v/>
+      </c>
+      <c r="F40" s="10">
+        <f>(D39/D40-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6">
+      <c r="A41" s="15">
+        <f>EDATE(Quotes!$E$2,3*39)</f>
+        <v/>
+      </c>
+      <c r="B41" s="6">
         <f>Interpolation!A41</f>
         <v/>
       </c>
-      <c r="B41" s="12">
+      <c r="C41" s="12">
         <f>Interpolation!E41</f>
         <v/>
       </c>
-      <c r="C41" s="13">
-        <f>(1-B41*Quotes!$B$2*SUM($C$3:C40))/(1+B41*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D41" s="10">
-        <f>(1/C41-1)/A41</f>
+      <c r="D41" s="13">
+        <f>(1-C41*Quotes!$B$2*SUM($D$3:D40))/(1+C41*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E41" s="10">
-        <f>(C40/C41-1)/Quotes!$B$2</f>
+        <f>(1/D41-1)/B41</f>
+        <v/>
+      </c>
+      <c r="F41" s="10">
+        <f>(D40/D41-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6">
+      <c r="A42" s="15">
+        <f>EDATE(Quotes!$E$2,3*40)</f>
+        <v/>
+      </c>
+      <c r="B42" s="6">
         <f>Interpolation!A42</f>
         <v/>
       </c>
-      <c r="B42" s="12">
+      <c r="C42" s="12">
         <f>Interpolation!E42</f>
         <v/>
       </c>
-      <c r="C42" s="13">
-        <f>(1-B42*Quotes!$B$2*SUM($C$3:C41))/(1+B42*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D42" s="10">
-        <f>(1/C42-1)/A42</f>
+      <c r="D42" s="13">
+        <f>(1-C42*Quotes!$B$2*SUM($D$3:D41))/(1+C42*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E42" s="10">
-        <f>(C41/C42-1)/Quotes!$B$2</f>
+        <f>(1/D42-1)/B42</f>
+        <v/>
+      </c>
+      <c r="F42" s="10">
+        <f>(D41/D42-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6">
+      <c r="A43" s="15">
+        <f>EDATE(Quotes!$E$2,3*41)</f>
+        <v/>
+      </c>
+      <c r="B43" s="6">
         <f>Interpolation!A43</f>
         <v/>
       </c>
-      <c r="B43" s="12">
+      <c r="C43" s="12">
         <f>Interpolation!E43</f>
         <v/>
       </c>
-      <c r="C43" s="13">
-        <f>(1-B43*Quotes!$B$2*SUM($C$3:C42))/(1+B43*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D43" s="10">
-        <f>(1/C43-1)/A43</f>
+      <c r="D43" s="13">
+        <f>(1-C43*Quotes!$B$2*SUM($D$3:D42))/(1+C43*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E43" s="10">
-        <f>(C42/C43-1)/Quotes!$B$2</f>
+        <f>(1/D43-1)/B43</f>
+        <v/>
+      </c>
+      <c r="F43" s="10">
+        <f>(D42/D43-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6">
+      <c r="A44" s="15">
+        <f>EDATE(Quotes!$E$2,3*42)</f>
+        <v/>
+      </c>
+      <c r="B44" s="6">
         <f>Interpolation!A44</f>
         <v/>
       </c>
-      <c r="B44" s="12">
+      <c r="C44" s="12">
         <f>Interpolation!E44</f>
         <v/>
       </c>
-      <c r="C44" s="13">
-        <f>(1-B44*Quotes!$B$2*SUM($C$3:C43))/(1+B44*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D44" s="10">
-        <f>(1/C44-1)/A44</f>
+      <c r="D44" s="13">
+        <f>(1-C44*Quotes!$B$2*SUM($D$3:D43))/(1+C44*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E44" s="10">
-        <f>(C43/C44-1)/Quotes!$B$2</f>
+        <f>(1/D44-1)/B44</f>
+        <v/>
+      </c>
+      <c r="F44" s="10">
+        <f>(D43/D44-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6">
+      <c r="A45" s="15">
+        <f>EDATE(Quotes!$E$2,3*43)</f>
+        <v/>
+      </c>
+      <c r="B45" s="6">
         <f>Interpolation!A45</f>
         <v/>
       </c>
-      <c r="B45" s="12">
+      <c r="C45" s="12">
         <f>Interpolation!E45</f>
         <v/>
       </c>
-      <c r="C45" s="13">
-        <f>(1-B45*Quotes!$B$2*SUM($C$3:C44))/(1+B45*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D45" s="10">
-        <f>(1/C45-1)/A45</f>
+      <c r="D45" s="13">
+        <f>(1-C45*Quotes!$B$2*SUM($D$3:D44))/(1+C45*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E45" s="10">
-        <f>(C44/C45-1)/Quotes!$B$2</f>
+        <f>(1/D45-1)/B45</f>
+        <v/>
+      </c>
+      <c r="F45" s="10">
+        <f>(D44/D45-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6">
+      <c r="A46" s="15">
+        <f>EDATE(Quotes!$E$2,3*44)</f>
+        <v/>
+      </c>
+      <c r="B46" s="6">
         <f>Interpolation!A46</f>
         <v/>
       </c>
-      <c r="B46" s="12">
+      <c r="C46" s="12">
         <f>Interpolation!E46</f>
         <v/>
       </c>
-      <c r="C46" s="13">
-        <f>(1-B46*Quotes!$B$2*SUM($C$3:C45))/(1+B46*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D46" s="10">
-        <f>(1/C46-1)/A46</f>
+      <c r="D46" s="13">
+        <f>(1-C46*Quotes!$B$2*SUM($D$3:D45))/(1+C46*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E46" s="10">
-        <f>(C45/C46-1)/Quotes!$B$2</f>
+        <f>(1/D46-1)/B46</f>
+        <v/>
+      </c>
+      <c r="F46" s="10">
+        <f>(D45/D46-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6">
+      <c r="A47" s="15">
+        <f>EDATE(Quotes!$E$2,3*45)</f>
+        <v/>
+      </c>
+      <c r="B47" s="6">
         <f>Interpolation!A47</f>
         <v/>
       </c>
-      <c r="B47" s="12">
+      <c r="C47" s="12">
         <f>Interpolation!E47</f>
         <v/>
       </c>
-      <c r="C47" s="13">
-        <f>(1-B47*Quotes!$B$2*SUM($C$3:C46))/(1+B47*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D47" s="10">
-        <f>(1/C47-1)/A47</f>
+      <c r="D47" s="13">
+        <f>(1-C47*Quotes!$B$2*SUM($D$3:D46))/(1+C47*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E47" s="10">
-        <f>(C46/C47-1)/Quotes!$B$2</f>
+        <f>(1/D47-1)/B47</f>
+        <v/>
+      </c>
+      <c r="F47" s="10">
+        <f>(D46/D47-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="6">
+      <c r="A48" s="15">
+        <f>EDATE(Quotes!$E$2,3*46)</f>
+        <v/>
+      </c>
+      <c r="B48" s="6">
         <f>Interpolation!A48</f>
         <v/>
       </c>
-      <c r="B48" s="12">
+      <c r="C48" s="12">
         <f>Interpolation!E48</f>
         <v/>
       </c>
-      <c r="C48" s="13">
-        <f>(1-B48*Quotes!$B$2*SUM($C$3:C47))/(1+B48*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D48" s="10">
-        <f>(1/C48-1)/A48</f>
+      <c r="D48" s="13">
+        <f>(1-C48*Quotes!$B$2*SUM($D$3:D47))/(1+C48*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E48" s="10">
-        <f>(C47/C48-1)/Quotes!$B$2</f>
+        <f>(1/D48-1)/B48</f>
+        <v/>
+      </c>
+      <c r="F48" s="10">
+        <f>(D47/D48-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="6">
+      <c r="A49" s="15">
+        <f>EDATE(Quotes!$E$2,3*47)</f>
+        <v/>
+      </c>
+      <c r="B49" s="6">
         <f>Interpolation!A49</f>
         <v/>
       </c>
-      <c r="B49" s="12">
+      <c r="C49" s="12">
         <f>Interpolation!E49</f>
         <v/>
       </c>
-      <c r="C49" s="13">
-        <f>(1-B49*Quotes!$B$2*SUM($C$3:C48))/(1+B49*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D49" s="10">
-        <f>(1/C49-1)/A49</f>
+      <c r="D49" s="13">
+        <f>(1-C49*Quotes!$B$2*SUM($D$3:D48))/(1+C49*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E49" s="10">
-        <f>(C48/C49-1)/Quotes!$B$2</f>
+        <f>(1/D49-1)/B49</f>
+        <v/>
+      </c>
+      <c r="F49" s="10">
+        <f>(D48/D49-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6">
+      <c r="A50" s="15">
+        <f>EDATE(Quotes!$E$2,3*48)</f>
+        <v/>
+      </c>
+      <c r="B50" s="6">
         <f>Interpolation!A50</f>
         <v/>
       </c>
-      <c r="B50" s="12">
+      <c r="C50" s="12">
         <f>Interpolation!E50</f>
         <v/>
       </c>
-      <c r="C50" s="13">
-        <f>(1-B50*Quotes!$B$2*SUM($C$3:C49))/(1+B50*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D50" s="10">
-        <f>(1/C50-1)/A50</f>
+      <c r="D50" s="13">
+        <f>(1-C50*Quotes!$B$2*SUM($D$3:D49))/(1+C50*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E50" s="10">
-        <f>(C49/C50-1)/Quotes!$B$2</f>
+        <f>(1/D50-1)/B50</f>
+        <v/>
+      </c>
+      <c r="F50" s="10">
+        <f>(D49/D50-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6">
+      <c r="A51" s="15">
+        <f>EDATE(Quotes!$E$2,3*49)</f>
+        <v/>
+      </c>
+      <c r="B51" s="6">
         <f>Interpolation!A51</f>
         <v/>
       </c>
-      <c r="B51" s="12">
+      <c r="C51" s="12">
         <f>Interpolation!E51</f>
         <v/>
       </c>
-      <c r="C51" s="13">
-        <f>(1-B51*Quotes!$B$2*SUM($C$3:C50))/(1+B51*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D51" s="10">
-        <f>(1/C51-1)/A51</f>
+      <c r="D51" s="13">
+        <f>(1-C51*Quotes!$B$2*SUM($D$3:D50))/(1+C51*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E51" s="10">
-        <f>(C50/C51-1)/Quotes!$B$2</f>
+        <f>(1/D51-1)/B51</f>
+        <v/>
+      </c>
+      <c r="F51" s="10">
+        <f>(D50/D51-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="6">
+      <c r="A52" s="15">
+        <f>EDATE(Quotes!$E$2,3*50)</f>
+        <v/>
+      </c>
+      <c r="B52" s="6">
         <f>Interpolation!A52</f>
         <v/>
       </c>
-      <c r="B52" s="12">
+      <c r="C52" s="12">
         <f>Interpolation!E52</f>
         <v/>
       </c>
-      <c r="C52" s="13">
-        <f>(1-B52*Quotes!$B$2*SUM($C$3:C51))/(1+B52*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D52" s="10">
-        <f>(1/C52-1)/A52</f>
+      <c r="D52" s="13">
+        <f>(1-C52*Quotes!$B$2*SUM($D$3:D51))/(1+C52*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E52" s="10">
-        <f>(C51/C52-1)/Quotes!$B$2</f>
+        <f>(1/D52-1)/B52</f>
+        <v/>
+      </c>
+      <c r="F52" s="10">
+        <f>(D51/D52-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6">
+      <c r="A53" s="15">
+        <f>EDATE(Quotes!$E$2,3*51)</f>
+        <v/>
+      </c>
+      <c r="B53" s="6">
         <f>Interpolation!A53</f>
         <v/>
       </c>
-      <c r="B53" s="12">
+      <c r="C53" s="12">
         <f>Interpolation!E53</f>
         <v/>
       </c>
-      <c r="C53" s="13">
-        <f>(1-B53*Quotes!$B$2*SUM($C$3:C52))/(1+B53*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D53" s="10">
-        <f>(1/C53-1)/A53</f>
+      <c r="D53" s="13">
+        <f>(1-C53*Quotes!$B$2*SUM($D$3:D52))/(1+C53*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E53" s="10">
-        <f>(C52/C53-1)/Quotes!$B$2</f>
+        <f>(1/D53-1)/B53</f>
+        <v/>
+      </c>
+      <c r="F53" s="10">
+        <f>(D52/D53-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6">
+      <c r="A54" s="15">
+        <f>EDATE(Quotes!$E$2,3*52)</f>
+        <v/>
+      </c>
+      <c r="B54" s="6">
         <f>Interpolation!A54</f>
         <v/>
       </c>
-      <c r="B54" s="12">
+      <c r="C54" s="12">
         <f>Interpolation!E54</f>
         <v/>
       </c>
-      <c r="C54" s="13">
-        <f>(1-B54*Quotes!$B$2*SUM($C$3:C53))/(1+B54*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D54" s="10">
-        <f>(1/C54-1)/A54</f>
+      <c r="D54" s="13">
+        <f>(1-C54*Quotes!$B$2*SUM($D$3:D53))/(1+C54*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E54" s="10">
-        <f>(C53/C54-1)/Quotes!$B$2</f>
+        <f>(1/D54-1)/B54</f>
+        <v/>
+      </c>
+      <c r="F54" s="10">
+        <f>(D53/D54-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6">
+      <c r="A55" s="15">
+        <f>EDATE(Quotes!$E$2,3*53)</f>
+        <v/>
+      </c>
+      <c r="B55" s="6">
         <f>Interpolation!A55</f>
         <v/>
       </c>
-      <c r="B55" s="12">
+      <c r="C55" s="12">
         <f>Interpolation!E55</f>
         <v/>
       </c>
-      <c r="C55" s="13">
-        <f>(1-B55*Quotes!$B$2*SUM($C$3:C54))/(1+B55*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D55" s="10">
-        <f>(1/C55-1)/A55</f>
+      <c r="D55" s="13">
+        <f>(1-C55*Quotes!$B$2*SUM($D$3:D54))/(1+C55*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E55" s="10">
-        <f>(C54/C55-1)/Quotes!$B$2</f>
+        <f>(1/D55-1)/B55</f>
+        <v/>
+      </c>
+      <c r="F55" s="10">
+        <f>(D54/D55-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6">
+      <c r="A56" s="15">
+        <f>EDATE(Quotes!$E$2,3*54)</f>
+        <v/>
+      </c>
+      <c r="B56" s="6">
         <f>Interpolation!A56</f>
         <v/>
       </c>
-      <c r="B56" s="12">
+      <c r="C56" s="12">
         <f>Interpolation!E56</f>
         <v/>
       </c>
-      <c r="C56" s="13">
-        <f>(1-B56*Quotes!$B$2*SUM($C$3:C55))/(1+B56*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D56" s="10">
-        <f>(1/C56-1)/A56</f>
+      <c r="D56" s="13">
+        <f>(1-C56*Quotes!$B$2*SUM($D$3:D55))/(1+C56*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E56" s="10">
-        <f>(C55/C56-1)/Quotes!$B$2</f>
+        <f>(1/D56-1)/B56</f>
+        <v/>
+      </c>
+      <c r="F56" s="10">
+        <f>(D55/D56-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="6">
+      <c r="A57" s="15">
+        <f>EDATE(Quotes!$E$2,3*55)</f>
+        <v/>
+      </c>
+      <c r="B57" s="6">
         <f>Interpolation!A57</f>
         <v/>
       </c>
-      <c r="B57" s="12">
+      <c r="C57" s="12">
         <f>Interpolation!E57</f>
         <v/>
       </c>
-      <c r="C57" s="13">
-        <f>(1-B57*Quotes!$B$2*SUM($C$3:C56))/(1+B57*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D57" s="10">
-        <f>(1/C57-1)/A57</f>
+      <c r="D57" s="13">
+        <f>(1-C57*Quotes!$B$2*SUM($D$3:D56))/(1+C57*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E57" s="10">
-        <f>(C56/C57-1)/Quotes!$B$2</f>
+        <f>(1/D57-1)/B57</f>
+        <v/>
+      </c>
+      <c r="F57" s="10">
+        <f>(D56/D57-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6">
+      <c r="A58" s="15">
+        <f>EDATE(Quotes!$E$2,3*56)</f>
+        <v/>
+      </c>
+      <c r="B58" s="6">
         <f>Interpolation!A58</f>
         <v/>
       </c>
-      <c r="B58" s="12">
+      <c r="C58" s="12">
         <f>Interpolation!E58</f>
         <v/>
       </c>
-      <c r="C58" s="13">
-        <f>(1-B58*Quotes!$B$2*SUM($C$3:C57))/(1+B58*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D58" s="10">
-        <f>(1/C58-1)/A58</f>
+      <c r="D58" s="13">
+        <f>(1-C58*Quotes!$B$2*SUM($D$3:D57))/(1+C58*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E58" s="10">
-        <f>(C57/C58-1)/Quotes!$B$2</f>
+        <f>(1/D58-1)/B58</f>
+        <v/>
+      </c>
+      <c r="F58" s="10">
+        <f>(D57/D58-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6">
+      <c r="A59" s="15">
+        <f>EDATE(Quotes!$E$2,3*57)</f>
+        <v/>
+      </c>
+      <c r="B59" s="6">
         <f>Interpolation!A59</f>
         <v/>
       </c>
-      <c r="B59" s="12">
+      <c r="C59" s="12">
         <f>Interpolation!E59</f>
         <v/>
       </c>
-      <c r="C59" s="13">
-        <f>(1-B59*Quotes!$B$2*SUM($C$3:C58))/(1+B59*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D59" s="10">
-        <f>(1/C59-1)/A59</f>
+      <c r="D59" s="13">
+        <f>(1-C59*Quotes!$B$2*SUM($D$3:D58))/(1+C59*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E59" s="10">
-        <f>(C58/C59-1)/Quotes!$B$2</f>
+        <f>(1/D59-1)/B59</f>
+        <v/>
+      </c>
+      <c r="F59" s="10">
+        <f>(D58/D59-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6">
+      <c r="A60" s="15">
+        <f>EDATE(Quotes!$E$2,3*58)</f>
+        <v/>
+      </c>
+      <c r="B60" s="6">
         <f>Interpolation!A60</f>
         <v/>
       </c>
-      <c r="B60" s="12">
+      <c r="C60" s="12">
         <f>Interpolation!E60</f>
         <v/>
       </c>
-      <c r="C60" s="13">
-        <f>(1-B60*Quotes!$B$2*SUM($C$3:C59))/(1+B60*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D60" s="10">
-        <f>(1/C60-1)/A60</f>
+      <c r="D60" s="13">
+        <f>(1-C60*Quotes!$B$2*SUM($D$3:D59))/(1+C60*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E60" s="10">
-        <f>(C59/C60-1)/Quotes!$B$2</f>
+        <f>(1/D60-1)/B60</f>
+        <v/>
+      </c>
+      <c r="F60" s="10">
+        <f>(D59/D60-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="6">
+      <c r="A61" s="15">
+        <f>EDATE(Quotes!$E$2,3*59)</f>
+        <v/>
+      </c>
+      <c r="B61" s="6">
         <f>Interpolation!A61</f>
         <v/>
       </c>
-      <c r="B61" s="12">
+      <c r="C61" s="12">
         <f>Interpolation!E61</f>
         <v/>
       </c>
-      <c r="C61" s="13">
-        <f>(1-B61*Quotes!$B$2*SUM($C$3:C60))/(1+B61*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D61" s="10">
-        <f>(1/C61-1)/A61</f>
+      <c r="D61" s="13">
+        <f>(1-C61*Quotes!$B$2*SUM($D$3:D60))/(1+C61*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E61" s="10">
-        <f>(C60/C61-1)/Quotes!$B$2</f>
+        <f>(1/D61-1)/B61</f>
+        <v/>
+      </c>
+      <c r="F61" s="10">
+        <f>(D60/D61-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="6">
+      <c r="A62" s="15">
+        <f>EDATE(Quotes!$E$2,3*60)</f>
+        <v/>
+      </c>
+      <c r="B62" s="6">
         <f>Interpolation!A62</f>
         <v/>
       </c>
-      <c r="B62" s="12">
+      <c r="C62" s="12">
         <f>Interpolation!E62</f>
         <v/>
       </c>
-      <c r="C62" s="13">
-        <f>(1-B62*Quotes!$B$2*SUM($C$3:C61))/(1+B62*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D62" s="10">
-        <f>(1/C62-1)/A62</f>
+      <c r="D62" s="13">
+        <f>(1-C62*Quotes!$B$2*SUM($D$3:D61))/(1+C62*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E62" s="10">
-        <f>(C61/C62-1)/Quotes!$B$2</f>
+        <f>(1/D62-1)/B62</f>
+        <v/>
+      </c>
+      <c r="F62" s="10">
+        <f>(D61/D62-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="6">
+      <c r="A63" s="15">
+        <f>EDATE(Quotes!$E$2,3*61)</f>
+        <v/>
+      </c>
+      <c r="B63" s="6">
         <f>Interpolation!A63</f>
         <v/>
       </c>
-      <c r="B63" s="12">
+      <c r="C63" s="12">
         <f>Interpolation!E63</f>
         <v/>
       </c>
-      <c r="C63" s="13">
-        <f>(1-B63*Quotes!$B$2*SUM($C$3:C62))/(1+B63*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D63" s="10">
-        <f>(1/C63-1)/A63</f>
+      <c r="D63" s="13">
+        <f>(1-C63*Quotes!$B$2*SUM($D$3:D62))/(1+C63*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E63" s="10">
-        <f>(C62/C63-1)/Quotes!$B$2</f>
+        <f>(1/D63-1)/B63</f>
+        <v/>
+      </c>
+      <c r="F63" s="10">
+        <f>(D62/D63-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6">
+      <c r="A64" s="15">
+        <f>EDATE(Quotes!$E$2,3*62)</f>
+        <v/>
+      </c>
+      <c r="B64" s="6">
         <f>Interpolation!A64</f>
         <v/>
       </c>
-      <c r="B64" s="12">
+      <c r="C64" s="12">
         <f>Interpolation!E64</f>
         <v/>
       </c>
-      <c r="C64" s="13">
-        <f>(1-B64*Quotes!$B$2*SUM($C$3:C63))/(1+B64*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D64" s="10">
-        <f>(1/C64-1)/A64</f>
+      <c r="D64" s="13">
+        <f>(1-C64*Quotes!$B$2*SUM($D$3:D63))/(1+C64*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E64" s="10">
-        <f>(C63/C64-1)/Quotes!$B$2</f>
+        <f>(1/D64-1)/B64</f>
+        <v/>
+      </c>
+      <c r="F64" s="10">
+        <f>(D63/D64-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6">
+      <c r="A65" s="15">
+        <f>EDATE(Quotes!$E$2,3*63)</f>
+        <v/>
+      </c>
+      <c r="B65" s="6">
         <f>Interpolation!A65</f>
         <v/>
       </c>
-      <c r="B65" s="12">
+      <c r="C65" s="12">
         <f>Interpolation!E65</f>
         <v/>
       </c>
-      <c r="C65" s="13">
-        <f>(1-B65*Quotes!$B$2*SUM($C$3:C64))/(1+B65*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D65" s="10">
-        <f>(1/C65-1)/A65</f>
+      <c r="D65" s="13">
+        <f>(1-C65*Quotes!$B$2*SUM($D$3:D64))/(1+C65*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E65" s="10">
-        <f>(C64/C65-1)/Quotes!$B$2</f>
+        <f>(1/D65-1)/B65</f>
+        <v/>
+      </c>
+      <c r="F65" s="10">
+        <f>(D64/D65-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6">
+      <c r="A66" s="15">
+        <f>EDATE(Quotes!$E$2,3*64)</f>
+        <v/>
+      </c>
+      <c r="B66" s="6">
         <f>Interpolation!A66</f>
         <v/>
       </c>
-      <c r="B66" s="12">
+      <c r="C66" s="12">
         <f>Interpolation!E66</f>
         <v/>
       </c>
-      <c r="C66" s="13">
-        <f>(1-B66*Quotes!$B$2*SUM($C$3:C65))/(1+B66*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D66" s="10">
-        <f>(1/C66-1)/A66</f>
+      <c r="D66" s="13">
+        <f>(1-C66*Quotes!$B$2*SUM($D$3:D65))/(1+C66*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E66" s="10">
-        <f>(C65/C66-1)/Quotes!$B$2</f>
+        <f>(1/D66-1)/B66</f>
+        <v/>
+      </c>
+      <c r="F66" s="10">
+        <f>(D65/D66-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="6">
+      <c r="A67" s="15">
+        <f>EDATE(Quotes!$E$2,3*65)</f>
+        <v/>
+      </c>
+      <c r="B67" s="6">
         <f>Interpolation!A67</f>
         <v/>
       </c>
-      <c r="B67" s="12">
+      <c r="C67" s="12">
         <f>Interpolation!E67</f>
         <v/>
       </c>
-      <c r="C67" s="13">
-        <f>(1-B67*Quotes!$B$2*SUM($C$3:C66))/(1+B67*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D67" s="10">
-        <f>(1/C67-1)/A67</f>
+      <c r="D67" s="13">
+        <f>(1-C67*Quotes!$B$2*SUM($D$3:D66))/(1+C67*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E67" s="10">
-        <f>(C66/C67-1)/Quotes!$B$2</f>
+        <f>(1/D67-1)/B67</f>
+        <v/>
+      </c>
+      <c r="F67" s="10">
+        <f>(D66/D67-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="6">
+      <c r="A68" s="15">
+        <f>EDATE(Quotes!$E$2,3*66)</f>
+        <v/>
+      </c>
+      <c r="B68" s="6">
         <f>Interpolation!A68</f>
         <v/>
       </c>
-      <c r="B68" s="12">
+      <c r="C68" s="12">
         <f>Interpolation!E68</f>
         <v/>
       </c>
-      <c r="C68" s="13">
-        <f>(1-B68*Quotes!$B$2*SUM($C$3:C67))/(1+B68*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D68" s="10">
-        <f>(1/C68-1)/A68</f>
+      <c r="D68" s="13">
+        <f>(1-C68*Quotes!$B$2*SUM($D$3:D67))/(1+C68*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E68" s="10">
-        <f>(C67/C68-1)/Quotes!$B$2</f>
+        <f>(1/D68-1)/B68</f>
+        <v/>
+      </c>
+      <c r="F68" s="10">
+        <f>(D67/D68-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6">
+      <c r="A69" s="15">
+        <f>EDATE(Quotes!$E$2,3*67)</f>
+        <v/>
+      </c>
+      <c r="B69" s="6">
         <f>Interpolation!A69</f>
         <v/>
       </c>
-      <c r="B69" s="12">
+      <c r="C69" s="12">
         <f>Interpolation!E69</f>
         <v/>
       </c>
-      <c r="C69" s="13">
-        <f>(1-B69*Quotes!$B$2*SUM($C$3:C68))/(1+B69*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D69" s="10">
-        <f>(1/C69-1)/A69</f>
+      <c r="D69" s="13">
+        <f>(1-C69*Quotes!$B$2*SUM($D$3:D68))/(1+C69*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E69" s="10">
-        <f>(C68/C69-1)/Quotes!$B$2</f>
+        <f>(1/D69-1)/B69</f>
+        <v/>
+      </c>
+      <c r="F69" s="10">
+        <f>(D68/D69-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="6">
+      <c r="A70" s="15">
+        <f>EDATE(Quotes!$E$2,3*68)</f>
+        <v/>
+      </c>
+      <c r="B70" s="6">
         <f>Interpolation!A70</f>
         <v/>
       </c>
-      <c r="B70" s="12">
+      <c r="C70" s="12">
         <f>Interpolation!E70</f>
         <v/>
       </c>
-      <c r="C70" s="13">
-        <f>(1-B70*Quotes!$B$2*SUM($C$3:C69))/(1+B70*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D70" s="10">
-        <f>(1/C70-1)/A70</f>
+      <c r="D70" s="13">
+        <f>(1-C70*Quotes!$B$2*SUM($D$3:D69))/(1+C70*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E70" s="10">
-        <f>(C69/C70-1)/Quotes!$B$2</f>
+        <f>(1/D70-1)/B70</f>
+        <v/>
+      </c>
+      <c r="F70" s="10">
+        <f>(D69/D70-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="6">
+      <c r="A71" s="15">
+        <f>EDATE(Quotes!$E$2,3*69)</f>
+        <v/>
+      </c>
+      <c r="B71" s="6">
         <f>Interpolation!A71</f>
         <v/>
       </c>
-      <c r="B71" s="12">
+      <c r="C71" s="12">
         <f>Interpolation!E71</f>
         <v/>
       </c>
-      <c r="C71" s="13">
-        <f>(1-B71*Quotes!$B$2*SUM($C$3:C70))/(1+B71*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D71" s="10">
-        <f>(1/C71-1)/A71</f>
+      <c r="D71" s="13">
+        <f>(1-C71*Quotes!$B$2*SUM($D$3:D70))/(1+C71*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E71" s="10">
-        <f>(C70/C71-1)/Quotes!$B$2</f>
+        <f>(1/D71-1)/B71</f>
+        <v/>
+      </c>
+      <c r="F71" s="10">
+        <f>(D70/D71-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="6">
+      <c r="A72" s="15">
+        <f>EDATE(Quotes!$E$2,3*70)</f>
+        <v/>
+      </c>
+      <c r="B72" s="6">
         <f>Interpolation!A72</f>
         <v/>
       </c>
-      <c r="B72" s="12">
+      <c r="C72" s="12">
         <f>Interpolation!E72</f>
         <v/>
       </c>
-      <c r="C72" s="13">
-        <f>(1-B72*Quotes!$B$2*SUM($C$3:C71))/(1+B72*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D72" s="10">
-        <f>(1/C72-1)/A72</f>
+      <c r="D72" s="13">
+        <f>(1-C72*Quotes!$B$2*SUM($D$3:D71))/(1+C72*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E72" s="10">
-        <f>(C71/C72-1)/Quotes!$B$2</f>
+        <f>(1/D72-1)/B72</f>
+        <v/>
+      </c>
+      <c r="F72" s="10">
+        <f>(D71/D72-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="6">
+      <c r="A73" s="15">
+        <f>EDATE(Quotes!$E$2,3*71)</f>
+        <v/>
+      </c>
+      <c r="B73" s="6">
         <f>Interpolation!A73</f>
         <v/>
       </c>
-      <c r="B73" s="12">
+      <c r="C73" s="12">
         <f>Interpolation!E73</f>
         <v/>
       </c>
-      <c r="C73" s="13">
-        <f>(1-B73*Quotes!$B$2*SUM($C$3:C72))/(1+B73*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D73" s="10">
-        <f>(1/C73-1)/A73</f>
+      <c r="D73" s="13">
+        <f>(1-C73*Quotes!$B$2*SUM($D$3:D72))/(1+C73*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E73" s="10">
-        <f>(C72/C73-1)/Quotes!$B$2</f>
+        <f>(1/D73-1)/B73</f>
+        <v/>
+      </c>
+      <c r="F73" s="10">
+        <f>(D72/D73-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="6">
+      <c r="A74" s="15">
+        <f>EDATE(Quotes!$E$2,3*72)</f>
+        <v/>
+      </c>
+      <c r="B74" s="6">
         <f>Interpolation!A74</f>
         <v/>
       </c>
-      <c r="B74" s="12">
+      <c r="C74" s="12">
         <f>Interpolation!E74</f>
         <v/>
       </c>
-      <c r="C74" s="13">
-        <f>(1-B74*Quotes!$B$2*SUM($C$3:C73))/(1+B74*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D74" s="10">
-        <f>(1/C74-1)/A74</f>
+      <c r="D74" s="13">
+        <f>(1-C74*Quotes!$B$2*SUM($D$3:D73))/(1+C74*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E74" s="10">
-        <f>(C73/C74-1)/Quotes!$B$2</f>
+        <f>(1/D74-1)/B74</f>
+        <v/>
+      </c>
+      <c r="F74" s="10">
+        <f>(D73/D74-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="6">
+      <c r="A75" s="15">
+        <f>EDATE(Quotes!$E$2,3*73)</f>
+        <v/>
+      </c>
+      <c r="B75" s="6">
         <f>Interpolation!A75</f>
         <v/>
       </c>
-      <c r="B75" s="12">
+      <c r="C75" s="12">
         <f>Interpolation!E75</f>
         <v/>
       </c>
-      <c r="C75" s="13">
-        <f>(1-B75*Quotes!$B$2*SUM($C$3:C74))/(1+B75*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D75" s="10">
-        <f>(1/C75-1)/A75</f>
+      <c r="D75" s="13">
+        <f>(1-C75*Quotes!$B$2*SUM($D$3:D74))/(1+C75*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E75" s="10">
-        <f>(C74/C75-1)/Quotes!$B$2</f>
+        <f>(1/D75-1)/B75</f>
+        <v/>
+      </c>
+      <c r="F75" s="10">
+        <f>(D74/D75-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="6">
+      <c r="A76" s="15">
+        <f>EDATE(Quotes!$E$2,3*74)</f>
+        <v/>
+      </c>
+      <c r="B76" s="6">
         <f>Interpolation!A76</f>
         <v/>
       </c>
-      <c r="B76" s="12">
+      <c r="C76" s="12">
         <f>Interpolation!E76</f>
         <v/>
       </c>
-      <c r="C76" s="13">
-        <f>(1-B76*Quotes!$B$2*SUM($C$3:C75))/(1+B76*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D76" s="10">
-        <f>(1/C76-1)/A76</f>
+      <c r="D76" s="13">
+        <f>(1-C76*Quotes!$B$2*SUM($D$3:D75))/(1+C76*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E76" s="10">
-        <f>(C75/C76-1)/Quotes!$B$2</f>
+        <f>(1/D76-1)/B76</f>
+        <v/>
+      </c>
+      <c r="F76" s="10">
+        <f>(D75/D76-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="6">
+      <c r="A77" s="15">
+        <f>EDATE(Quotes!$E$2,3*75)</f>
+        <v/>
+      </c>
+      <c r="B77" s="6">
         <f>Interpolation!A77</f>
         <v/>
       </c>
-      <c r="B77" s="12">
+      <c r="C77" s="12">
         <f>Interpolation!E77</f>
         <v/>
       </c>
-      <c r="C77" s="13">
-        <f>(1-B77*Quotes!$B$2*SUM($C$3:C76))/(1+B77*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D77" s="10">
-        <f>(1/C77-1)/A77</f>
+      <c r="D77" s="13">
+        <f>(1-C77*Quotes!$B$2*SUM($D$3:D76))/(1+C77*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E77" s="10">
-        <f>(C76/C77-1)/Quotes!$B$2</f>
+        <f>(1/D77-1)/B77</f>
+        <v/>
+      </c>
+      <c r="F77" s="10">
+        <f>(D76/D77-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="6">
+      <c r="A78" s="15">
+        <f>EDATE(Quotes!$E$2,3*76)</f>
+        <v/>
+      </c>
+      <c r="B78" s="6">
         <f>Interpolation!A78</f>
         <v/>
       </c>
-      <c r="B78" s="12">
+      <c r="C78" s="12">
         <f>Interpolation!E78</f>
         <v/>
       </c>
-      <c r="C78" s="13">
-        <f>(1-B78*Quotes!$B$2*SUM($C$3:C77))/(1+B78*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D78" s="10">
-        <f>(1/C78-1)/A78</f>
+      <c r="D78" s="13">
+        <f>(1-C78*Quotes!$B$2*SUM($D$3:D77))/(1+C78*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E78" s="10">
-        <f>(C77/C78-1)/Quotes!$B$2</f>
+        <f>(1/D78-1)/B78</f>
+        <v/>
+      </c>
+      <c r="F78" s="10">
+        <f>(D77/D78-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="6">
+      <c r="A79" s="15">
+        <f>EDATE(Quotes!$E$2,3*77)</f>
+        <v/>
+      </c>
+      <c r="B79" s="6">
         <f>Interpolation!A79</f>
         <v/>
       </c>
-      <c r="B79" s="12">
+      <c r="C79" s="12">
         <f>Interpolation!E79</f>
         <v/>
       </c>
-      <c r="C79" s="13">
-        <f>(1-B79*Quotes!$B$2*SUM($C$3:C78))/(1+B79*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D79" s="10">
-        <f>(1/C79-1)/A79</f>
+      <c r="D79" s="13">
+        <f>(1-C79*Quotes!$B$2*SUM($D$3:D78))/(1+C79*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E79" s="10">
-        <f>(C78/C79-1)/Quotes!$B$2</f>
+        <f>(1/D79-1)/B79</f>
+        <v/>
+      </c>
+      <c r="F79" s="10">
+        <f>(D78/D79-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="6">
+      <c r="A80" s="15">
+        <f>EDATE(Quotes!$E$2,3*78)</f>
+        <v/>
+      </c>
+      <c r="B80" s="6">
         <f>Interpolation!A80</f>
         <v/>
       </c>
-      <c r="B80" s="12">
+      <c r="C80" s="12">
         <f>Interpolation!E80</f>
         <v/>
       </c>
-      <c r="C80" s="13">
-        <f>(1-B80*Quotes!$B$2*SUM($C$3:C79))/(1+B80*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D80" s="10">
-        <f>(1/C80-1)/A80</f>
+      <c r="D80" s="13">
+        <f>(1-C80*Quotes!$B$2*SUM($D$3:D79))/(1+C80*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E80" s="10">
-        <f>(C79/C80-1)/Quotes!$B$2</f>
+        <f>(1/D80-1)/B80</f>
+        <v/>
+      </c>
+      <c r="F80" s="10">
+        <f>(D79/D80-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="6">
+      <c r="A81" s="15">
+        <f>EDATE(Quotes!$E$2,3*79)</f>
+        <v/>
+      </c>
+      <c r="B81" s="6">
         <f>Interpolation!A81</f>
         <v/>
       </c>
-      <c r="B81" s="12">
+      <c r="C81" s="12">
         <f>Interpolation!E81</f>
         <v/>
       </c>
-      <c r="C81" s="13">
-        <f>(1-B81*Quotes!$B$2*SUM($C$3:C80))/(1+B81*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D81" s="10">
-        <f>(1/C81-1)/A81</f>
+      <c r="D81" s="13">
+        <f>(1-C81*Quotes!$B$2*SUM($D$3:D80))/(1+C81*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E81" s="10">
-        <f>(C80/C81-1)/Quotes!$B$2</f>
+        <f>(1/D81-1)/B81</f>
+        <v/>
+      </c>
+      <c r="F81" s="10">
+        <f>(D80/D81-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="6">
+      <c r="A82" s="15">
+        <f>EDATE(Quotes!$E$2,3*80)</f>
+        <v/>
+      </c>
+      <c r="B82" s="6">
         <f>Interpolation!A82</f>
         <v/>
       </c>
-      <c r="B82" s="12">
+      <c r="C82" s="12">
         <f>Interpolation!E82</f>
         <v/>
       </c>
-      <c r="C82" s="13">
-        <f>(1-B82*Quotes!$B$2*SUM($C$3:C81))/(1+B82*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D82" s="10">
-        <f>(1/C82-1)/A82</f>
+      <c r="D82" s="13">
+        <f>(1-C82*Quotes!$B$2*SUM($D$3:D81))/(1+C82*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E82" s="10">
-        <f>(C81/C82-1)/Quotes!$B$2</f>
+        <f>(1/D82-1)/B82</f>
+        <v/>
+      </c>
+      <c r="F82" s="10">
+        <f>(D81/D82-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="6">
+      <c r="A83" s="15">
+        <f>EDATE(Quotes!$E$2,3*81)</f>
+        <v/>
+      </c>
+      <c r="B83" s="6">
         <f>Interpolation!A83</f>
         <v/>
       </c>
-      <c r="B83" s="12">
+      <c r="C83" s="12">
         <f>Interpolation!E83</f>
         <v/>
       </c>
-      <c r="C83" s="13">
-        <f>(1-B83*Quotes!$B$2*SUM($C$3:C82))/(1+B83*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D83" s="10">
-        <f>(1/C83-1)/A83</f>
+      <c r="D83" s="13">
+        <f>(1-C83*Quotes!$B$2*SUM($D$3:D82))/(1+C83*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E83" s="10">
-        <f>(C82/C83-1)/Quotes!$B$2</f>
+        <f>(1/D83-1)/B83</f>
+        <v/>
+      </c>
+      <c r="F83" s="10">
+        <f>(D82/D83-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="6">
+      <c r="A84" s="15">
+        <f>EDATE(Quotes!$E$2,3*82)</f>
+        <v/>
+      </c>
+      <c r="B84" s="6">
         <f>Interpolation!A84</f>
         <v/>
       </c>
-      <c r="B84" s="12">
+      <c r="C84" s="12">
         <f>Interpolation!E84</f>
         <v/>
       </c>
-      <c r="C84" s="13">
-        <f>(1-B84*Quotes!$B$2*SUM($C$3:C83))/(1+B84*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D84" s="10">
-        <f>(1/C84-1)/A84</f>
+      <c r="D84" s="13">
+        <f>(1-C84*Quotes!$B$2*SUM($D$3:D83))/(1+C84*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E84" s="10">
-        <f>(C83/C84-1)/Quotes!$B$2</f>
+        <f>(1/D84-1)/B84</f>
+        <v/>
+      </c>
+      <c r="F84" s="10">
+        <f>(D83/D84-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="6">
+      <c r="A85" s="15">
+        <f>EDATE(Quotes!$E$2,3*83)</f>
+        <v/>
+      </c>
+      <c r="B85" s="6">
         <f>Interpolation!A85</f>
         <v/>
       </c>
-      <c r="B85" s="12">
+      <c r="C85" s="12">
         <f>Interpolation!E85</f>
         <v/>
       </c>
-      <c r="C85" s="13">
-        <f>(1-B85*Quotes!$B$2*SUM($C$3:C84))/(1+B85*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D85" s="10">
-        <f>(1/C85-1)/A85</f>
+      <c r="D85" s="13">
+        <f>(1-C85*Quotes!$B$2*SUM($D$3:D84))/(1+C85*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E85" s="10">
-        <f>(C84/C85-1)/Quotes!$B$2</f>
+        <f>(1/D85-1)/B85</f>
+        <v/>
+      </c>
+      <c r="F85" s="10">
+        <f>(D84/D85-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="6">
+      <c r="A86" s="15">
+        <f>EDATE(Quotes!$E$2,3*84)</f>
+        <v/>
+      </c>
+      <c r="B86" s="6">
         <f>Interpolation!A86</f>
         <v/>
       </c>
-      <c r="B86" s="12">
+      <c r="C86" s="12">
         <f>Interpolation!E86</f>
         <v/>
       </c>
-      <c r="C86" s="13">
-        <f>(1-B86*Quotes!$B$2*SUM($C$3:C85))/(1+B86*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D86" s="10">
-        <f>(1/C86-1)/A86</f>
+      <c r="D86" s="13">
+        <f>(1-C86*Quotes!$B$2*SUM($D$3:D85))/(1+C86*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E86" s="10">
-        <f>(C85/C86-1)/Quotes!$B$2</f>
+        <f>(1/D86-1)/B86</f>
+        <v/>
+      </c>
+      <c r="F86" s="10">
+        <f>(D85/D86-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="6">
+      <c r="A87" s="15">
+        <f>EDATE(Quotes!$E$2,3*85)</f>
+        <v/>
+      </c>
+      <c r="B87" s="6">
         <f>Interpolation!A87</f>
         <v/>
       </c>
-      <c r="B87" s="12">
+      <c r="C87" s="12">
         <f>Interpolation!E87</f>
         <v/>
       </c>
-      <c r="C87" s="13">
-        <f>(1-B87*Quotes!$B$2*SUM($C$3:C86))/(1+B87*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D87" s="10">
-        <f>(1/C87-1)/A87</f>
+      <c r="D87" s="13">
+        <f>(1-C87*Quotes!$B$2*SUM($D$3:D86))/(1+C87*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E87" s="10">
-        <f>(C86/C87-1)/Quotes!$B$2</f>
+        <f>(1/D87-1)/B87</f>
+        <v/>
+      </c>
+      <c r="F87" s="10">
+        <f>(D86/D87-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="6">
+      <c r="A88" s="15">
+        <f>EDATE(Quotes!$E$2,3*86)</f>
+        <v/>
+      </c>
+      <c r="B88" s="6">
         <f>Interpolation!A88</f>
         <v/>
       </c>
-      <c r="B88" s="12">
+      <c r="C88" s="12">
         <f>Interpolation!E88</f>
         <v/>
       </c>
-      <c r="C88" s="13">
-        <f>(1-B88*Quotes!$B$2*SUM($C$3:C87))/(1+B88*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D88" s="10">
-        <f>(1/C88-1)/A88</f>
+      <c r="D88" s="13">
+        <f>(1-C88*Quotes!$B$2*SUM($D$3:D87))/(1+C88*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E88" s="10">
-        <f>(C87/C88-1)/Quotes!$B$2</f>
+        <f>(1/D88-1)/B88</f>
+        <v/>
+      </c>
+      <c r="F88" s="10">
+        <f>(D87/D88-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="6">
+      <c r="A89" s="15">
+        <f>EDATE(Quotes!$E$2,3*87)</f>
+        <v/>
+      </c>
+      <c r="B89" s="6">
         <f>Interpolation!A89</f>
         <v/>
       </c>
-      <c r="B89" s="12">
+      <c r="C89" s="12">
         <f>Interpolation!E89</f>
         <v/>
       </c>
-      <c r="C89" s="13">
-        <f>(1-B89*Quotes!$B$2*SUM($C$3:C88))/(1+B89*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D89" s="10">
-        <f>(1/C89-1)/A89</f>
+      <c r="D89" s="13">
+        <f>(1-C89*Quotes!$B$2*SUM($D$3:D88))/(1+C89*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E89" s="10">
-        <f>(C88/C89-1)/Quotes!$B$2</f>
+        <f>(1/D89-1)/B89</f>
+        <v/>
+      </c>
+      <c r="F89" s="10">
+        <f>(D88/D89-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="6">
+      <c r="A90" s="15">
+        <f>EDATE(Quotes!$E$2,3*88)</f>
+        <v/>
+      </c>
+      <c r="B90" s="6">
         <f>Interpolation!A90</f>
         <v/>
       </c>
-      <c r="B90" s="12">
+      <c r="C90" s="12">
         <f>Interpolation!E90</f>
         <v/>
       </c>
-      <c r="C90" s="13">
-        <f>(1-B90*Quotes!$B$2*SUM($C$3:C89))/(1+B90*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D90" s="10">
-        <f>(1/C90-1)/A90</f>
+      <c r="D90" s="13">
+        <f>(1-C90*Quotes!$B$2*SUM($D$3:D89))/(1+C90*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E90" s="10">
-        <f>(C89/C90-1)/Quotes!$B$2</f>
+        <f>(1/D90-1)/B90</f>
+        <v/>
+      </c>
+      <c r="F90" s="10">
+        <f>(D89/D90-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="6">
+      <c r="A91" s="15">
+        <f>EDATE(Quotes!$E$2,3*89)</f>
+        <v/>
+      </c>
+      <c r="B91" s="6">
         <f>Interpolation!A91</f>
         <v/>
       </c>
-      <c r="B91" s="12">
+      <c r="C91" s="12">
         <f>Interpolation!E91</f>
         <v/>
       </c>
-      <c r="C91" s="13">
-        <f>(1-B91*Quotes!$B$2*SUM($C$3:C90))/(1+B91*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D91" s="10">
-        <f>(1/C91-1)/A91</f>
+      <c r="D91" s="13">
+        <f>(1-C91*Quotes!$B$2*SUM($D$3:D90))/(1+C91*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E91" s="10">
-        <f>(C90/C91-1)/Quotes!$B$2</f>
+        <f>(1/D91-1)/B91</f>
+        <v/>
+      </c>
+      <c r="F91" s="10">
+        <f>(D90/D91-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="6">
+      <c r="A92" s="15">
+        <f>EDATE(Quotes!$E$2,3*90)</f>
+        <v/>
+      </c>
+      <c r="B92" s="6">
         <f>Interpolation!A92</f>
         <v/>
       </c>
-      <c r="B92" s="12">
+      <c r="C92" s="12">
         <f>Interpolation!E92</f>
         <v/>
       </c>
-      <c r="C92" s="13">
-        <f>(1-B92*Quotes!$B$2*SUM($C$3:C91))/(1+B92*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D92" s="10">
-        <f>(1/C92-1)/A92</f>
+      <c r="D92" s="13">
+        <f>(1-C92*Quotes!$B$2*SUM($D$3:D91))/(1+C92*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E92" s="10">
-        <f>(C91/C92-1)/Quotes!$B$2</f>
+        <f>(1/D92-1)/B92</f>
+        <v/>
+      </c>
+      <c r="F92" s="10">
+        <f>(D91/D92-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="6">
+      <c r="A93" s="15">
+        <f>EDATE(Quotes!$E$2,3*91)</f>
+        <v/>
+      </c>
+      <c r="B93" s="6">
         <f>Interpolation!A93</f>
         <v/>
       </c>
-      <c r="B93" s="12">
+      <c r="C93" s="12">
         <f>Interpolation!E93</f>
         <v/>
       </c>
-      <c r="C93" s="13">
-        <f>(1-B93*Quotes!$B$2*SUM($C$3:C92))/(1+B93*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D93" s="10">
-        <f>(1/C93-1)/A93</f>
+      <c r="D93" s="13">
+        <f>(1-C93*Quotes!$B$2*SUM($D$3:D92))/(1+C93*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E93" s="10">
-        <f>(C92/C93-1)/Quotes!$B$2</f>
+        <f>(1/D93-1)/B93</f>
+        <v/>
+      </c>
+      <c r="F93" s="10">
+        <f>(D92/D93-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="6">
+      <c r="A94" s="15">
+        <f>EDATE(Quotes!$E$2,3*92)</f>
+        <v/>
+      </c>
+      <c r="B94" s="6">
         <f>Interpolation!A94</f>
         <v/>
       </c>
-      <c r="B94" s="12">
+      <c r="C94" s="12">
         <f>Interpolation!E94</f>
         <v/>
       </c>
-      <c r="C94" s="13">
-        <f>(1-B94*Quotes!$B$2*SUM($C$3:C93))/(1+B94*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D94" s="10">
-        <f>(1/C94-1)/A94</f>
+      <c r="D94" s="13">
+        <f>(1-C94*Quotes!$B$2*SUM($D$3:D93))/(1+C94*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E94" s="10">
-        <f>(C93/C94-1)/Quotes!$B$2</f>
+        <f>(1/D94-1)/B94</f>
+        <v/>
+      </c>
+      <c r="F94" s="10">
+        <f>(D93/D94-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="6">
+      <c r="A95" s="15">
+        <f>EDATE(Quotes!$E$2,3*93)</f>
+        <v/>
+      </c>
+      <c r="B95" s="6">
         <f>Interpolation!A95</f>
         <v/>
       </c>
-      <c r="B95" s="12">
+      <c r="C95" s="12">
         <f>Interpolation!E95</f>
         <v/>
       </c>
-      <c r="C95" s="13">
-        <f>(1-B95*Quotes!$B$2*SUM($C$3:C94))/(1+B95*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D95" s="10">
-        <f>(1/C95-1)/A95</f>
+      <c r="D95" s="13">
+        <f>(1-C95*Quotes!$B$2*SUM($D$3:D94))/(1+C95*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E95" s="10">
-        <f>(C94/C95-1)/Quotes!$B$2</f>
+        <f>(1/D95-1)/B95</f>
+        <v/>
+      </c>
+      <c r="F95" s="10">
+        <f>(D94/D95-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="6">
+      <c r="A96" s="15">
+        <f>EDATE(Quotes!$E$2,3*94)</f>
+        <v/>
+      </c>
+      <c r="B96" s="6">
         <f>Interpolation!A96</f>
         <v/>
       </c>
-      <c r="B96" s="12">
+      <c r="C96" s="12">
         <f>Interpolation!E96</f>
         <v/>
       </c>
-      <c r="C96" s="13">
-        <f>(1-B96*Quotes!$B$2*SUM($C$3:C95))/(1+B96*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D96" s="10">
-        <f>(1/C96-1)/A96</f>
+      <c r="D96" s="13">
+        <f>(1-C96*Quotes!$B$2*SUM($D$3:D95))/(1+C96*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E96" s="10">
-        <f>(C95/C96-1)/Quotes!$B$2</f>
+        <f>(1/D96-1)/B96</f>
+        <v/>
+      </c>
+      <c r="F96" s="10">
+        <f>(D95/D96-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="6">
+      <c r="A97" s="15">
+        <f>EDATE(Quotes!$E$2,3*95)</f>
+        <v/>
+      </c>
+      <c r="B97" s="6">
         <f>Interpolation!A97</f>
         <v/>
       </c>
-      <c r="B97" s="12">
+      <c r="C97" s="12">
         <f>Interpolation!E97</f>
         <v/>
       </c>
-      <c r="C97" s="13">
-        <f>(1-B97*Quotes!$B$2*SUM($C$3:C96))/(1+B97*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D97" s="10">
-        <f>(1/C97-1)/A97</f>
+      <c r="D97" s="13">
+        <f>(1-C97*Quotes!$B$2*SUM($D$3:D96))/(1+C97*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E97" s="10">
-        <f>(C96/C97-1)/Quotes!$B$2</f>
+        <f>(1/D97-1)/B97</f>
+        <v/>
+      </c>
+      <c r="F97" s="10">
+        <f>(D96/D97-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="6">
+      <c r="A98" s="15">
+        <f>EDATE(Quotes!$E$2,3*96)</f>
+        <v/>
+      </c>
+      <c r="B98" s="6">
         <f>Interpolation!A98</f>
         <v/>
       </c>
-      <c r="B98" s="12">
+      <c r="C98" s="12">
         <f>Interpolation!E98</f>
         <v/>
       </c>
-      <c r="C98" s="13">
-        <f>(1-B98*Quotes!$B$2*SUM($C$3:C97))/(1+B98*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D98" s="10">
-        <f>(1/C98-1)/A98</f>
+      <c r="D98" s="13">
+        <f>(1-C98*Quotes!$B$2*SUM($D$3:D97))/(1+C98*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E98" s="10">
-        <f>(C97/C98-1)/Quotes!$B$2</f>
+        <f>(1/D98-1)/B98</f>
+        <v/>
+      </c>
+      <c r="F98" s="10">
+        <f>(D97/D98-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="6">
+      <c r="A99" s="15">
+        <f>EDATE(Quotes!$E$2,3*97)</f>
+        <v/>
+      </c>
+      <c r="B99" s="6">
         <f>Interpolation!A99</f>
         <v/>
       </c>
-      <c r="B99" s="12">
+      <c r="C99" s="12">
         <f>Interpolation!E99</f>
         <v/>
       </c>
-      <c r="C99" s="13">
-        <f>(1-B99*Quotes!$B$2*SUM($C$3:C98))/(1+B99*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D99" s="10">
-        <f>(1/C99-1)/A99</f>
+      <c r="D99" s="13">
+        <f>(1-C99*Quotes!$B$2*SUM($D$3:D98))/(1+C99*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E99" s="10">
-        <f>(C98/C99-1)/Quotes!$B$2</f>
+        <f>(1/D99-1)/B99</f>
+        <v/>
+      </c>
+      <c r="F99" s="10">
+        <f>(D98/D99-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="6">
+      <c r="A100" s="15">
+        <f>EDATE(Quotes!$E$2,3*98)</f>
+        <v/>
+      </c>
+      <c r="B100" s="6">
         <f>Interpolation!A100</f>
         <v/>
       </c>
-      <c r="B100" s="12">
+      <c r="C100" s="12">
         <f>Interpolation!E100</f>
         <v/>
       </c>
-      <c r="C100" s="13">
-        <f>(1-B100*Quotes!$B$2*SUM($C$3:C99))/(1+B100*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D100" s="10">
-        <f>(1/C100-1)/A100</f>
+      <c r="D100" s="13">
+        <f>(1-C100*Quotes!$B$2*SUM($D$3:D99))/(1+C100*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E100" s="10">
-        <f>(C99/C100-1)/Quotes!$B$2</f>
+        <f>(1/D100-1)/B100</f>
+        <v/>
+      </c>
+      <c r="F100" s="10">
+        <f>(D99/D100-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="6">
+      <c r="A101" s="15">
+        <f>EDATE(Quotes!$E$2,3*99)</f>
+        <v/>
+      </c>
+      <c r="B101" s="6">
         <f>Interpolation!A101</f>
         <v/>
       </c>
-      <c r="B101" s="12">
+      <c r="C101" s="12">
         <f>Interpolation!E101</f>
         <v/>
       </c>
-      <c r="C101" s="13">
-        <f>(1-B101*Quotes!$B$2*SUM($C$3:C100))/(1+B101*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D101" s="10">
-        <f>(1/C101-1)/A101</f>
+      <c r="D101" s="13">
+        <f>(1-C101*Quotes!$B$2*SUM($D$3:D100))/(1+C101*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E101" s="10">
-        <f>(C100/C101-1)/Quotes!$B$2</f>
+        <f>(1/D101-1)/B101</f>
+        <v/>
+      </c>
+      <c r="F101" s="10">
+        <f>(D100/D101-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="6">
+      <c r="A102" s="15">
+        <f>EDATE(Quotes!$E$2,3*100)</f>
+        <v/>
+      </c>
+      <c r="B102" s="6">
         <f>Interpolation!A102</f>
         <v/>
       </c>
-      <c r="B102" s="12">
+      <c r="C102" s="12">
         <f>Interpolation!E102</f>
         <v/>
       </c>
-      <c r="C102" s="13">
-        <f>(1-B102*Quotes!$B$2*SUM($C$3:C101))/(1+B102*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D102" s="10">
-        <f>(1/C102-1)/A102</f>
+      <c r="D102" s="13">
+        <f>(1-C102*Quotes!$B$2*SUM($D$3:D101))/(1+C102*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E102" s="10">
-        <f>(C101/C102-1)/Quotes!$B$2</f>
+        <f>(1/D102-1)/B102</f>
+        <v/>
+      </c>
+      <c r="F102" s="10">
+        <f>(D101/D102-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="6">
+      <c r="A103" s="15">
+        <f>EDATE(Quotes!$E$2,3*101)</f>
+        <v/>
+      </c>
+      <c r="B103" s="6">
         <f>Interpolation!A103</f>
         <v/>
       </c>
-      <c r="B103" s="12">
+      <c r="C103" s="12">
         <f>Interpolation!E103</f>
         <v/>
       </c>
-      <c r="C103" s="13">
-        <f>(1-B103*Quotes!$B$2*SUM($C$3:C102))/(1+B103*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D103" s="10">
-        <f>(1/C103-1)/A103</f>
+      <c r="D103" s="13">
+        <f>(1-C103*Quotes!$B$2*SUM($D$3:D102))/(1+C103*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E103" s="10">
-        <f>(C102/C103-1)/Quotes!$B$2</f>
+        <f>(1/D103-1)/B103</f>
+        <v/>
+      </c>
+      <c r="F103" s="10">
+        <f>(D102/D103-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="6">
+      <c r="A104" s="15">
+        <f>EDATE(Quotes!$E$2,3*102)</f>
+        <v/>
+      </c>
+      <c r="B104" s="6">
         <f>Interpolation!A104</f>
         <v/>
       </c>
-      <c r="B104" s="12">
+      <c r="C104" s="12">
         <f>Interpolation!E104</f>
         <v/>
       </c>
-      <c r="C104" s="13">
-        <f>(1-B104*Quotes!$B$2*SUM($C$3:C103))/(1+B104*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D104" s="10">
-        <f>(1/C104-1)/A104</f>
+      <c r="D104" s="13">
+        <f>(1-C104*Quotes!$B$2*SUM($D$3:D103))/(1+C104*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E104" s="10">
-        <f>(C103/C104-1)/Quotes!$B$2</f>
+        <f>(1/D104-1)/B104</f>
+        <v/>
+      </c>
+      <c r="F104" s="10">
+        <f>(D103/D104-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="6">
+      <c r="A105" s="15">
+        <f>EDATE(Quotes!$E$2,3*103)</f>
+        <v/>
+      </c>
+      <c r="B105" s="6">
         <f>Interpolation!A105</f>
         <v/>
       </c>
-      <c r="B105" s="12">
+      <c r="C105" s="12">
         <f>Interpolation!E105</f>
         <v/>
       </c>
-      <c r="C105" s="13">
-        <f>(1-B105*Quotes!$B$2*SUM($C$3:C104))/(1+B105*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D105" s="10">
-        <f>(1/C105-1)/A105</f>
+      <c r="D105" s="13">
+        <f>(1-C105*Quotes!$B$2*SUM($D$3:D104))/(1+C105*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E105" s="10">
-        <f>(C104/C105-1)/Quotes!$B$2</f>
+        <f>(1/D105-1)/B105</f>
+        <v/>
+      </c>
+      <c r="F105" s="10">
+        <f>(D104/D105-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="6">
+      <c r="A106" s="15">
+        <f>EDATE(Quotes!$E$2,3*104)</f>
+        <v/>
+      </c>
+      <c r="B106" s="6">
         <f>Interpolation!A106</f>
         <v/>
       </c>
-      <c r="B106" s="12">
+      <c r="C106" s="12">
         <f>Interpolation!E106</f>
         <v/>
       </c>
-      <c r="C106" s="13">
-        <f>(1-B106*Quotes!$B$2*SUM($C$3:C105))/(1+B106*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D106" s="10">
-        <f>(1/C106-1)/A106</f>
+      <c r="D106" s="13">
+        <f>(1-C106*Quotes!$B$2*SUM($D$3:D105))/(1+C106*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E106" s="10">
-        <f>(C105/C106-1)/Quotes!$B$2</f>
+        <f>(1/D106-1)/B106</f>
+        <v/>
+      </c>
+      <c r="F106" s="10">
+        <f>(D105/D106-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="6">
+      <c r="A107" s="15">
+        <f>EDATE(Quotes!$E$2,3*105)</f>
+        <v/>
+      </c>
+      <c r="B107" s="6">
         <f>Interpolation!A107</f>
         <v/>
       </c>
-      <c r="B107" s="12">
+      <c r="C107" s="12">
         <f>Interpolation!E107</f>
         <v/>
       </c>
-      <c r="C107" s="13">
-        <f>(1-B107*Quotes!$B$2*SUM($C$3:C106))/(1+B107*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D107" s="10">
-        <f>(1/C107-1)/A107</f>
+      <c r="D107" s="13">
+        <f>(1-C107*Quotes!$B$2*SUM($D$3:D106))/(1+C107*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E107" s="10">
-        <f>(C106/C107-1)/Quotes!$B$2</f>
+        <f>(1/D107-1)/B107</f>
+        <v/>
+      </c>
+      <c r="F107" s="10">
+        <f>(D106/D107-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="6">
+      <c r="A108" s="15">
+        <f>EDATE(Quotes!$E$2,3*106)</f>
+        <v/>
+      </c>
+      <c r="B108" s="6">
         <f>Interpolation!A108</f>
         <v/>
       </c>
-      <c r="B108" s="12">
+      <c r="C108" s="12">
         <f>Interpolation!E108</f>
         <v/>
       </c>
-      <c r="C108" s="13">
-        <f>(1-B108*Quotes!$B$2*SUM($C$3:C107))/(1+B108*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D108" s="10">
-        <f>(1/C108-1)/A108</f>
+      <c r="D108" s="13">
+        <f>(1-C108*Quotes!$B$2*SUM($D$3:D107))/(1+C108*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E108" s="10">
-        <f>(C107/C108-1)/Quotes!$B$2</f>
+        <f>(1/D108-1)/B108</f>
+        <v/>
+      </c>
+      <c r="F108" s="10">
+        <f>(D107/D108-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="6">
+      <c r="A109" s="15">
+        <f>EDATE(Quotes!$E$2,3*107)</f>
+        <v/>
+      </c>
+      <c r="B109" s="6">
         <f>Interpolation!A109</f>
         <v/>
       </c>
-      <c r="B109" s="12">
+      <c r="C109" s="12">
         <f>Interpolation!E109</f>
         <v/>
       </c>
-      <c r="C109" s="13">
-        <f>(1-B109*Quotes!$B$2*SUM($C$3:C108))/(1+B109*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D109" s="10">
-        <f>(1/C109-1)/A109</f>
+      <c r="D109" s="13">
+        <f>(1-C109*Quotes!$B$2*SUM($D$3:D108))/(1+C109*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E109" s="10">
-        <f>(C108/C109-1)/Quotes!$B$2</f>
+        <f>(1/D109-1)/B109</f>
+        <v/>
+      </c>
+      <c r="F109" s="10">
+        <f>(D108/D109-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="6">
+      <c r="A110" s="15">
+        <f>EDATE(Quotes!$E$2,3*108)</f>
+        <v/>
+      </c>
+      <c r="B110" s="6">
         <f>Interpolation!A110</f>
         <v/>
       </c>
-      <c r="B110" s="12">
+      <c r="C110" s="12">
         <f>Interpolation!E110</f>
         <v/>
       </c>
-      <c r="C110" s="13">
-        <f>(1-B110*Quotes!$B$2*SUM($C$3:C109))/(1+B110*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D110" s="10">
-        <f>(1/C110-1)/A110</f>
+      <c r="D110" s="13">
+        <f>(1-C110*Quotes!$B$2*SUM($D$3:D109))/(1+C110*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E110" s="10">
-        <f>(C109/C110-1)/Quotes!$B$2</f>
+        <f>(1/D110-1)/B110</f>
+        <v/>
+      </c>
+      <c r="F110" s="10">
+        <f>(D109/D110-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="6">
+      <c r="A111" s="15">
+        <f>EDATE(Quotes!$E$2,3*109)</f>
+        <v/>
+      </c>
+      <c r="B111" s="6">
         <f>Interpolation!A111</f>
         <v/>
       </c>
-      <c r="B111" s="12">
+      <c r="C111" s="12">
         <f>Interpolation!E111</f>
         <v/>
       </c>
-      <c r="C111" s="13">
-        <f>(1-B111*Quotes!$B$2*SUM($C$3:C110))/(1+B111*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D111" s="10">
-        <f>(1/C111-1)/A111</f>
+      <c r="D111" s="13">
+        <f>(1-C111*Quotes!$B$2*SUM($D$3:D110))/(1+C111*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E111" s="10">
-        <f>(C110/C111-1)/Quotes!$B$2</f>
+        <f>(1/D111-1)/B111</f>
+        <v/>
+      </c>
+      <c r="F111" s="10">
+        <f>(D110/D111-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="6">
+      <c r="A112" s="15">
+        <f>EDATE(Quotes!$E$2,3*110)</f>
+        <v/>
+      </c>
+      <c r="B112" s="6">
         <f>Interpolation!A112</f>
         <v/>
       </c>
-      <c r="B112" s="12">
+      <c r="C112" s="12">
         <f>Interpolation!E112</f>
         <v/>
       </c>
-      <c r="C112" s="13">
-        <f>(1-B112*Quotes!$B$2*SUM($C$3:C111))/(1+B112*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D112" s="10">
-        <f>(1/C112-1)/A112</f>
+      <c r="D112" s="13">
+        <f>(1-C112*Quotes!$B$2*SUM($D$3:D111))/(1+C112*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E112" s="10">
-        <f>(C111/C112-1)/Quotes!$B$2</f>
+        <f>(1/D112-1)/B112</f>
+        <v/>
+      </c>
+      <c r="F112" s="10">
+        <f>(D111/D112-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="6">
+      <c r="A113" s="15">
+        <f>EDATE(Quotes!$E$2,3*111)</f>
+        <v/>
+      </c>
+      <c r="B113" s="6">
         <f>Interpolation!A113</f>
         <v/>
       </c>
-      <c r="B113" s="12">
+      <c r="C113" s="12">
         <f>Interpolation!E113</f>
         <v/>
       </c>
-      <c r="C113" s="13">
-        <f>(1-B113*Quotes!$B$2*SUM($C$3:C112))/(1+B113*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D113" s="10">
-        <f>(1/C113-1)/A113</f>
+      <c r="D113" s="13">
+        <f>(1-C113*Quotes!$B$2*SUM($D$3:D112))/(1+C113*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E113" s="10">
-        <f>(C112/C113-1)/Quotes!$B$2</f>
+        <f>(1/D113-1)/B113</f>
+        <v/>
+      </c>
+      <c r="F113" s="10">
+        <f>(D112/D113-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="6">
+      <c r="A114" s="15">
+        <f>EDATE(Quotes!$E$2,3*112)</f>
+        <v/>
+      </c>
+      <c r="B114" s="6">
         <f>Interpolation!A114</f>
         <v/>
       </c>
-      <c r="B114" s="12">
+      <c r="C114" s="12">
         <f>Interpolation!E114</f>
         <v/>
       </c>
-      <c r="C114" s="13">
-        <f>(1-B114*Quotes!$B$2*SUM($C$3:C113))/(1+B114*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D114" s="10">
-        <f>(1/C114-1)/A114</f>
+      <c r="D114" s="13">
+        <f>(1-C114*Quotes!$B$2*SUM($D$3:D113))/(1+C114*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E114" s="10">
-        <f>(C113/C114-1)/Quotes!$B$2</f>
+        <f>(1/D114-1)/B114</f>
+        <v/>
+      </c>
+      <c r="F114" s="10">
+        <f>(D113/D114-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="6">
+      <c r="A115" s="15">
+        <f>EDATE(Quotes!$E$2,3*113)</f>
+        <v/>
+      </c>
+      <c r="B115" s="6">
         <f>Interpolation!A115</f>
         <v/>
       </c>
-      <c r="B115" s="12">
+      <c r="C115" s="12">
         <f>Interpolation!E115</f>
         <v/>
       </c>
-      <c r="C115" s="13">
-        <f>(1-B115*Quotes!$B$2*SUM($C$3:C114))/(1+B115*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D115" s="10">
-        <f>(1/C115-1)/A115</f>
+      <c r="D115" s="13">
+        <f>(1-C115*Quotes!$B$2*SUM($D$3:D114))/(1+C115*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E115" s="10">
-        <f>(C114/C115-1)/Quotes!$B$2</f>
+        <f>(1/D115-1)/B115</f>
+        <v/>
+      </c>
+      <c r="F115" s="10">
+        <f>(D114/D115-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="6">
+      <c r="A116" s="15">
+        <f>EDATE(Quotes!$E$2,3*114)</f>
+        <v/>
+      </c>
+      <c r="B116" s="6">
         <f>Interpolation!A116</f>
         <v/>
       </c>
-      <c r="B116" s="12">
+      <c r="C116" s="12">
         <f>Interpolation!E116</f>
         <v/>
       </c>
-      <c r="C116" s="13">
-        <f>(1-B116*Quotes!$B$2*SUM($C$3:C115))/(1+B116*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D116" s="10">
-        <f>(1/C116-1)/A116</f>
+      <c r="D116" s="13">
+        <f>(1-C116*Quotes!$B$2*SUM($D$3:D115))/(1+C116*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E116" s="10">
-        <f>(C115/C116-1)/Quotes!$B$2</f>
+        <f>(1/D116-1)/B116</f>
+        <v/>
+      </c>
+      <c r="F116" s="10">
+        <f>(D115/D116-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="6">
+      <c r="A117" s="15">
+        <f>EDATE(Quotes!$E$2,3*115)</f>
+        <v/>
+      </c>
+      <c r="B117" s="6">
         <f>Interpolation!A117</f>
         <v/>
       </c>
-      <c r="B117" s="12">
+      <c r="C117" s="12">
         <f>Interpolation!E117</f>
         <v/>
       </c>
-      <c r="C117" s="13">
-        <f>(1-B117*Quotes!$B$2*SUM($C$3:C116))/(1+B117*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D117" s="10">
-        <f>(1/C117-1)/A117</f>
+      <c r="D117" s="13">
+        <f>(1-C117*Quotes!$B$2*SUM($D$3:D116))/(1+C117*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E117" s="10">
-        <f>(C116/C117-1)/Quotes!$B$2</f>
+        <f>(1/D117-1)/B117</f>
+        <v/>
+      </c>
+      <c r="F117" s="10">
+        <f>(D116/D117-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="6">
+      <c r="A118" s="15">
+        <f>EDATE(Quotes!$E$2,3*116)</f>
+        <v/>
+      </c>
+      <c r="B118" s="6">
         <f>Interpolation!A118</f>
         <v/>
       </c>
-      <c r="B118" s="12">
+      <c r="C118" s="12">
         <f>Interpolation!E118</f>
         <v/>
       </c>
-      <c r="C118" s="13">
-        <f>(1-B118*Quotes!$B$2*SUM($C$3:C117))/(1+B118*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D118" s="10">
-        <f>(1/C118-1)/A118</f>
+      <c r="D118" s="13">
+        <f>(1-C118*Quotes!$B$2*SUM($D$3:D117))/(1+C118*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E118" s="10">
-        <f>(C117/C118-1)/Quotes!$B$2</f>
+        <f>(1/D118-1)/B118</f>
+        <v/>
+      </c>
+      <c r="F118" s="10">
+        <f>(D117/D118-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="6">
+      <c r="A119" s="15">
+        <f>EDATE(Quotes!$E$2,3*117)</f>
+        <v/>
+      </c>
+      <c r="B119" s="6">
         <f>Interpolation!A119</f>
         <v/>
       </c>
-      <c r="B119" s="12">
+      <c r="C119" s="12">
         <f>Interpolation!E119</f>
         <v/>
       </c>
-      <c r="C119" s="13">
-        <f>(1-B119*Quotes!$B$2*SUM($C$3:C118))/(1+B119*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D119" s="10">
-        <f>(1/C119-1)/A119</f>
+      <c r="D119" s="13">
+        <f>(1-C119*Quotes!$B$2*SUM($D$3:D118))/(1+C119*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E119" s="10">
-        <f>(C118/C119-1)/Quotes!$B$2</f>
+        <f>(1/D119-1)/B119</f>
+        <v/>
+      </c>
+      <c r="F119" s="10">
+        <f>(D118/D119-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="6">
+      <c r="A120" s="15">
+        <f>EDATE(Quotes!$E$2,3*118)</f>
+        <v/>
+      </c>
+      <c r="B120" s="6">
         <f>Interpolation!A120</f>
         <v/>
       </c>
-      <c r="B120" s="12">
+      <c r="C120" s="12">
         <f>Interpolation!E120</f>
         <v/>
       </c>
-      <c r="C120" s="13">
-        <f>(1-B120*Quotes!$B$2*SUM($C$3:C119))/(1+B120*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D120" s="10">
-        <f>(1/C120-1)/A120</f>
+      <c r="D120" s="13">
+        <f>(1-C120*Quotes!$B$2*SUM($D$3:D119))/(1+C120*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E120" s="10">
-        <f>(C119/C120-1)/Quotes!$B$2</f>
+        <f>(1/D120-1)/B120</f>
+        <v/>
+      </c>
+      <c r="F120" s="10">
+        <f>(D119/D120-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="6">
+      <c r="A121" s="15">
+        <f>EDATE(Quotes!$E$2,3*119)</f>
+        <v/>
+      </c>
+      <c r="B121" s="6">
         <f>Interpolation!A121</f>
         <v/>
       </c>
-      <c r="B121" s="12">
+      <c r="C121" s="12">
         <f>Interpolation!E121</f>
         <v/>
       </c>
-      <c r="C121" s="13">
-        <f>(1-B121*Quotes!$B$2*SUM($C$3:C120))/(1+B121*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D121" s="10">
-        <f>(1/C121-1)/A121</f>
+      <c r="D121" s="13">
+        <f>(1-C121*Quotes!$B$2*SUM($D$3:D120))/(1+C121*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E121" s="10">
-        <f>(C120/C121-1)/Quotes!$B$2</f>
+        <f>(1/D121-1)/B121</f>
+        <v/>
+      </c>
+      <c r="F121" s="10">
+        <f>(D120/D121-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="6">
+      <c r="A122" s="15">
+        <f>EDATE(Quotes!$E$2,3*120)</f>
+        <v/>
+      </c>
+      <c r="B122" s="6">
         <f>Interpolation!A122</f>
         <v/>
       </c>
-      <c r="B122" s="12">
+      <c r="C122" s="12">
         <f>Interpolation!E122</f>
         <v/>
       </c>
-      <c r="C122" s="13">
-        <f>(1-B122*Quotes!$B$2*SUM($C$3:C121))/(1+B122*Quotes!$B$2)</f>
-        <v/>
-      </c>
-      <c r="D122" s="10">
-        <f>(1/C122-1)/A122</f>
+      <c r="D122" s="13">
+        <f>(1-C122*Quotes!$B$2*SUM($D$3:D121))/(1+C122*Quotes!$B$2)</f>
         <v/>
       </c>
       <c r="E122" s="10">
-        <f>(C121/C122-1)/Quotes!$B$2</f>
+        <f>(1/D122-1)/B122</f>
+        <v/>
+      </c>
+      <c r="F122" s="10">
+        <f>(D121/D122-1)/Quotes!$B$2</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
KRW: add Swap_Check - the 5Y reprice Kevin asked for
Kevin's next step: value a 5Y fixed-vs-float swap off the curve's own DF and
Future % and confirm it returns the 5Y quote. New Swap_Check sheet does exactly
that - 20 quarterly rows to 5Y, fixed CF = S*tau, float CF projected from the
forward column, both PV'd on the DFs, then the par rate = float PV / annuity.

Fixed leg 0.18422770, float leg 0.18422770 (equals 1 - DF(5Y), the telescoping
identity), net PV 0.00000000, par rate 4.0775% against the 4.0775% input - 0.0000
bp. It reprices to the last decimal because the par formula is the bootstrap
equation solved for S, so a match confirms no arithmetic slipped; a mismatch
would localise a broken DF or forward.

Caught before shipping: a note cell that began with "=" parsed as a formula.
Rewritten as plain text; zero formula errors after.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interpolation" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bootstrap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,14 +19,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.000%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="168" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="167" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="168" formatCode="0.0000%"/>
+    <numFmt numFmtId="169" formatCode="0.000000"/>
+    <numFmt numFmtId="170" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,8 +67,14 @@
       <color rgb="00008000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +99,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -119,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,8 +152,24 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -534,7 +564,7 @@
           <t>curve date</t>
         </is>
       </c>
-      <c r="E2" s="14" t="n">
+      <c r="E2" s="16" t="n">
         <v>46226</v>
       </c>
     </row>
@@ -4357,7 +4387,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15">
+      <c r="A3" s="17">
         <f>EDATE(Quotes!$E$2,3*1)</f>
         <v/>
       </c>
@@ -4383,7 +4413,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15">
+      <c r="A4" s="17">
         <f>EDATE(Quotes!$E$2,3*2)</f>
         <v/>
       </c>
@@ -4409,7 +4439,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15">
+      <c r="A5" s="17">
         <f>EDATE(Quotes!$E$2,3*3)</f>
         <v/>
       </c>
@@ -4435,7 +4465,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15">
+      <c r="A6" s="17">
         <f>EDATE(Quotes!$E$2,3*4)</f>
         <v/>
       </c>
@@ -4461,7 +4491,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15">
+      <c r="A7" s="17">
         <f>EDATE(Quotes!$E$2,3*5)</f>
         <v/>
       </c>
@@ -4487,7 +4517,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15">
+      <c r="A8" s="17">
         <f>EDATE(Quotes!$E$2,3*6)</f>
         <v/>
       </c>
@@ -4513,7 +4543,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15">
+      <c r="A9" s="17">
         <f>EDATE(Quotes!$E$2,3*7)</f>
         <v/>
       </c>
@@ -4539,7 +4569,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15">
+      <c r="A10" s="17">
         <f>EDATE(Quotes!$E$2,3*8)</f>
         <v/>
       </c>
@@ -4565,7 +4595,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15">
+      <c r="A11" s="17">
         <f>EDATE(Quotes!$E$2,3*9)</f>
         <v/>
       </c>
@@ -4591,7 +4621,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15">
+      <c r="A12" s="17">
         <f>EDATE(Quotes!$E$2,3*10)</f>
         <v/>
       </c>
@@ -4617,7 +4647,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15">
+      <c r="A13" s="17">
         <f>EDATE(Quotes!$E$2,3*11)</f>
         <v/>
       </c>
@@ -4643,7 +4673,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15">
+      <c r="A14" s="17">
         <f>EDATE(Quotes!$E$2,3*12)</f>
         <v/>
       </c>
@@ -4669,7 +4699,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15">
+      <c r="A15" s="17">
         <f>EDATE(Quotes!$E$2,3*13)</f>
         <v/>
       </c>
@@ -4695,7 +4725,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15">
+      <c r="A16" s="17">
         <f>EDATE(Quotes!$E$2,3*14)</f>
         <v/>
       </c>
@@ -4721,7 +4751,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15">
+      <c r="A17" s="17">
         <f>EDATE(Quotes!$E$2,3*15)</f>
         <v/>
       </c>
@@ -4747,7 +4777,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15">
+      <c r="A18" s="17">
         <f>EDATE(Quotes!$E$2,3*16)</f>
         <v/>
       </c>
@@ -4773,7 +4803,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15">
+      <c r="A19" s="17">
         <f>EDATE(Quotes!$E$2,3*17)</f>
         <v/>
       </c>
@@ -4799,7 +4829,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15">
+      <c r="A20" s="17">
         <f>EDATE(Quotes!$E$2,3*18)</f>
         <v/>
       </c>
@@ -4825,7 +4855,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15">
+      <c r="A21" s="17">
         <f>EDATE(Quotes!$E$2,3*19)</f>
         <v/>
       </c>
@@ -4851,7 +4881,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15">
+      <c r="A22" s="17">
         <f>EDATE(Quotes!$E$2,3*20)</f>
         <v/>
       </c>
@@ -4877,7 +4907,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15">
+      <c r="A23" s="17">
         <f>EDATE(Quotes!$E$2,3*21)</f>
         <v/>
       </c>
@@ -4903,7 +4933,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15">
+      <c r="A24" s="17">
         <f>EDATE(Quotes!$E$2,3*22)</f>
         <v/>
       </c>
@@ -4929,7 +4959,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15">
+      <c r="A25" s="17">
         <f>EDATE(Quotes!$E$2,3*23)</f>
         <v/>
       </c>
@@ -4955,7 +4985,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15">
+      <c r="A26" s="17">
         <f>EDATE(Quotes!$E$2,3*24)</f>
         <v/>
       </c>
@@ -4981,7 +5011,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15">
+      <c r="A27" s="17">
         <f>EDATE(Quotes!$E$2,3*25)</f>
         <v/>
       </c>
@@ -5007,7 +5037,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15">
+      <c r="A28" s="17">
         <f>EDATE(Quotes!$E$2,3*26)</f>
         <v/>
       </c>
@@ -5033,7 +5063,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15">
+      <c r="A29" s="17">
         <f>EDATE(Quotes!$E$2,3*27)</f>
         <v/>
       </c>
@@ -5059,7 +5089,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15">
+      <c r="A30" s="17">
         <f>EDATE(Quotes!$E$2,3*28)</f>
         <v/>
       </c>
@@ -5085,7 +5115,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="15">
+      <c r="A31" s="17">
         <f>EDATE(Quotes!$E$2,3*29)</f>
         <v/>
       </c>
@@ -5111,7 +5141,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="15">
+      <c r="A32" s="17">
         <f>EDATE(Quotes!$E$2,3*30)</f>
         <v/>
       </c>
@@ -5137,7 +5167,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15">
+      <c r="A33" s="17">
         <f>EDATE(Quotes!$E$2,3*31)</f>
         <v/>
       </c>
@@ -5163,7 +5193,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="15">
+      <c r="A34" s="17">
         <f>EDATE(Quotes!$E$2,3*32)</f>
         <v/>
       </c>
@@ -5189,7 +5219,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="15">
+      <c r="A35" s="17">
         <f>EDATE(Quotes!$E$2,3*33)</f>
         <v/>
       </c>
@@ -5215,7 +5245,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="15">
+      <c r="A36" s="17">
         <f>EDATE(Quotes!$E$2,3*34)</f>
         <v/>
       </c>
@@ -5241,7 +5271,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="15">
+      <c r="A37" s="17">
         <f>EDATE(Quotes!$E$2,3*35)</f>
         <v/>
       </c>
@@ -5267,7 +5297,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="15">
+      <c r="A38" s="17">
         <f>EDATE(Quotes!$E$2,3*36)</f>
         <v/>
       </c>
@@ -5293,7 +5323,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="15">
+      <c r="A39" s="17">
         <f>EDATE(Quotes!$E$2,3*37)</f>
         <v/>
       </c>
@@ -5319,7 +5349,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="15">
+      <c r="A40" s="17">
         <f>EDATE(Quotes!$E$2,3*38)</f>
         <v/>
       </c>
@@ -5345,7 +5375,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="15">
+      <c r="A41" s="17">
         <f>EDATE(Quotes!$E$2,3*39)</f>
         <v/>
       </c>
@@ -5371,7 +5401,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="15">
+      <c r="A42" s="17">
         <f>EDATE(Quotes!$E$2,3*40)</f>
         <v/>
       </c>
@@ -5397,7 +5427,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="15">
+      <c r="A43" s="17">
         <f>EDATE(Quotes!$E$2,3*41)</f>
         <v/>
       </c>
@@ -5423,7 +5453,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="15">
+      <c r="A44" s="17">
         <f>EDATE(Quotes!$E$2,3*42)</f>
         <v/>
       </c>
@@ -5449,7 +5479,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="15">
+      <c r="A45" s="17">
         <f>EDATE(Quotes!$E$2,3*43)</f>
         <v/>
       </c>
@@ -5475,7 +5505,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="15">
+      <c r="A46" s="17">
         <f>EDATE(Quotes!$E$2,3*44)</f>
         <v/>
       </c>
@@ -5501,7 +5531,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="15">
+      <c r="A47" s="17">
         <f>EDATE(Quotes!$E$2,3*45)</f>
         <v/>
       </c>
@@ -5527,7 +5557,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="15">
+      <c r="A48" s="17">
         <f>EDATE(Quotes!$E$2,3*46)</f>
         <v/>
       </c>
@@ -5553,7 +5583,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="15">
+      <c r="A49" s="17">
         <f>EDATE(Quotes!$E$2,3*47)</f>
         <v/>
       </c>
@@ -5579,7 +5609,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="15">
+      <c r="A50" s="17">
         <f>EDATE(Quotes!$E$2,3*48)</f>
         <v/>
       </c>
@@ -5605,7 +5635,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="15">
+      <c r="A51" s="17">
         <f>EDATE(Quotes!$E$2,3*49)</f>
         <v/>
       </c>
@@ -5631,7 +5661,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="15">
+      <c r="A52" s="17">
         <f>EDATE(Quotes!$E$2,3*50)</f>
         <v/>
       </c>
@@ -5657,7 +5687,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="15">
+      <c r="A53" s="17">
         <f>EDATE(Quotes!$E$2,3*51)</f>
         <v/>
       </c>
@@ -5683,7 +5713,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="15">
+      <c r="A54" s="17">
         <f>EDATE(Quotes!$E$2,3*52)</f>
         <v/>
       </c>
@@ -5709,7 +5739,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="15">
+      <c r="A55" s="17">
         <f>EDATE(Quotes!$E$2,3*53)</f>
         <v/>
       </c>
@@ -5735,7 +5765,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="15">
+      <c r="A56" s="17">
         <f>EDATE(Quotes!$E$2,3*54)</f>
         <v/>
       </c>
@@ -5761,7 +5791,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="15">
+      <c r="A57" s="17">
         <f>EDATE(Quotes!$E$2,3*55)</f>
         <v/>
       </c>
@@ -5787,7 +5817,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="15">
+      <c r="A58" s="17">
         <f>EDATE(Quotes!$E$2,3*56)</f>
         <v/>
       </c>
@@ -5813,7 +5843,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="15">
+      <c r="A59" s="17">
         <f>EDATE(Quotes!$E$2,3*57)</f>
         <v/>
       </c>
@@ -5839,7 +5869,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="15">
+      <c r="A60" s="17">
         <f>EDATE(Quotes!$E$2,3*58)</f>
         <v/>
       </c>
@@ -5865,7 +5895,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="15">
+      <c r="A61" s="17">
         <f>EDATE(Quotes!$E$2,3*59)</f>
         <v/>
       </c>
@@ -5891,7 +5921,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="15">
+      <c r="A62" s="17">
         <f>EDATE(Quotes!$E$2,3*60)</f>
         <v/>
       </c>
@@ -5917,7 +5947,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="15">
+      <c r="A63" s="17">
         <f>EDATE(Quotes!$E$2,3*61)</f>
         <v/>
       </c>
@@ -5943,7 +5973,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="15">
+      <c r="A64" s="17">
         <f>EDATE(Quotes!$E$2,3*62)</f>
         <v/>
       </c>
@@ -5969,7 +5999,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="15">
+      <c r="A65" s="17">
         <f>EDATE(Quotes!$E$2,3*63)</f>
         <v/>
       </c>
@@ -5995,7 +6025,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="15">
+      <c r="A66" s="17">
         <f>EDATE(Quotes!$E$2,3*64)</f>
         <v/>
       </c>
@@ -6021,7 +6051,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="15">
+      <c r="A67" s="17">
         <f>EDATE(Quotes!$E$2,3*65)</f>
         <v/>
       </c>
@@ -6047,7 +6077,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="15">
+      <c r="A68" s="17">
         <f>EDATE(Quotes!$E$2,3*66)</f>
         <v/>
       </c>
@@ -6073,7 +6103,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="15">
+      <c r="A69" s="17">
         <f>EDATE(Quotes!$E$2,3*67)</f>
         <v/>
       </c>
@@ -6099,7 +6129,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="15">
+      <c r="A70" s="17">
         <f>EDATE(Quotes!$E$2,3*68)</f>
         <v/>
       </c>
@@ -6125,7 +6155,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="15">
+      <c r="A71" s="17">
         <f>EDATE(Quotes!$E$2,3*69)</f>
         <v/>
       </c>
@@ -6151,7 +6181,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="15">
+      <c r="A72" s="17">
         <f>EDATE(Quotes!$E$2,3*70)</f>
         <v/>
       </c>
@@ -6177,7 +6207,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="15">
+      <c r="A73" s="17">
         <f>EDATE(Quotes!$E$2,3*71)</f>
         <v/>
       </c>
@@ -6203,7 +6233,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="15">
+      <c r="A74" s="17">
         <f>EDATE(Quotes!$E$2,3*72)</f>
         <v/>
       </c>
@@ -6229,7 +6259,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="15">
+      <c r="A75" s="17">
         <f>EDATE(Quotes!$E$2,3*73)</f>
         <v/>
       </c>
@@ -6255,7 +6285,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="15">
+      <c r="A76" s="17">
         <f>EDATE(Quotes!$E$2,3*74)</f>
         <v/>
       </c>
@@ -6281,7 +6311,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="15">
+      <c r="A77" s="17">
         <f>EDATE(Quotes!$E$2,3*75)</f>
         <v/>
       </c>
@@ -6307,7 +6337,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="15">
+      <c r="A78" s="17">
         <f>EDATE(Quotes!$E$2,3*76)</f>
         <v/>
       </c>
@@ -6333,7 +6363,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="15">
+      <c r="A79" s="17">
         <f>EDATE(Quotes!$E$2,3*77)</f>
         <v/>
       </c>
@@ -6359,7 +6389,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="15">
+      <c r="A80" s="17">
         <f>EDATE(Quotes!$E$2,3*78)</f>
         <v/>
       </c>
@@ -6385,7 +6415,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="15">
+      <c r="A81" s="17">
         <f>EDATE(Quotes!$E$2,3*79)</f>
         <v/>
       </c>
@@ -6411,7 +6441,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="15">
+      <c r="A82" s="17">
         <f>EDATE(Quotes!$E$2,3*80)</f>
         <v/>
       </c>
@@ -6437,7 +6467,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="15">
+      <c r="A83" s="17">
         <f>EDATE(Quotes!$E$2,3*81)</f>
         <v/>
       </c>
@@ -6463,7 +6493,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="15">
+      <c r="A84" s="17">
         <f>EDATE(Quotes!$E$2,3*82)</f>
         <v/>
       </c>
@@ -6489,7 +6519,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="15">
+      <c r="A85" s="17">
         <f>EDATE(Quotes!$E$2,3*83)</f>
         <v/>
       </c>
@@ -6515,7 +6545,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="15">
+      <c r="A86" s="17">
         <f>EDATE(Quotes!$E$2,3*84)</f>
         <v/>
       </c>
@@ -6541,7 +6571,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="15">
+      <c r="A87" s="17">
         <f>EDATE(Quotes!$E$2,3*85)</f>
         <v/>
       </c>
@@ -6567,7 +6597,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="15">
+      <c r="A88" s="17">
         <f>EDATE(Quotes!$E$2,3*86)</f>
         <v/>
       </c>
@@ -6593,7 +6623,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="15">
+      <c r="A89" s="17">
         <f>EDATE(Quotes!$E$2,3*87)</f>
         <v/>
       </c>
@@ -6619,7 +6649,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="15">
+      <c r="A90" s="17">
         <f>EDATE(Quotes!$E$2,3*88)</f>
         <v/>
       </c>
@@ -6645,7 +6675,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="15">
+      <c r="A91" s="17">
         <f>EDATE(Quotes!$E$2,3*89)</f>
         <v/>
       </c>
@@ -6671,7 +6701,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="15">
+      <c r="A92" s="17">
         <f>EDATE(Quotes!$E$2,3*90)</f>
         <v/>
       </c>
@@ -6697,7 +6727,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="15">
+      <c r="A93" s="17">
         <f>EDATE(Quotes!$E$2,3*91)</f>
         <v/>
       </c>
@@ -6723,7 +6753,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="15">
+      <c r="A94" s="17">
         <f>EDATE(Quotes!$E$2,3*92)</f>
         <v/>
       </c>
@@ -6749,7 +6779,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="15">
+      <c r="A95" s="17">
         <f>EDATE(Quotes!$E$2,3*93)</f>
         <v/>
       </c>
@@ -6775,7 +6805,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="15">
+      <c r="A96" s="17">
         <f>EDATE(Quotes!$E$2,3*94)</f>
         <v/>
       </c>
@@ -6801,7 +6831,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="15">
+      <c r="A97" s="17">
         <f>EDATE(Quotes!$E$2,3*95)</f>
         <v/>
       </c>
@@ -6827,7 +6857,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="15">
+      <c r="A98" s="17">
         <f>EDATE(Quotes!$E$2,3*96)</f>
         <v/>
       </c>
@@ -6853,7 +6883,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="15">
+      <c r="A99" s="17">
         <f>EDATE(Quotes!$E$2,3*97)</f>
         <v/>
       </c>
@@ -6879,7 +6909,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="15">
+      <c r="A100" s="17">
         <f>EDATE(Quotes!$E$2,3*98)</f>
         <v/>
       </c>
@@ -6905,7 +6935,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="15">
+      <c r="A101" s="17">
         <f>EDATE(Quotes!$E$2,3*99)</f>
         <v/>
       </c>
@@ -6931,7 +6961,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="15">
+      <c r="A102" s="17">
         <f>EDATE(Quotes!$E$2,3*100)</f>
         <v/>
       </c>
@@ -6957,7 +6987,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="15">
+      <c r="A103" s="17">
         <f>EDATE(Quotes!$E$2,3*101)</f>
         <v/>
       </c>
@@ -6983,7 +7013,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="15">
+      <c r="A104" s="17">
         <f>EDATE(Quotes!$E$2,3*102)</f>
         <v/>
       </c>
@@ -7009,7 +7039,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="15">
+      <c r="A105" s="17">
         <f>EDATE(Quotes!$E$2,3*103)</f>
         <v/>
       </c>
@@ -7035,7 +7065,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="15">
+      <c r="A106" s="17">
         <f>EDATE(Quotes!$E$2,3*104)</f>
         <v/>
       </c>
@@ -7061,7 +7091,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="15">
+      <c r="A107" s="17">
         <f>EDATE(Quotes!$E$2,3*105)</f>
         <v/>
       </c>
@@ -7087,7 +7117,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="15">
+      <c r="A108" s="17">
         <f>EDATE(Quotes!$E$2,3*106)</f>
         <v/>
       </c>
@@ -7113,7 +7143,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="15">
+      <c r="A109" s="17">
         <f>EDATE(Quotes!$E$2,3*107)</f>
         <v/>
       </c>
@@ -7139,7 +7169,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="15">
+      <c r="A110" s="17">
         <f>EDATE(Quotes!$E$2,3*108)</f>
         <v/>
       </c>
@@ -7165,7 +7195,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="15">
+      <c r="A111" s="17">
         <f>EDATE(Quotes!$E$2,3*109)</f>
         <v/>
       </c>
@@ -7191,7 +7221,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="15">
+      <c r="A112" s="17">
         <f>EDATE(Quotes!$E$2,3*110)</f>
         <v/>
       </c>
@@ -7217,7 +7247,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="15">
+      <c r="A113" s="17">
         <f>EDATE(Quotes!$E$2,3*111)</f>
         <v/>
       </c>
@@ -7243,7 +7273,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="15">
+      <c r="A114" s="17">
         <f>EDATE(Quotes!$E$2,3*112)</f>
         <v/>
       </c>
@@ -7269,7 +7299,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="15">
+      <c r="A115" s="17">
         <f>EDATE(Quotes!$E$2,3*113)</f>
         <v/>
       </c>
@@ -7295,7 +7325,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="15">
+      <c r="A116" s="17">
         <f>EDATE(Quotes!$E$2,3*114)</f>
         <v/>
       </c>
@@ -7321,7 +7351,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="15">
+      <c r="A117" s="17">
         <f>EDATE(Quotes!$E$2,3*115)</f>
         <v/>
       </c>
@@ -7347,7 +7377,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="15">
+      <c r="A118" s="17">
         <f>EDATE(Quotes!$E$2,3*116)</f>
         <v/>
       </c>
@@ -7373,7 +7403,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="15">
+      <c r="A119" s="17">
         <f>EDATE(Quotes!$E$2,3*117)</f>
         <v/>
       </c>
@@ -7399,7 +7429,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="15">
+      <c r="A120" s="17">
         <f>EDATE(Quotes!$E$2,3*118)</f>
         <v/>
       </c>
@@ -7425,7 +7455,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="15">
+      <c r="A121" s="17">
         <f>EDATE(Quotes!$E$2,3*119)</f>
         <v/>
       </c>
@@ -7451,7 +7481,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="15">
+      <c r="A122" s="17">
         <f>EDATE(Quotes!$E$2,3*120)</f>
         <v/>
       </c>
@@ -7474,6 +7504,966 @@
       <c r="F122" s="10">
         <f>(D121/D122-1)/Quotes!$B$2</f>
         <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>5Y swap repriced on the curve</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Kevin's check: value a 5Y fixed-vs-float swap using the DF and Future % from Bootstrap. The par rate should come back to the 5Y quote you built the curve from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Maturity (yrs)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Fixed rate (test)</t>
+        </is>
+      </c>
+      <c r="B5" s="18">
+        <f>Quotes!B12</f>
+        <v/>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>the 5Y quote (4.0775%); struck here, net PV should be ~0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>tau</t>
+        </is>
+      </c>
+      <c r="B6" s="19">
+        <f>Quotes!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>Forward %</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Fixed CF</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Float CF</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>PV fixed</t>
+        </is>
+      </c>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>PV float</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="21">
+        <f>Bootstrap!B3</f>
+        <v/>
+      </c>
+      <c r="C9" s="22">
+        <f>Bootstrap!A3</f>
+        <v/>
+      </c>
+      <c r="D9" s="23">
+        <f>Bootstrap!D3</f>
+        <v/>
+      </c>
+      <c r="E9" s="24">
+        <f>Bootstrap!F3</f>
+        <v/>
+      </c>
+      <c r="F9" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G9" s="25">
+        <f>E9*$B$6</f>
+        <v/>
+      </c>
+      <c r="H9" s="25">
+        <f>F9*D9</f>
+        <v/>
+      </c>
+      <c r="I9" s="25">
+        <f>G9*D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="21">
+        <f>Bootstrap!B4</f>
+        <v/>
+      </c>
+      <c r="C10" s="22">
+        <f>Bootstrap!A4</f>
+        <v/>
+      </c>
+      <c r="D10" s="23">
+        <f>Bootstrap!D4</f>
+        <v/>
+      </c>
+      <c r="E10" s="24">
+        <f>Bootstrap!F4</f>
+        <v/>
+      </c>
+      <c r="F10" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G10" s="25">
+        <f>E10*$B$6</f>
+        <v/>
+      </c>
+      <c r="H10" s="25">
+        <f>F10*D10</f>
+        <v/>
+      </c>
+      <c r="I10" s="25">
+        <f>G10*D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="21">
+        <f>Bootstrap!B5</f>
+        <v/>
+      </c>
+      <c r="C11" s="22">
+        <f>Bootstrap!A5</f>
+        <v/>
+      </c>
+      <c r="D11" s="23">
+        <f>Bootstrap!D5</f>
+        <v/>
+      </c>
+      <c r="E11" s="24">
+        <f>Bootstrap!F5</f>
+        <v/>
+      </c>
+      <c r="F11" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G11" s="25">
+        <f>E11*$B$6</f>
+        <v/>
+      </c>
+      <c r="H11" s="25">
+        <f>F11*D11</f>
+        <v/>
+      </c>
+      <c r="I11" s="25">
+        <f>G11*D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="21">
+        <f>Bootstrap!B6</f>
+        <v/>
+      </c>
+      <c r="C12" s="22">
+        <f>Bootstrap!A6</f>
+        <v/>
+      </c>
+      <c r="D12" s="23">
+        <f>Bootstrap!D6</f>
+        <v/>
+      </c>
+      <c r="E12" s="24">
+        <f>Bootstrap!F6</f>
+        <v/>
+      </c>
+      <c r="F12" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G12" s="25">
+        <f>E12*$B$6</f>
+        <v/>
+      </c>
+      <c r="H12" s="25">
+        <f>F12*D12</f>
+        <v/>
+      </c>
+      <c r="I12" s="25">
+        <f>G12*D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="21">
+        <f>Bootstrap!B7</f>
+        <v/>
+      </c>
+      <c r="C13" s="22">
+        <f>Bootstrap!A7</f>
+        <v/>
+      </c>
+      <c r="D13" s="23">
+        <f>Bootstrap!D7</f>
+        <v/>
+      </c>
+      <c r="E13" s="24">
+        <f>Bootstrap!F7</f>
+        <v/>
+      </c>
+      <c r="F13" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G13" s="25">
+        <f>E13*$B$6</f>
+        <v/>
+      </c>
+      <c r="H13" s="25">
+        <f>F13*D13</f>
+        <v/>
+      </c>
+      <c r="I13" s="25">
+        <f>G13*D13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="21">
+        <f>Bootstrap!B8</f>
+        <v/>
+      </c>
+      <c r="C14" s="22">
+        <f>Bootstrap!A8</f>
+        <v/>
+      </c>
+      <c r="D14" s="23">
+        <f>Bootstrap!D8</f>
+        <v/>
+      </c>
+      <c r="E14" s="24">
+        <f>Bootstrap!F8</f>
+        <v/>
+      </c>
+      <c r="F14" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G14" s="25">
+        <f>E14*$B$6</f>
+        <v/>
+      </c>
+      <c r="H14" s="25">
+        <f>F14*D14</f>
+        <v/>
+      </c>
+      <c r="I14" s="25">
+        <f>G14*D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="21">
+        <f>Bootstrap!B9</f>
+        <v/>
+      </c>
+      <c r="C15" s="22">
+        <f>Bootstrap!A9</f>
+        <v/>
+      </c>
+      <c r="D15" s="23">
+        <f>Bootstrap!D9</f>
+        <v/>
+      </c>
+      <c r="E15" s="24">
+        <f>Bootstrap!F9</f>
+        <v/>
+      </c>
+      <c r="F15" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G15" s="25">
+        <f>E15*$B$6</f>
+        <v/>
+      </c>
+      <c r="H15" s="25">
+        <f>F15*D15</f>
+        <v/>
+      </c>
+      <c r="I15" s="25">
+        <f>G15*D15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="21">
+        <f>Bootstrap!B10</f>
+        <v/>
+      </c>
+      <c r="C16" s="22">
+        <f>Bootstrap!A10</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>Bootstrap!D10</f>
+        <v/>
+      </c>
+      <c r="E16" s="24">
+        <f>Bootstrap!F10</f>
+        <v/>
+      </c>
+      <c r="F16" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G16" s="25">
+        <f>E16*$B$6</f>
+        <v/>
+      </c>
+      <c r="H16" s="25">
+        <f>F16*D16</f>
+        <v/>
+      </c>
+      <c r="I16" s="25">
+        <f>G16*D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="21">
+        <f>Bootstrap!B11</f>
+        <v/>
+      </c>
+      <c r="C17" s="22">
+        <f>Bootstrap!A11</f>
+        <v/>
+      </c>
+      <c r="D17" s="23">
+        <f>Bootstrap!D11</f>
+        <v/>
+      </c>
+      <c r="E17" s="24">
+        <f>Bootstrap!F11</f>
+        <v/>
+      </c>
+      <c r="F17" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G17" s="25">
+        <f>E17*$B$6</f>
+        <v/>
+      </c>
+      <c r="H17" s="25">
+        <f>F17*D17</f>
+        <v/>
+      </c>
+      <c r="I17" s="25">
+        <f>G17*D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="21">
+        <f>Bootstrap!B12</f>
+        <v/>
+      </c>
+      <c r="C18" s="22">
+        <f>Bootstrap!A12</f>
+        <v/>
+      </c>
+      <c r="D18" s="23">
+        <f>Bootstrap!D12</f>
+        <v/>
+      </c>
+      <c r="E18" s="24">
+        <f>Bootstrap!F12</f>
+        <v/>
+      </c>
+      <c r="F18" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G18" s="25">
+        <f>E18*$B$6</f>
+        <v/>
+      </c>
+      <c r="H18" s="25">
+        <f>F18*D18</f>
+        <v/>
+      </c>
+      <c r="I18" s="25">
+        <f>G18*D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="21">
+        <f>Bootstrap!B13</f>
+        <v/>
+      </c>
+      <c r="C19" s="22">
+        <f>Bootstrap!A13</f>
+        <v/>
+      </c>
+      <c r="D19" s="23">
+        <f>Bootstrap!D13</f>
+        <v/>
+      </c>
+      <c r="E19" s="24">
+        <f>Bootstrap!F13</f>
+        <v/>
+      </c>
+      <c r="F19" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G19" s="25">
+        <f>E19*$B$6</f>
+        <v/>
+      </c>
+      <c r="H19" s="25">
+        <f>F19*D19</f>
+        <v/>
+      </c>
+      <c r="I19" s="25">
+        <f>G19*D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" s="21">
+        <f>Bootstrap!B14</f>
+        <v/>
+      </c>
+      <c r="C20" s="22">
+        <f>Bootstrap!A14</f>
+        <v/>
+      </c>
+      <c r="D20" s="23">
+        <f>Bootstrap!D14</f>
+        <v/>
+      </c>
+      <c r="E20" s="24">
+        <f>Bootstrap!F14</f>
+        <v/>
+      </c>
+      <c r="F20" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G20" s="25">
+        <f>E20*$B$6</f>
+        <v/>
+      </c>
+      <c r="H20" s="25">
+        <f>F20*D20</f>
+        <v/>
+      </c>
+      <c r="I20" s="25">
+        <f>G20*D20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B21" s="21">
+        <f>Bootstrap!B15</f>
+        <v/>
+      </c>
+      <c r="C21" s="22">
+        <f>Bootstrap!A15</f>
+        <v/>
+      </c>
+      <c r="D21" s="23">
+        <f>Bootstrap!D15</f>
+        <v/>
+      </c>
+      <c r="E21" s="24">
+        <f>Bootstrap!F15</f>
+        <v/>
+      </c>
+      <c r="F21" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G21" s="25">
+        <f>E21*$B$6</f>
+        <v/>
+      </c>
+      <c r="H21" s="25">
+        <f>F21*D21</f>
+        <v/>
+      </c>
+      <c r="I21" s="25">
+        <f>G21*D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B22" s="21">
+        <f>Bootstrap!B16</f>
+        <v/>
+      </c>
+      <c r="C22" s="22">
+        <f>Bootstrap!A16</f>
+        <v/>
+      </c>
+      <c r="D22" s="23">
+        <f>Bootstrap!D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="24">
+        <f>Bootstrap!F16</f>
+        <v/>
+      </c>
+      <c r="F22" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G22" s="25">
+        <f>E22*$B$6</f>
+        <v/>
+      </c>
+      <c r="H22" s="25">
+        <f>F22*D22</f>
+        <v/>
+      </c>
+      <c r="I22" s="25">
+        <f>G22*D22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="21">
+        <f>Bootstrap!B17</f>
+        <v/>
+      </c>
+      <c r="C23" s="22">
+        <f>Bootstrap!A17</f>
+        <v/>
+      </c>
+      <c r="D23" s="23">
+        <f>Bootstrap!D17</f>
+        <v/>
+      </c>
+      <c r="E23" s="24">
+        <f>Bootstrap!F17</f>
+        <v/>
+      </c>
+      <c r="F23" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G23" s="25">
+        <f>E23*$B$6</f>
+        <v/>
+      </c>
+      <c r="H23" s="25">
+        <f>F23*D23</f>
+        <v/>
+      </c>
+      <c r="I23" s="25">
+        <f>G23*D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="21">
+        <f>Bootstrap!B18</f>
+        <v/>
+      </c>
+      <c r="C24" s="22">
+        <f>Bootstrap!A18</f>
+        <v/>
+      </c>
+      <c r="D24" s="23">
+        <f>Bootstrap!D18</f>
+        <v/>
+      </c>
+      <c r="E24" s="24">
+        <f>Bootstrap!F18</f>
+        <v/>
+      </c>
+      <c r="F24" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G24" s="25">
+        <f>E24*$B$6</f>
+        <v/>
+      </c>
+      <c r="H24" s="25">
+        <f>F24*D24</f>
+        <v/>
+      </c>
+      <c r="I24" s="25">
+        <f>G24*D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" s="21">
+        <f>Bootstrap!B19</f>
+        <v/>
+      </c>
+      <c r="C25" s="22">
+        <f>Bootstrap!A19</f>
+        <v/>
+      </c>
+      <c r="D25" s="23">
+        <f>Bootstrap!D19</f>
+        <v/>
+      </c>
+      <c r="E25" s="24">
+        <f>Bootstrap!F19</f>
+        <v/>
+      </c>
+      <c r="F25" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G25" s="25">
+        <f>E25*$B$6</f>
+        <v/>
+      </c>
+      <c r="H25" s="25">
+        <f>F25*D25</f>
+        <v/>
+      </c>
+      <c r="I25" s="25">
+        <f>G25*D25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B26" s="21">
+        <f>Bootstrap!B20</f>
+        <v/>
+      </c>
+      <c r="C26" s="22">
+        <f>Bootstrap!A20</f>
+        <v/>
+      </c>
+      <c r="D26" s="23">
+        <f>Bootstrap!D20</f>
+        <v/>
+      </c>
+      <c r="E26" s="24">
+        <f>Bootstrap!F20</f>
+        <v/>
+      </c>
+      <c r="F26" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G26" s="25">
+        <f>E26*$B$6</f>
+        <v/>
+      </c>
+      <c r="H26" s="25">
+        <f>F26*D26</f>
+        <v/>
+      </c>
+      <c r="I26" s="25">
+        <f>G26*D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B27" s="21">
+        <f>Bootstrap!B21</f>
+        <v/>
+      </c>
+      <c r="C27" s="22">
+        <f>Bootstrap!A21</f>
+        <v/>
+      </c>
+      <c r="D27" s="23">
+        <f>Bootstrap!D21</f>
+        <v/>
+      </c>
+      <c r="E27" s="24">
+        <f>Bootstrap!F21</f>
+        <v/>
+      </c>
+      <c r="F27" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G27" s="25">
+        <f>E27*$B$6</f>
+        <v/>
+      </c>
+      <c r="H27" s="25">
+        <f>F27*D27</f>
+        <v/>
+      </c>
+      <c r="I27" s="25">
+        <f>G27*D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B28" s="21">
+        <f>Bootstrap!B22</f>
+        <v/>
+      </c>
+      <c r="C28" s="22">
+        <f>Bootstrap!A22</f>
+        <v/>
+      </c>
+      <c r="D28" s="23">
+        <f>Bootstrap!D22</f>
+        <v/>
+      </c>
+      <c r="E28" s="24">
+        <f>Bootstrap!F22</f>
+        <v/>
+      </c>
+      <c r="F28" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G28" s="25">
+        <f>E28*$B$6</f>
+        <v/>
+      </c>
+      <c r="H28" s="25">
+        <f>F28*D28</f>
+        <v/>
+      </c>
+      <c r="I28" s="25">
+        <f>G28*D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>PV fixed leg</t>
+        </is>
+      </c>
+      <c r="C30" s="26">
+        <f>SUM(H9:H28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>PV float leg</t>
+        </is>
+      </c>
+      <c r="C31" s="26">
+        <f>SUM(I9:I28)</f>
+        <v/>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>should equal 1 - DF(5Y)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Annuity  (tau*sum DF)</t>
+        </is>
+      </c>
+      <c r="C32" s="26">
+        <f>$B$6*SUM(D9:D28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Net PV  (float - fixed)</t>
+        </is>
+      </c>
+      <c r="C33" s="27">
+        <f>SUM(I9:I28)-SUM(H9:H28)</f>
+        <v/>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>~0 when struck at par</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>PAR SWAP RATE</t>
+        </is>
+      </c>
+      <c r="C35" s="28">
+        <f>SUM(I9:I28)/($B$6*SUM(D9:D28))</f>
+        <v/>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>float PV / annuity</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>5Y quote (target)</t>
+        </is>
+      </c>
+      <c r="C36" s="24">
+        <f>Quotes!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>difference (bp)</t>
+        </is>
+      </c>
+      <c r="C37" s="29">
+        <f>(C35-Quotes!B12)*10000</f>
+        <v/>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>should be ~0 — the curve reprices its own 5Y input</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add KRD-v3: Kevin's format by folding 8Y/9Y (full-grid, base NPV 0)
Third option that avoids the grid-approximation residual. Reads the
untouched full-grid KRD deltas (U69:AF69) and re-buckets 8Y/9Y into 7Y/10Y
by linear distance (8Y: 2/3->7Y,1/3->10Y; 9Y: 1/3->7Y,2/3->10Y). Frozen
rate and base NPV are KRD's own, so rate ties to Amort-Set-up!B12 and base
NPV=0, while TOTAL still equals the parallel DV01 (fold preserves the sum).
Fold 7Y/10Y match v2's from-scratch rebuild to ~1000 KRW.

Also repoint KRD-v2 frozen rate to 'Amort-Set-up'!B12 for consistency.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -14,8 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amort-Set-up" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD-v2" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD-v3" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -246,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -326,6 +327,8 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -941,6 +944,966 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>5Y swap repriced on the curve</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Kevin's check: value a 5Y fixed-vs-float swap using the DF and Future % from Bootstrap. The par rate should come back to the 5Y quote you built the curve from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Maturity (yrs)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Fixed rate (test)</t>
+        </is>
+      </c>
+      <c r="B5" s="18">
+        <f>Quotes!B12</f>
+        <v/>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>the 5Y quote (4.0775%); struck here, net PV should be ~0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>tau</t>
+        </is>
+      </c>
+      <c r="B6" s="19">
+        <f>Quotes!$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>Forward %</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Fixed CF</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Float CF</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>PV fixed</t>
+        </is>
+      </c>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>PV float</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="21">
+        <f>Bootstrap!B3</f>
+        <v/>
+      </c>
+      <c r="C9" s="22">
+        <f>Bootstrap!A3</f>
+        <v/>
+      </c>
+      <c r="D9" s="23">
+        <f>Bootstrap!D3</f>
+        <v/>
+      </c>
+      <c r="E9" s="24">
+        <f>Bootstrap!F3</f>
+        <v/>
+      </c>
+      <c r="F9" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G9" s="25">
+        <f>E9*$B$6</f>
+        <v/>
+      </c>
+      <c r="H9" s="25">
+        <f>F9*D9</f>
+        <v/>
+      </c>
+      <c r="I9" s="25">
+        <f>G9*D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="21">
+        <f>Bootstrap!B4</f>
+        <v/>
+      </c>
+      <c r="C10" s="22">
+        <f>Bootstrap!A4</f>
+        <v/>
+      </c>
+      <c r="D10" s="23">
+        <f>Bootstrap!D4</f>
+        <v/>
+      </c>
+      <c r="E10" s="24">
+        <f>Bootstrap!F4</f>
+        <v/>
+      </c>
+      <c r="F10" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G10" s="25">
+        <f>E10*$B$6</f>
+        <v/>
+      </c>
+      <c r="H10" s="25">
+        <f>F10*D10</f>
+        <v/>
+      </c>
+      <c r="I10" s="25">
+        <f>G10*D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="21">
+        <f>Bootstrap!B5</f>
+        <v/>
+      </c>
+      <c r="C11" s="22">
+        <f>Bootstrap!A5</f>
+        <v/>
+      </c>
+      <c r="D11" s="23">
+        <f>Bootstrap!D5</f>
+        <v/>
+      </c>
+      <c r="E11" s="24">
+        <f>Bootstrap!F5</f>
+        <v/>
+      </c>
+      <c r="F11" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G11" s="25">
+        <f>E11*$B$6</f>
+        <v/>
+      </c>
+      <c r="H11" s="25">
+        <f>F11*D11</f>
+        <v/>
+      </c>
+      <c r="I11" s="25">
+        <f>G11*D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="21">
+        <f>Bootstrap!B6</f>
+        <v/>
+      </c>
+      <c r="C12" s="22">
+        <f>Bootstrap!A6</f>
+        <v/>
+      </c>
+      <c r="D12" s="23">
+        <f>Bootstrap!D6</f>
+        <v/>
+      </c>
+      <c r="E12" s="24">
+        <f>Bootstrap!F6</f>
+        <v/>
+      </c>
+      <c r="F12" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G12" s="25">
+        <f>E12*$B$6</f>
+        <v/>
+      </c>
+      <c r="H12" s="25">
+        <f>F12*D12</f>
+        <v/>
+      </c>
+      <c r="I12" s="25">
+        <f>G12*D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="21">
+        <f>Bootstrap!B7</f>
+        <v/>
+      </c>
+      <c r="C13" s="22">
+        <f>Bootstrap!A7</f>
+        <v/>
+      </c>
+      <c r="D13" s="23">
+        <f>Bootstrap!D7</f>
+        <v/>
+      </c>
+      <c r="E13" s="24">
+        <f>Bootstrap!F7</f>
+        <v/>
+      </c>
+      <c r="F13" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G13" s="25">
+        <f>E13*$B$6</f>
+        <v/>
+      </c>
+      <c r="H13" s="25">
+        <f>F13*D13</f>
+        <v/>
+      </c>
+      <c r="I13" s="25">
+        <f>G13*D13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="21">
+        <f>Bootstrap!B8</f>
+        <v/>
+      </c>
+      <c r="C14" s="22">
+        <f>Bootstrap!A8</f>
+        <v/>
+      </c>
+      <c r="D14" s="23">
+        <f>Bootstrap!D8</f>
+        <v/>
+      </c>
+      <c r="E14" s="24">
+        <f>Bootstrap!F8</f>
+        <v/>
+      </c>
+      <c r="F14" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G14" s="25">
+        <f>E14*$B$6</f>
+        <v/>
+      </c>
+      <c r="H14" s="25">
+        <f>F14*D14</f>
+        <v/>
+      </c>
+      <c r="I14" s="25">
+        <f>G14*D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="21">
+        <f>Bootstrap!B9</f>
+        <v/>
+      </c>
+      <c r="C15" s="22">
+        <f>Bootstrap!A9</f>
+        <v/>
+      </c>
+      <c r="D15" s="23">
+        <f>Bootstrap!D9</f>
+        <v/>
+      </c>
+      <c r="E15" s="24">
+        <f>Bootstrap!F9</f>
+        <v/>
+      </c>
+      <c r="F15" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G15" s="25">
+        <f>E15*$B$6</f>
+        <v/>
+      </c>
+      <c r="H15" s="25">
+        <f>F15*D15</f>
+        <v/>
+      </c>
+      <c r="I15" s="25">
+        <f>G15*D15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="21">
+        <f>Bootstrap!B10</f>
+        <v/>
+      </c>
+      <c r="C16" s="22">
+        <f>Bootstrap!A10</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>Bootstrap!D10</f>
+        <v/>
+      </c>
+      <c r="E16" s="24">
+        <f>Bootstrap!F10</f>
+        <v/>
+      </c>
+      <c r="F16" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G16" s="25">
+        <f>E16*$B$6</f>
+        <v/>
+      </c>
+      <c r="H16" s="25">
+        <f>F16*D16</f>
+        <v/>
+      </c>
+      <c r="I16" s="25">
+        <f>G16*D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="21">
+        <f>Bootstrap!B11</f>
+        <v/>
+      </c>
+      <c r="C17" s="22">
+        <f>Bootstrap!A11</f>
+        <v/>
+      </c>
+      <c r="D17" s="23">
+        <f>Bootstrap!D11</f>
+        <v/>
+      </c>
+      <c r="E17" s="24">
+        <f>Bootstrap!F11</f>
+        <v/>
+      </c>
+      <c r="F17" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G17" s="25">
+        <f>E17*$B$6</f>
+        <v/>
+      </c>
+      <c r="H17" s="25">
+        <f>F17*D17</f>
+        <v/>
+      </c>
+      <c r="I17" s="25">
+        <f>G17*D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="21">
+        <f>Bootstrap!B12</f>
+        <v/>
+      </c>
+      <c r="C18" s="22">
+        <f>Bootstrap!A12</f>
+        <v/>
+      </c>
+      <c r="D18" s="23">
+        <f>Bootstrap!D12</f>
+        <v/>
+      </c>
+      <c r="E18" s="24">
+        <f>Bootstrap!F12</f>
+        <v/>
+      </c>
+      <c r="F18" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G18" s="25">
+        <f>E18*$B$6</f>
+        <v/>
+      </c>
+      <c r="H18" s="25">
+        <f>F18*D18</f>
+        <v/>
+      </c>
+      <c r="I18" s="25">
+        <f>G18*D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="21">
+        <f>Bootstrap!B13</f>
+        <v/>
+      </c>
+      <c r="C19" s="22">
+        <f>Bootstrap!A13</f>
+        <v/>
+      </c>
+      <c r="D19" s="23">
+        <f>Bootstrap!D13</f>
+        <v/>
+      </c>
+      <c r="E19" s="24">
+        <f>Bootstrap!F13</f>
+        <v/>
+      </c>
+      <c r="F19" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G19" s="25">
+        <f>E19*$B$6</f>
+        <v/>
+      </c>
+      <c r="H19" s="25">
+        <f>F19*D19</f>
+        <v/>
+      </c>
+      <c r="I19" s="25">
+        <f>G19*D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" s="21">
+        <f>Bootstrap!B14</f>
+        <v/>
+      </c>
+      <c r="C20" s="22">
+        <f>Bootstrap!A14</f>
+        <v/>
+      </c>
+      <c r="D20" s="23">
+        <f>Bootstrap!D14</f>
+        <v/>
+      </c>
+      <c r="E20" s="24">
+        <f>Bootstrap!F14</f>
+        <v/>
+      </c>
+      <c r="F20" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G20" s="25">
+        <f>E20*$B$6</f>
+        <v/>
+      </c>
+      <c r="H20" s="25">
+        <f>F20*D20</f>
+        <v/>
+      </c>
+      <c r="I20" s="25">
+        <f>G20*D20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B21" s="21">
+        <f>Bootstrap!B15</f>
+        <v/>
+      </c>
+      <c r="C21" s="22">
+        <f>Bootstrap!A15</f>
+        <v/>
+      </c>
+      <c r="D21" s="23">
+        <f>Bootstrap!D15</f>
+        <v/>
+      </c>
+      <c r="E21" s="24">
+        <f>Bootstrap!F15</f>
+        <v/>
+      </c>
+      <c r="F21" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G21" s="25">
+        <f>E21*$B$6</f>
+        <v/>
+      </c>
+      <c r="H21" s="25">
+        <f>F21*D21</f>
+        <v/>
+      </c>
+      <c r="I21" s="25">
+        <f>G21*D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B22" s="21">
+        <f>Bootstrap!B16</f>
+        <v/>
+      </c>
+      <c r="C22" s="22">
+        <f>Bootstrap!A16</f>
+        <v/>
+      </c>
+      <c r="D22" s="23">
+        <f>Bootstrap!D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="24">
+        <f>Bootstrap!F16</f>
+        <v/>
+      </c>
+      <c r="F22" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G22" s="25">
+        <f>E22*$B$6</f>
+        <v/>
+      </c>
+      <c r="H22" s="25">
+        <f>F22*D22</f>
+        <v/>
+      </c>
+      <c r="I22" s="25">
+        <f>G22*D22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="21">
+        <f>Bootstrap!B17</f>
+        <v/>
+      </c>
+      <c r="C23" s="22">
+        <f>Bootstrap!A17</f>
+        <v/>
+      </c>
+      <c r="D23" s="23">
+        <f>Bootstrap!D17</f>
+        <v/>
+      </c>
+      <c r="E23" s="24">
+        <f>Bootstrap!F17</f>
+        <v/>
+      </c>
+      <c r="F23" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G23" s="25">
+        <f>E23*$B$6</f>
+        <v/>
+      </c>
+      <c r="H23" s="25">
+        <f>F23*D23</f>
+        <v/>
+      </c>
+      <c r="I23" s="25">
+        <f>G23*D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="21">
+        <f>Bootstrap!B18</f>
+        <v/>
+      </c>
+      <c r="C24" s="22">
+        <f>Bootstrap!A18</f>
+        <v/>
+      </c>
+      <c r="D24" s="23">
+        <f>Bootstrap!D18</f>
+        <v/>
+      </c>
+      <c r="E24" s="24">
+        <f>Bootstrap!F18</f>
+        <v/>
+      </c>
+      <c r="F24" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G24" s="25">
+        <f>E24*$B$6</f>
+        <v/>
+      </c>
+      <c r="H24" s="25">
+        <f>F24*D24</f>
+        <v/>
+      </c>
+      <c r="I24" s="25">
+        <f>G24*D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" s="21">
+        <f>Bootstrap!B19</f>
+        <v/>
+      </c>
+      <c r="C25" s="22">
+        <f>Bootstrap!A19</f>
+        <v/>
+      </c>
+      <c r="D25" s="23">
+        <f>Bootstrap!D19</f>
+        <v/>
+      </c>
+      <c r="E25" s="24">
+        <f>Bootstrap!F19</f>
+        <v/>
+      </c>
+      <c r="F25" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G25" s="25">
+        <f>E25*$B$6</f>
+        <v/>
+      </c>
+      <c r="H25" s="25">
+        <f>F25*D25</f>
+        <v/>
+      </c>
+      <c r="I25" s="25">
+        <f>G25*D25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B26" s="21">
+        <f>Bootstrap!B20</f>
+        <v/>
+      </c>
+      <c r="C26" s="22">
+        <f>Bootstrap!A20</f>
+        <v/>
+      </c>
+      <c r="D26" s="23">
+        <f>Bootstrap!D20</f>
+        <v/>
+      </c>
+      <c r="E26" s="24">
+        <f>Bootstrap!F20</f>
+        <v/>
+      </c>
+      <c r="F26" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G26" s="25">
+        <f>E26*$B$6</f>
+        <v/>
+      </c>
+      <c r="H26" s="25">
+        <f>F26*D26</f>
+        <v/>
+      </c>
+      <c r="I26" s="25">
+        <f>G26*D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B27" s="21">
+        <f>Bootstrap!B21</f>
+        <v/>
+      </c>
+      <c r="C27" s="22">
+        <f>Bootstrap!A21</f>
+        <v/>
+      </c>
+      <c r="D27" s="23">
+        <f>Bootstrap!D21</f>
+        <v/>
+      </c>
+      <c r="E27" s="24">
+        <f>Bootstrap!F21</f>
+        <v/>
+      </c>
+      <c r="F27" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G27" s="25">
+        <f>E27*$B$6</f>
+        <v/>
+      </c>
+      <c r="H27" s="25">
+        <f>F27*D27</f>
+        <v/>
+      </c>
+      <c r="I27" s="25">
+        <f>G27*D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B28" s="21">
+        <f>Bootstrap!B22</f>
+        <v/>
+      </c>
+      <c r="C28" s="22">
+        <f>Bootstrap!A22</f>
+        <v/>
+      </c>
+      <c r="D28" s="23">
+        <f>Bootstrap!D22</f>
+        <v/>
+      </c>
+      <c r="E28" s="24">
+        <f>Bootstrap!F22</f>
+        <v/>
+      </c>
+      <c r="F28" s="25">
+        <f>$B$5*$B$6</f>
+        <v/>
+      </c>
+      <c r="G28" s="25">
+        <f>E28*$B$6</f>
+        <v/>
+      </c>
+      <c r="H28" s="25">
+        <f>F28*D28</f>
+        <v/>
+      </c>
+      <c r="I28" s="25">
+        <f>G28*D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>PV fixed leg</t>
+        </is>
+      </c>
+      <c r="C30" s="26">
+        <f>SUM(H9:H28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>PV float leg</t>
+        </is>
+      </c>
+      <c r="C31" s="26">
+        <f>SUM(I9:I28)</f>
+        <v/>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>should equal 1 - DF(5Y)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Annuity  (tau*sum DF)</t>
+        </is>
+      </c>
+      <c r="C32" s="26">
+        <f>$B$6*SUM(D9:D28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Net PV  (float - fixed)</t>
+        </is>
+      </c>
+      <c r="C33" s="27">
+        <f>SUM(I9:I28)-SUM(H9:H28)</f>
+        <v/>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>~0 when struck at par</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>PAR SWAP RATE</t>
+        </is>
+      </c>
+      <c r="C35" s="28">
+        <f>SUM(I9:I28)/($B$6*SUM(D9:D28))</f>
+        <v/>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>float PV / annuity</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>5Y quote (target)</t>
+        </is>
+      </c>
+      <c r="C36" s="24">
+        <f>Quotes!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>difference (bp)</t>
+        </is>
+      </c>
+      <c r="C37" s="29">
+        <f>(C35-Quotes!B12)*10000</f>
+        <v/>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>should be ~0 — the curve reprices its own 5Y input</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -23792,35 +24755,49 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="inlineStr">
+      <c r="A92" s="7" t="inlineStr">
         <is>
-          <t>base Float PV</t>
+          <t xml:space="preserve">  Kevin-grid float PV (diag)</t>
         </is>
       </c>
       <c r="C92" s="55">
         <f>SUMPRODUCT($E$51:$E$90,X$50:X$89-X$51:X$90)</f>
         <v/>
       </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>Kevin-grid par (diag):</t>
+        </is>
+      </c>
+      <c r="G92" s="73">
+        <f>C92/C93</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="inlineStr">
+      <c r="A93" s="7" t="inlineStr">
         <is>
-          <t>base annuity</t>
+          <t xml:space="preserve">  Kevin-grid annuity (diag)</t>
         </is>
       </c>
       <c r="C93" s="55">
         <f>Quotes!$B$2*SUMPRODUCT($E$51:$E$90,X$51:X$90)</f>
         <v/>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>base NPV residual = tiny grid diff (trade struck full-grid, priced Kevin-grid)</t>
+        </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>frozen par rate</t>
+          <t>frozen par rate (= trade rate, same as KRD)</t>
         </is>
       </c>
       <c r="C94" s="71">
-        <f>C92/C93</f>
+        <f>'Amort-Set-up'!$B$12</f>
         <v/>
       </c>
     </row>
@@ -24156,6 +25133,313 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KRD-v3 — Kevin's format by folding 8Y/9Y (full-grid pricing, untouched)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>No curve change: reads the existing KRD full-grid deltas and re-buckets 8Y/9Y into 7Y/10Y by linear distance (8Y: 2/3-&gt;7Y, 1/3-&gt;10Y; 9Y: 1/3-&gt;7Y, 2/3-&gt;10Y). Frozen rate and base NPV are KRD's own, so rate=4.2725% (your Amort-Set-up) and base NPV=0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Frozen rate (from KRD):</t>
+        </is>
+      </c>
+      <c r="C4" s="71">
+        <f>KRD!$D$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Base NPV (from KRD):</t>
+        </is>
+      </c>
+      <c r="C5" s="55">
+        <f>KRD!$T$68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="50" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="inlineStr">
+        <is>
+          <t>dv01</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2D</t>
+        </is>
+      </c>
+      <c r="B8" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="B9" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="B10" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
+      <c r="B11" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="B12" s="67">
+        <f>KRD!U69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>6M</t>
+        </is>
+      </c>
+      <c r="B13" s="67">
+        <f>KRD!V69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>9M</t>
+        </is>
+      </c>
+      <c r="B14" s="67">
+        <f>KRD!W69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1Y</t>
+        </is>
+      </c>
+      <c r="B15" s="67">
+        <f>KRD!X69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B16" s="67">
+        <f>KRD!Y69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B17" s="67">
+        <f>KRD!Z69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>4Y</t>
+        </is>
+      </c>
+      <c r="B18" s="67">
+        <f>KRD!AA69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B19" s="67">
+        <f>KRD!AB69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="B20" s="67">
+        <f>KRD!AC69+(2/3)*KRD!AD69+(1/3)*KRD!AE69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B21" s="67">
+        <f>KRD!AF69+(1/3)*KRD!AD69+(2/3)*KRD!AE69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>12Y</t>
+        </is>
+      </c>
+      <c r="B22" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>15Y</t>
+        </is>
+      </c>
+      <c r="B23" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>20Y</t>
+        </is>
+      </c>
+      <c r="B24" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>25Y</t>
+        </is>
+      </c>
+      <c r="B25" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>30Y</t>
+        </is>
+      </c>
+      <c r="B26" s="67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="68" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="69">
+        <f>SUM(B8:B26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL ties to KRD's parallel DV01 exactly: the fold keeps 7Y+8Y+9Y+10Y all in the sum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>folded 8Y (KRD AD69):</t>
+        </is>
+      </c>
+      <c r="C31" s="74">
+        <f>KRD!AD69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>folded 9Y (KRD AE69):</t>
+        </is>
+      </c>
+      <c r="C32" s="74">
+        <f>KRD!AE69</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28899,964 +30183,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>5Y swap repriced on the curve</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Kevin's check: value a 5Y fixed-vs-float swap using the DF and Future % from Bootstrap. The par rate should come back to the 5Y quote you built the curve from.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Maturity (yrs)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Fixed rate (test)</t>
-        </is>
-      </c>
-      <c r="B5" s="18">
-        <f>Quotes!B12</f>
-        <v/>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>the 5Y quote (4.0775%); struck here, net PV should be ~0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>tau</t>
-        </is>
-      </c>
-      <c r="B6" s="19">
-        <f>Quotes!$B$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>DF</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t>Forward %</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t>Fixed CF</t>
-        </is>
-      </c>
-      <c r="G8" s="20" t="inlineStr">
-        <is>
-          <t>Float CF</t>
-        </is>
-      </c>
-      <c r="H8" s="20" t="inlineStr">
-        <is>
-          <t>PV fixed</t>
-        </is>
-      </c>
-      <c r="I8" s="20" t="inlineStr">
-        <is>
-          <t>PV float</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="21">
-        <f>Bootstrap!B3</f>
-        <v/>
-      </c>
-      <c r="C9" s="22">
-        <f>Bootstrap!A3</f>
-        <v/>
-      </c>
-      <c r="D9" s="23">
-        <f>Bootstrap!D3</f>
-        <v/>
-      </c>
-      <c r="E9" s="24">
-        <f>Bootstrap!F3</f>
-        <v/>
-      </c>
-      <c r="F9" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G9" s="25">
-        <f>E9*$B$6</f>
-        <v/>
-      </c>
-      <c r="H9" s="25">
-        <f>F9*D9</f>
-        <v/>
-      </c>
-      <c r="I9" s="25">
-        <f>G9*D9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" s="21">
-        <f>Bootstrap!B4</f>
-        <v/>
-      </c>
-      <c r="C10" s="22">
-        <f>Bootstrap!A4</f>
-        <v/>
-      </c>
-      <c r="D10" s="23">
-        <f>Bootstrap!D4</f>
-        <v/>
-      </c>
-      <c r="E10" s="24">
-        <f>Bootstrap!F4</f>
-        <v/>
-      </c>
-      <c r="F10" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G10" s="25">
-        <f>E10*$B$6</f>
-        <v/>
-      </c>
-      <c r="H10" s="25">
-        <f>F10*D10</f>
-        <v/>
-      </c>
-      <c r="I10" s="25">
-        <f>G10*D10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B11" s="21">
-        <f>Bootstrap!B5</f>
-        <v/>
-      </c>
-      <c r="C11" s="22">
-        <f>Bootstrap!A5</f>
-        <v/>
-      </c>
-      <c r="D11" s="23">
-        <f>Bootstrap!D5</f>
-        <v/>
-      </c>
-      <c r="E11" s="24">
-        <f>Bootstrap!F5</f>
-        <v/>
-      </c>
-      <c r="F11" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G11" s="25">
-        <f>E11*$B$6</f>
-        <v/>
-      </c>
-      <c r="H11" s="25">
-        <f>F11*D11</f>
-        <v/>
-      </c>
-      <c r="I11" s="25">
-        <f>G11*D11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B12" s="21">
-        <f>Bootstrap!B6</f>
-        <v/>
-      </c>
-      <c r="C12" s="22">
-        <f>Bootstrap!A6</f>
-        <v/>
-      </c>
-      <c r="D12" s="23">
-        <f>Bootstrap!D6</f>
-        <v/>
-      </c>
-      <c r="E12" s="24">
-        <f>Bootstrap!F6</f>
-        <v/>
-      </c>
-      <c r="F12" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G12" s="25">
-        <f>E12*$B$6</f>
-        <v/>
-      </c>
-      <c r="H12" s="25">
-        <f>F12*D12</f>
-        <v/>
-      </c>
-      <c r="I12" s="25">
-        <f>G12*D12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B13" s="21">
-        <f>Bootstrap!B7</f>
-        <v/>
-      </c>
-      <c r="C13" s="22">
-        <f>Bootstrap!A7</f>
-        <v/>
-      </c>
-      <c r="D13" s="23">
-        <f>Bootstrap!D7</f>
-        <v/>
-      </c>
-      <c r="E13" s="24">
-        <f>Bootstrap!F7</f>
-        <v/>
-      </c>
-      <c r="F13" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G13" s="25">
-        <f>E13*$B$6</f>
-        <v/>
-      </c>
-      <c r="H13" s="25">
-        <f>F13*D13</f>
-        <v/>
-      </c>
-      <c r="I13" s="25">
-        <f>G13*D13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B14" s="21">
-        <f>Bootstrap!B8</f>
-        <v/>
-      </c>
-      <c r="C14" s="22">
-        <f>Bootstrap!A8</f>
-        <v/>
-      </c>
-      <c r="D14" s="23">
-        <f>Bootstrap!D8</f>
-        <v/>
-      </c>
-      <c r="E14" s="24">
-        <f>Bootstrap!F8</f>
-        <v/>
-      </c>
-      <c r="F14" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G14" s="25">
-        <f>E14*$B$6</f>
-        <v/>
-      </c>
-      <c r="H14" s="25">
-        <f>F14*D14</f>
-        <v/>
-      </c>
-      <c r="I14" s="25">
-        <f>G14*D14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B15" s="21">
-        <f>Bootstrap!B9</f>
-        <v/>
-      </c>
-      <c r="C15" s="22">
-        <f>Bootstrap!A9</f>
-        <v/>
-      </c>
-      <c r="D15" s="23">
-        <f>Bootstrap!D9</f>
-        <v/>
-      </c>
-      <c r="E15" s="24">
-        <f>Bootstrap!F9</f>
-        <v/>
-      </c>
-      <c r="F15" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G15" s="25">
-        <f>E15*$B$6</f>
-        <v/>
-      </c>
-      <c r="H15" s="25">
-        <f>F15*D15</f>
-        <v/>
-      </c>
-      <c r="I15" s="25">
-        <f>G15*D15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B16" s="21">
-        <f>Bootstrap!B10</f>
-        <v/>
-      </c>
-      <c r="C16" s="22">
-        <f>Bootstrap!A10</f>
-        <v/>
-      </c>
-      <c r="D16" s="23">
-        <f>Bootstrap!D10</f>
-        <v/>
-      </c>
-      <c r="E16" s="24">
-        <f>Bootstrap!F10</f>
-        <v/>
-      </c>
-      <c r="F16" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G16" s="25">
-        <f>E16*$B$6</f>
-        <v/>
-      </c>
-      <c r="H16" s="25">
-        <f>F16*D16</f>
-        <v/>
-      </c>
-      <c r="I16" s="25">
-        <f>G16*D16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B17" s="21">
-        <f>Bootstrap!B11</f>
-        <v/>
-      </c>
-      <c r="C17" s="22">
-        <f>Bootstrap!A11</f>
-        <v/>
-      </c>
-      <c r="D17" s="23">
-        <f>Bootstrap!D11</f>
-        <v/>
-      </c>
-      <c r="E17" s="24">
-        <f>Bootstrap!F11</f>
-        <v/>
-      </c>
-      <c r="F17" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G17" s="25">
-        <f>E17*$B$6</f>
-        <v/>
-      </c>
-      <c r="H17" s="25">
-        <f>F17*D17</f>
-        <v/>
-      </c>
-      <c r="I17" s="25">
-        <f>G17*D17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" s="21">
-        <f>Bootstrap!B12</f>
-        <v/>
-      </c>
-      <c r="C18" s="22">
-        <f>Bootstrap!A12</f>
-        <v/>
-      </c>
-      <c r="D18" s="23">
-        <f>Bootstrap!D12</f>
-        <v/>
-      </c>
-      <c r="E18" s="24">
-        <f>Bootstrap!F12</f>
-        <v/>
-      </c>
-      <c r="F18" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G18" s="25">
-        <f>E18*$B$6</f>
-        <v/>
-      </c>
-      <c r="H18" s="25">
-        <f>F18*D18</f>
-        <v/>
-      </c>
-      <c r="I18" s="25">
-        <f>G18*D18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B19" s="21">
-        <f>Bootstrap!B13</f>
-        <v/>
-      </c>
-      <c r="C19" s="22">
-        <f>Bootstrap!A13</f>
-        <v/>
-      </c>
-      <c r="D19" s="23">
-        <f>Bootstrap!D13</f>
-        <v/>
-      </c>
-      <c r="E19" s="24">
-        <f>Bootstrap!F13</f>
-        <v/>
-      </c>
-      <c r="F19" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G19" s="25">
-        <f>E19*$B$6</f>
-        <v/>
-      </c>
-      <c r="H19" s="25">
-        <f>F19*D19</f>
-        <v/>
-      </c>
-      <c r="I19" s="25">
-        <f>G19*D19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B20" s="21">
-        <f>Bootstrap!B14</f>
-        <v/>
-      </c>
-      <c r="C20" s="22">
-        <f>Bootstrap!A14</f>
-        <v/>
-      </c>
-      <c r="D20" s="23">
-        <f>Bootstrap!D14</f>
-        <v/>
-      </c>
-      <c r="E20" s="24">
-        <f>Bootstrap!F14</f>
-        <v/>
-      </c>
-      <c r="F20" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G20" s="25">
-        <f>E20*$B$6</f>
-        <v/>
-      </c>
-      <c r="H20" s="25">
-        <f>F20*D20</f>
-        <v/>
-      </c>
-      <c r="I20" s="25">
-        <f>G20*D20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B21" s="21">
-        <f>Bootstrap!B15</f>
-        <v/>
-      </c>
-      <c r="C21" s="22">
-        <f>Bootstrap!A15</f>
-        <v/>
-      </c>
-      <c r="D21" s="23">
-        <f>Bootstrap!D15</f>
-        <v/>
-      </c>
-      <c r="E21" s="24">
-        <f>Bootstrap!F15</f>
-        <v/>
-      </c>
-      <c r="F21" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G21" s="25">
-        <f>E21*$B$6</f>
-        <v/>
-      </c>
-      <c r="H21" s="25">
-        <f>F21*D21</f>
-        <v/>
-      </c>
-      <c r="I21" s="25">
-        <f>G21*D21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B22" s="21">
-        <f>Bootstrap!B16</f>
-        <v/>
-      </c>
-      <c r="C22" s="22">
-        <f>Bootstrap!A16</f>
-        <v/>
-      </c>
-      <c r="D22" s="23">
-        <f>Bootstrap!D16</f>
-        <v/>
-      </c>
-      <c r="E22" s="24">
-        <f>Bootstrap!F16</f>
-        <v/>
-      </c>
-      <c r="F22" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G22" s="25">
-        <f>E22*$B$6</f>
-        <v/>
-      </c>
-      <c r="H22" s="25">
-        <f>F22*D22</f>
-        <v/>
-      </c>
-      <c r="I22" s="25">
-        <f>G22*D22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B23" s="21">
-        <f>Bootstrap!B17</f>
-        <v/>
-      </c>
-      <c r="C23" s="22">
-        <f>Bootstrap!A17</f>
-        <v/>
-      </c>
-      <c r="D23" s="23">
-        <f>Bootstrap!D17</f>
-        <v/>
-      </c>
-      <c r="E23" s="24">
-        <f>Bootstrap!F17</f>
-        <v/>
-      </c>
-      <c r="F23" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G23" s="25">
-        <f>E23*$B$6</f>
-        <v/>
-      </c>
-      <c r="H23" s="25">
-        <f>F23*D23</f>
-        <v/>
-      </c>
-      <c r="I23" s="25">
-        <f>G23*D23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B24" s="21">
-        <f>Bootstrap!B18</f>
-        <v/>
-      </c>
-      <c r="C24" s="22">
-        <f>Bootstrap!A18</f>
-        <v/>
-      </c>
-      <c r="D24" s="23">
-        <f>Bootstrap!D18</f>
-        <v/>
-      </c>
-      <c r="E24" s="24">
-        <f>Bootstrap!F18</f>
-        <v/>
-      </c>
-      <c r="F24" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G24" s="25">
-        <f>E24*$B$6</f>
-        <v/>
-      </c>
-      <c r="H24" s="25">
-        <f>F24*D24</f>
-        <v/>
-      </c>
-      <c r="I24" s="25">
-        <f>G24*D24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B25" s="21">
-        <f>Bootstrap!B19</f>
-        <v/>
-      </c>
-      <c r="C25" s="22">
-        <f>Bootstrap!A19</f>
-        <v/>
-      </c>
-      <c r="D25" s="23">
-        <f>Bootstrap!D19</f>
-        <v/>
-      </c>
-      <c r="E25" s="24">
-        <f>Bootstrap!F19</f>
-        <v/>
-      </c>
-      <c r="F25" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G25" s="25">
-        <f>E25*$B$6</f>
-        <v/>
-      </c>
-      <c r="H25" s="25">
-        <f>F25*D25</f>
-        <v/>
-      </c>
-      <c r="I25" s="25">
-        <f>G25*D25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B26" s="21">
-        <f>Bootstrap!B20</f>
-        <v/>
-      </c>
-      <c r="C26" s="22">
-        <f>Bootstrap!A20</f>
-        <v/>
-      </c>
-      <c r="D26" s="23">
-        <f>Bootstrap!D20</f>
-        <v/>
-      </c>
-      <c r="E26" s="24">
-        <f>Bootstrap!F20</f>
-        <v/>
-      </c>
-      <c r="F26" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G26" s="25">
-        <f>E26*$B$6</f>
-        <v/>
-      </c>
-      <c r="H26" s="25">
-        <f>F26*D26</f>
-        <v/>
-      </c>
-      <c r="I26" s="25">
-        <f>G26*D26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B27" s="21">
-        <f>Bootstrap!B21</f>
-        <v/>
-      </c>
-      <c r="C27" s="22">
-        <f>Bootstrap!A21</f>
-        <v/>
-      </c>
-      <c r="D27" s="23">
-        <f>Bootstrap!D21</f>
-        <v/>
-      </c>
-      <c r="E27" s="24">
-        <f>Bootstrap!F21</f>
-        <v/>
-      </c>
-      <c r="F27" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G27" s="25">
-        <f>E27*$B$6</f>
-        <v/>
-      </c>
-      <c r="H27" s="25">
-        <f>F27*D27</f>
-        <v/>
-      </c>
-      <c r="I27" s="25">
-        <f>G27*D27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B28" s="21">
-        <f>Bootstrap!B22</f>
-        <v/>
-      </c>
-      <c r="C28" s="22">
-        <f>Bootstrap!A22</f>
-        <v/>
-      </c>
-      <c r="D28" s="23">
-        <f>Bootstrap!D22</f>
-        <v/>
-      </c>
-      <c r="E28" s="24">
-        <f>Bootstrap!F22</f>
-        <v/>
-      </c>
-      <c r="F28" s="25">
-        <f>$B$5*$B$6</f>
-        <v/>
-      </c>
-      <c r="G28" s="25">
-        <f>E28*$B$6</f>
-        <v/>
-      </c>
-      <c r="H28" s="25">
-        <f>F28*D28</f>
-        <v/>
-      </c>
-      <c r="I28" s="25">
-        <f>G28*D28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>PV fixed leg</t>
-        </is>
-      </c>
-      <c r="C30" s="26">
-        <f>SUM(H9:H28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>PV float leg</t>
-        </is>
-      </c>
-      <c r="C31" s="26">
-        <f>SUM(I9:I28)</f>
-        <v/>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>should equal 1 - DF(5Y)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Annuity  (tau*sum DF)</t>
-        </is>
-      </c>
-      <c r="C32" s="26">
-        <f>$B$6*SUM(D9:D28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Net PV  (float - fixed)</t>
-        </is>
-      </c>
-      <c r="C33" s="27">
-        <f>SUM(I9:I28)-SUM(H9:H28)</f>
-        <v/>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>~0 when struck at par</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>PAR SWAP RATE</t>
-        </is>
-      </c>
-      <c r="C35" s="28">
-        <f>SUM(I9:I28)/($B$6*SUM(D9:D28))</f>
-        <v/>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>float PV / annuity</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>5Y quote (target)</t>
-        </is>
-      </c>
-      <c r="C36" s="24">
-        <f>Quotes!B12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>difference (bp)</t>
-        </is>
-      </c>
-      <c r="C37" s="29">
-        <f>(C35-Quotes!B12)*10000</f>
-        <v/>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>should be ~0 — the curve reprices its own 5Y input</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Develop Hedge into a one-page blotter slide
Reads the folded Kevin-format deltas (KRD-v3 / Sheet1 in the master), sizes
each benchmark swap live off curve annuities, states receive/pay direction,
and shows the risk shape (front long / back short / net receiver) plus
before/after residual and the optional 7Y split. Master mapping to Sheet1
cells documented on the sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -37,7 +37,7 @@
     <numFmt numFmtId="171" formatCode="0.00000"/>
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -179,8 +179,35 @@
       <color rgb="00008000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -222,6 +249,11 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -249,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -334,6 +366,17 @@
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="27" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="28" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="26" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="28" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -30196,465 +30239,537 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Hedge — live notional sizing off the KRD buckets</t>
+      <c r="A1" s="78" t="inlineStr">
+        <is>
+          <t>Hedge proposal — KRW amortising IRS (10Y, HSBC receives fixed)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>notional(T) = group DV01 / (annuity(T) x 1bp). Positive DV01 -&gt; receive fixed, negative -&gt; pay fixed. Buckets grouped to liquid benchmarks; 3M/6M/9M left unhedged (dust). Re-sizes automatically as the trade or curve moves.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Bucketed KRD (Sheet1) hedged at liquid benchmarks. Notional(T) = group DV01 / (annuity(T) x 1bp), sized live off the curve; direction from the bucket sign.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Benchmark PV01 (from Bootstrap curve)</t>
-        </is>
-      </c>
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>1 · The risk</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="n"/>
+      <c r="C4" s="31" t="n"/>
+      <c r="D4" s="31" t="n"/>
+      <c r="E4" s="31" t="n"/>
+      <c r="F4" s="31" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="51" t="inlineStr">
+      <c r="A5" s="79" t="inlineStr">
+        <is>
+          <t>Net DV01</t>
+        </is>
+      </c>
+      <c r="B5" s="80">
+        <f>'KRD-v3'!$B$27</f>
+        <v/>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>KRW per bp — net receiver</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>Front 1Y–3Y</t>
+        </is>
+      </c>
+      <c r="B6" s="81">
+        <f>'KRD-v3'!$B$15+'KRD-v3'!$B$16+'KRD-v3'!$B$17</f>
+        <v/>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>long (positive) — pays if rates rise</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="79" t="inlineStr">
+        <is>
+          <t>Back 4Y–10Y</t>
+        </is>
+      </c>
+      <c r="B7" s="82">
+        <f>'KRD-v3'!$B$18+'KRD-v3'!$B$19+'KRD-v3'!$B$20+'KRD-v3'!$B$21</f>
+        <v/>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>short (negative) — concentrated at 10Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="79" t="inlineStr">
+        <is>
+          <t>Sub-1Y (3M/6M/9M)</t>
+        </is>
+      </c>
+      <c r="B8" s="74">
+        <f>'KRD-v3'!$B$12+'KRD-v3'!$B$13+'KRD-v3'!$B$14</f>
+        <v/>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>dust — leave unhedged</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>2 · Strategy</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="31" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="31" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="83" t="inlineStr">
+        <is>
+          <t>•  Hedge points, not buckets — trade the 4 liquid benchmarks (2Y/3Y/5Y/10Y), not all 10 nodes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="83" t="inlineStr">
+        <is>
+          <t>•  Fold orphans into the nearest benchmark: 1Y→2Y, 4Y→5Y, 7Y→10Y. Size to null the group DV01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="83" t="inlineStr">
+        <is>
+          <t>•  Skip the sub-1Y dust — its bid/offer costs more than the risk it removes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>3 · The trades  (4 swaps)</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="H15" s="79" t="inlineStr">
+        <is>
+          <t>Benchmark annuity (curve)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="50" t="inlineStr">
+        <is>
+          <t>Swap</t>
+        </is>
+      </c>
+      <c r="B16" s="50" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C16" s="50" t="inlineStr">
+        <is>
+          <t>Notional (bn)</t>
+        </is>
+      </c>
+      <c r="D16" s="50" t="inlineStr">
+        <is>
+          <t>Absorbs</t>
+        </is>
+      </c>
+      <c r="E16" s="50" t="inlineStr">
+        <is>
+          <t>Group DV01 (KRW/bp)</t>
+        </is>
+      </c>
+      <c r="F16" s="50" t="inlineStr">
+        <is>
+          <t>Annuity</t>
+        </is>
+      </c>
+      <c r="H16" s="51" t="inlineStr">
         <is>
           <t>Tenor</t>
         </is>
       </c>
-      <c r="B5" s="51" t="inlineStr">
-        <is>
-          <t>T (yrs)</t>
-        </is>
-      </c>
-      <c r="C5" s="51" t="inlineStr">
+      <c r="I16" s="51" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="J16" s="51" t="inlineStr">
         <is>
           <t>Annuity</t>
         </is>
       </c>
-      <c r="D5" s="51" t="inlineStr">
-        <is>
-          <t>DV01 / 100bn</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    </row>
+    <row r="17">
+      <c r="A17" s="84" t="inlineStr">
         <is>
           <t>2Y</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B17" s="84">
+        <f>IF(E17&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C17" s="85">
+        <f>ABS(E17/(F17*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>1Y + 2Y</t>
+        </is>
+      </c>
+      <c r="E17" s="41">
+        <f>'KRD-v3'!$B$15+'KRD-v3'!$B$16</f>
+        <v/>
+      </c>
+      <c r="F17" s="86">
+        <f>$J$17</f>
+        <v/>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B6,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="D6" s="55">
-        <f>100000000000*C6*0.0001</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="J17" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I17,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="84" t="inlineStr">
         <is>
           <t>3Y</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B18" s="84">
+        <f>IF(E18&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C18" s="85">
+        <f>ABS(E18/(F18*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="E18" s="41">
+        <f>'KRD-v3'!$B$17</f>
+        <v/>
+      </c>
+      <c r="F18" s="86">
+        <f>$J$18</f>
+        <v/>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B7,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="D7" s="55">
-        <f>100000000000*C7*0.0001</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="J18" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I18,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="84" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B19" s="84">
+        <f>IF(E19&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C19" s="85">
+        <f>ABS(E19/(F19*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>4Y + 5Y</t>
+        </is>
+      </c>
+      <c r="E19" s="41">
+        <f>'KRD-v3'!$B$18+'KRD-v3'!$B$19</f>
+        <v/>
+      </c>
+      <c r="F19" s="86">
+        <f>$J$19</f>
+        <v/>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B8,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="D8" s="55">
-        <f>100000000000*C8*0.0001</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="J19" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I19,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="84" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B20" s="84">
+        <f>IF(E20&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C20" s="85">
+        <f>ABS(E20/(F20*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>7Y + 10Y</t>
+        </is>
+      </c>
+      <c r="E20" s="41">
+        <f>'KRD-v3'!$B$20+'KRD-v3'!$B$21</f>
+        <v/>
+      </c>
+      <c r="F20" s="86">
+        <f>$J$21</f>
+        <v/>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>7Y</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="I20" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B9,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="D9" s="55">
-        <f>100000000000*C9*0.0001</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="J20" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I20,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="H21" t="inlineStr">
         <is>
           <t>10Y</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="I21" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B10,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="D10" s="55">
-        <f>100000000000*C10*0.0001</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Hedge proposal — 4 swaps</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="51" t="inlineStr">
-        <is>
-          <t>Hedge swap</t>
-        </is>
-      </c>
-      <c r="B13" s="51" t="inlineStr">
-        <is>
-          <t>Absorbs buckets</t>
-        </is>
-      </c>
-      <c r="C13" s="51" t="inlineStr">
+      <c r="J21" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I21,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>4 · After the hedge</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="n"/>
+      <c r="C22" s="31" t="n"/>
+      <c r="D22" s="31" t="n"/>
+      <c r="E22" s="31" t="n"/>
+      <c r="F22" s="31" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="79" t="inlineStr">
+        <is>
+          <t>Grouped buckets 2Y/3Y/5Y/10Y</t>
+        </is>
+      </c>
+      <c r="C23" s="83" t="inlineStr">
+        <is>
+          <t>neutralized to 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="79" t="inlineStr">
+        <is>
+          <t>Residual DV01</t>
+        </is>
+      </c>
+      <c r="C24" s="87">
+        <f>'KRD-v3'!$B$12+'KRD-v3'!$B$13+'KRD-v3'!$B$14</f>
+        <v/>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>sub-1Y dust only</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="79" t="inlineStr">
+        <is>
+          <t>Curve residual</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>small 7s10s (7Y folded into 10Y) — see option below</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>5 · Optional — split 7Y out (kills the 7s10s residual, +1 ticket)</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="31" t="n"/>
+      <c r="D27" s="31" t="n"/>
+      <c r="E27" s="31" t="n"/>
+      <c r="F27" s="31" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
+          <t>Swap</t>
+        </is>
+      </c>
+      <c r="B28" s="50" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C28" s="50" t="inlineStr">
+        <is>
+          <t>Notional (bn)</t>
+        </is>
+      </c>
+      <c r="D28" s="50" t="inlineStr">
+        <is>
+          <t>Absorbs</t>
+        </is>
+      </c>
+      <c r="E28" s="50" t="inlineStr">
         <is>
           <t>Group DV01 (KRW/bp)</t>
         </is>
       </c>
-      <c r="D13" s="51" t="inlineStr">
+      <c r="F28" s="50" t="inlineStr">
         <is>
           <t>Annuity</t>
         </is>
       </c>
-      <c r="E13" s="51" t="inlineStr">
-        <is>
-          <t>Notional (bn)</t>
-        </is>
-      </c>
-      <c r="F13" s="51" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>1Y + 2Y</t>
-        </is>
-      </c>
-      <c r="C14" s="55">
-        <f>KRD!X69+KRD!Y69</f>
-        <v/>
-      </c>
-      <c r="D14" s="75">
-        <f>$C$6</f>
-        <v/>
-      </c>
-      <c r="E14" s="76">
-        <f>ABS(C14/(D14*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="F14" s="2">
-        <f>IF(C14&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="C15" s="55">
-        <f>KRD!Z69</f>
-        <v/>
-      </c>
-      <c r="D15" s="75">
-        <f>$C$7</f>
-        <v/>
-      </c>
-      <c r="E15" s="76">
-        <f>ABS(C15/(D15*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="F15" s="2">
-        <f>IF(C15&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>5Y</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>4Y + 5Y</t>
-        </is>
-      </c>
-      <c r="C16" s="55">
-        <f>KRD!AA69+KRD!AB69</f>
-        <v/>
-      </c>
-      <c r="D16" s="75">
-        <f>$C$8</f>
-        <v/>
-      </c>
-      <c r="E16" s="76">
-        <f>ABS(C16/(D16*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="F16" s="2">
-        <f>IF(C16&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    </row>
+    <row r="29">
+      <c r="A29" s="84" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="B29" s="84">
+        <f>IF(E29&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C29" s="88">
+        <f>ABS(E29/(F29*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="E29" s="41">
+        <f>'KRD-v3'!$B$20</f>
+        <v/>
+      </c>
+      <c r="F29" s="86">
+        <f>$J$20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="84" t="inlineStr">
         <is>
           <t>10Y</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>7Y + 8Y + 9Y + 10Y</t>
-        </is>
-      </c>
-      <c r="C17" s="55">
-        <f>KRD!AC69+KRD!AD69+KRD!AE69+KRD!AF69</f>
-        <v/>
-      </c>
-      <c r="D17" s="75">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="E17" s="76">
-        <f>ABS(C17/(D17*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="F17" s="2">
-        <f>IF(C17&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>(unhedged)</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>3M + 6M + 9M (dust)</t>
-        </is>
-      </c>
-      <c r="C18" s="74">
-        <f>KRD!U69+KRD!V69+KRD!W69</f>
-        <v/>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>leave — bid/offer &gt; risk</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Net DV01 before hedge:</t>
-        </is>
-      </c>
-      <c r="C20" s="77">
-        <f>SUM(C14:C17)+C18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Hedged buckets (2Y/3Y/5Y/10Y groups):</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>neutralized to 0 by construction</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Residual DV01 after hedge:</t>
-        </is>
-      </c>
-      <c r="C22" s="77">
-        <f>C18</f>
-        <v/>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>sub-1Y dust only</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Optional — split 7Y out to kill the 7s10s residual</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="51" t="inlineStr">
-        <is>
-          <t>Hedge swap</t>
-        </is>
-      </c>
-      <c r="B25" s="51" t="inlineStr">
-        <is>
-          <t>Absorbs buckets</t>
-        </is>
-      </c>
-      <c r="C25" s="51" t="inlineStr">
-        <is>
-          <t>Group DV01 (KRW/bp)</t>
-        </is>
-      </c>
-      <c r="D25" s="51" t="inlineStr">
-        <is>
-          <t>Annuity</t>
-        </is>
-      </c>
-      <c r="E25" s="51" t="inlineStr">
-        <is>
-          <t>Notional (bn)</t>
-        </is>
-      </c>
-      <c r="F25" s="51" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>7Y</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>7Y + 8Y (part)</t>
-        </is>
-      </c>
-      <c r="C26" s="55">
-        <f>KRD!AC69+KRD!AD69</f>
-        <v/>
-      </c>
-      <c r="D26" s="75">
-        <f>$C$9</f>
-        <v/>
-      </c>
-      <c r="E26" s="76">
-        <f>ABS(C26/(D26*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="F26" s="2">
-        <f>IF(C26&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="B30" s="84">
+        <f>IF(E30&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C30" s="88">
+        <f>ABS(E30/(F30*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>10Y</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>9Y + 10Y (part)</t>
-        </is>
-      </c>
-      <c r="C27" s="55">
-        <f>KRD!AE69+KRD!AF69</f>
-        <v/>
-      </c>
-      <c r="D27" s="75">
-        <f>$C$10</f>
-        <v/>
-      </c>
-      <c r="E27" s="76">
-        <f>ABS(C27/(D27*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="F27" s="2">
-        <f>IF(C27&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>Replaces the single 10Y line above with these two; +1 bid/offer.</t>
+      <c r="E30" s="41">
+        <f>'KRD-v3'!$B$21</f>
+        <v/>
+      </c>
+      <c r="F30" s="86">
+        <f>$J$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>In the master, repoint the KRD-v3 refs to Sheet1 (1Y=B9, 2Y=B10, 3Y=B11, 4Y=B12, 5Y=B13, 7Y=B14, 10Y=B15).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire Hedge through Sheet1 (drop-in for master)
Add Sheet1 mirroring the master's folded Kevin-format table (values from
KRD-v3) and repoint all Hedge references from KRD-v3 to Sheet1, so the Hedge
blotter drops into the master (which already has Sheet1) with no repointing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hedge" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -281,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -377,6 +378,7 @@
     <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="26" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="28" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6698,6 +6700,237 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="89" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B1" s="89" t="inlineStr">
+        <is>
+          <t>dv01</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>'KRD-v3'!A8</f>
+        <v/>
+      </c>
+      <c r="B2" s="55">
+        <f>'KRD-v3'!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <f>'KRD-v3'!A9</f>
+        <v/>
+      </c>
+      <c r="B3" s="55">
+        <f>'KRD-v3'!B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <f>'KRD-v3'!A10</f>
+        <v/>
+      </c>
+      <c r="B4" s="55">
+        <f>'KRD-v3'!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <f>'KRD-v3'!A11</f>
+        <v/>
+      </c>
+      <c r="B5" s="55">
+        <f>'KRD-v3'!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f>'KRD-v3'!A12</f>
+        <v/>
+      </c>
+      <c r="B6" s="55">
+        <f>'KRD-v3'!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <f>'KRD-v3'!A13</f>
+        <v/>
+      </c>
+      <c r="B7" s="55">
+        <f>'KRD-v3'!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>'KRD-v3'!A14</f>
+        <v/>
+      </c>
+      <c r="B8" s="55">
+        <f>'KRD-v3'!B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>'KRD-v3'!A15</f>
+        <v/>
+      </c>
+      <c r="B9" s="55">
+        <f>'KRD-v3'!B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <f>'KRD-v3'!A16</f>
+        <v/>
+      </c>
+      <c r="B10" s="55">
+        <f>'KRD-v3'!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <f>'KRD-v3'!A17</f>
+        <v/>
+      </c>
+      <c r="B11" s="55">
+        <f>'KRD-v3'!B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <f>'KRD-v3'!A18</f>
+        <v/>
+      </c>
+      <c r="B12" s="55">
+        <f>'KRD-v3'!B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>'KRD-v3'!A19</f>
+        <v/>
+      </c>
+      <c r="B13" s="55">
+        <f>'KRD-v3'!B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>'KRD-v3'!A20</f>
+        <v/>
+      </c>
+      <c r="B14" s="55">
+        <f>'KRD-v3'!B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <f>'KRD-v3'!A21</f>
+        <v/>
+      </c>
+      <c r="B15" s="55">
+        <f>'KRD-v3'!B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <f>'KRD-v3'!A22</f>
+        <v/>
+      </c>
+      <c r="B16" s="55">
+        <f>'KRD-v3'!B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <f>'KRD-v3'!A23</f>
+        <v/>
+      </c>
+      <c r="B17" s="55">
+        <f>'KRD-v3'!B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <f>'KRD-v3'!A24</f>
+        <v/>
+      </c>
+      <c r="B18" s="55">
+        <f>'KRD-v3'!B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <f>'KRD-v3'!A25</f>
+        <v/>
+      </c>
+      <c r="B19" s="55">
+        <f>'KRD-v3'!B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <f>'KRD-v3'!A26</f>
+        <v/>
+      </c>
+      <c r="B20" s="55">
+        <f>'KRD-v3'!B26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="79" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B21" s="87">
+        <f>'KRD-v3'!B27</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -30239,7 +30472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -30267,6 +30500,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="30" t="inlineStr">
         <is>
@@ -30286,7 +30520,7 @@
         </is>
       </c>
       <c r="B5" s="80">
-        <f>'KRD-v3'!$B$27</f>
+        <f>Sheet1!$B$21</f>
         <v/>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -30302,7 +30536,7 @@
         </is>
       </c>
       <c r="B6" s="81">
-        <f>'KRD-v3'!$B$15+'KRD-v3'!$B$16+'KRD-v3'!$B$17</f>
+        <f>Sheet1!$B$9+Sheet1!$B$10+Sheet1!$B$11</f>
         <v/>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -30318,7 +30552,7 @@
         </is>
       </c>
       <c r="B7" s="82">
-        <f>'KRD-v3'!$B$18+'KRD-v3'!$B$19+'KRD-v3'!$B$20+'KRD-v3'!$B$21</f>
+        <f>Sheet1!$B$12+Sheet1!$B$13+Sheet1!$B$14+Sheet1!$B$15</f>
         <v/>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -30334,7 +30568,7 @@
         </is>
       </c>
       <c r="B8" s="74">
-        <f>'KRD-v3'!$B$12+'KRD-v3'!$B$13+'KRD-v3'!$B$14</f>
+        <f>Sheet1!$B$6+Sheet1!$B$7+Sheet1!$B$8</f>
         <v/>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -30343,6 +30577,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="30" t="inlineStr">
         <is>
@@ -30376,6 +30611,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="30" t="inlineStr">
         <is>
@@ -30460,7 +30696,7 @@
         </is>
       </c>
       <c r="E17" s="41">
-        <f>'KRD-v3'!$B$15+'KRD-v3'!$B$16</f>
+        <f>Sheet1!$B$9+Sheet1!$B$10</f>
         <v/>
       </c>
       <c r="F17" s="86">
@@ -30500,7 +30736,7 @@
         </is>
       </c>
       <c r="E18" s="41">
-        <f>'KRD-v3'!$B$17</f>
+        <f>Sheet1!$B$11</f>
         <v/>
       </c>
       <c r="F18" s="86">
@@ -30540,7 +30776,7 @@
         </is>
       </c>
       <c r="E19" s="41">
-        <f>'KRD-v3'!$B$18+'KRD-v3'!$B$19</f>
+        <f>Sheet1!$B$12+Sheet1!$B$13</f>
         <v/>
       </c>
       <c r="F19" s="86">
@@ -30580,7 +30816,7 @@
         </is>
       </c>
       <c r="E20" s="41">
-        <f>'KRD-v3'!$B$20+'KRD-v3'!$B$21</f>
+        <f>Sheet1!$B$14+Sheet1!$B$15</f>
         <v/>
       </c>
       <c r="F20" s="86">
@@ -30645,7 +30881,7 @@
         </is>
       </c>
       <c r="C24" s="87">
-        <f>'KRD-v3'!$B$12+'KRD-v3'!$B$13+'KRD-v3'!$B$14</f>
+        <f>Sheet1!$B$6+Sheet1!$B$7+Sheet1!$B$8</f>
         <v/>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -30666,6 +30902,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="30" t="inlineStr">
         <is>
@@ -30730,7 +30967,7 @@
         </is>
       </c>
       <c r="E29" s="41">
-        <f>'KRD-v3'!$B$20</f>
+        <f>Sheet1!$B$14</f>
         <v/>
       </c>
       <c r="F29" s="86">
@@ -30758,7 +30995,7 @@
         </is>
       </c>
       <c r="E30" s="41">
-        <f>'KRD-v3'!$B$21</f>
+        <f>Sheet1!$B$15</f>
         <v/>
       </c>
       <c r="F30" s="86">
@@ -30769,10 +31006,19 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>In the master, repoint the KRD-v3 refs to Sheet1 (1Y=B9, 2Y=B10, 3Y=B11, 4Y=B12, 5Y=B13, 7Y=B14, 10Y=B15).</t>
-        </is>
-      </c>
-    </row>
+          <t>Wired to Sheet1 (1Y=B9 … 10Y=B15). Drops into the master as-is; confirm Bootstrap!B3:B122/D3:D122 match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hedge: add live Cost-to-hedge block (BDP bid/offer)
Per benchmark: BDP bid/ask -> spread(bp) -> crossing cost
(= notional x annuity x half-spread) -> break-even move (cost/DV01) -> verdict.
References the blotter notionals/annuities/DV01. Computes on the terminal.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -27,7 +27,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="0.000%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.00000000"/>
@@ -37,6 +37,7 @@
     <numFmt numFmtId="170" formatCode="0.0000"/>
     <numFmt numFmtId="171" formatCode="0.00000"/>
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
+    <numFmt numFmtId="173" formatCode="0.0"/>
   </numFmts>
   <fonts count="30">
     <font>
@@ -282,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -379,6 +380,8 @@
     <xf numFmtId="3" fontId="26" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="28" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -30472,7 +30475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -30480,8 +30483,9 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="5" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
@@ -30500,7 +30504,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="30" t="inlineStr">
         <is>
@@ -30577,7 +30580,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="30" t="inlineStr">
         <is>
@@ -30611,7 +30613,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="30" t="inlineStr">
         <is>
@@ -30902,7 +30903,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="30" t="inlineStr">
         <is>
@@ -31010,15 +31010,231 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>6 · Cost to hedge  (live bid/offer — computes on the terminal)</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="n"/>
+      <c r="C33" s="31" t="n"/>
+      <c r="D33" s="31" t="n"/>
+      <c r="E33" s="31" t="n"/>
+      <c r="F33" s="31" t="n"/>
+      <c r="G33" s="31" t="n"/>
+      <c r="H33" s="31" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="50" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B34" s="50" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="C34" s="50" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="D34" s="50" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="E34" s="50" t="inlineStr">
+        <is>
+          <t>Spread (bp)</t>
+        </is>
+      </c>
+      <c r="F34" s="50" t="inlineStr">
+        <is>
+          <t>Cost (KRW)</t>
+        </is>
+      </c>
+      <c r="G34" s="50" t="inlineStr">
+        <is>
+          <t>Break-even (bp)</t>
+        </is>
+      </c>
+      <c r="H34" s="50" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="84" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>KWSW2 Curncy</t>
+        </is>
+      </c>
+      <c r="C35" s="9">
+        <f>BDP(B35,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D35" s="9">
+        <f>BDP(B35,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E35" s="90">
+        <f>(D35-C35)*100</f>
+        <v/>
+      </c>
+      <c r="F35" s="41">
+        <f>C17*1000000000*F17*(E35/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="G35" s="9">
+        <f>F35/ABS(E17)</f>
+        <v/>
+      </c>
+      <c r="H35" s="84">
+        <f>IF(G35&lt;1,"TRADE","review")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="84" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>KWSW3 Curncy</t>
+        </is>
+      </c>
+      <c r="C36" s="9">
+        <f>BDP(B36,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D36" s="9">
+        <f>BDP(B36,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E36" s="90">
+        <f>(D36-C36)*100</f>
+        <v/>
+      </c>
+      <c r="F36" s="41">
+        <f>C18*1000000000*F18*(E36/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="G36" s="9">
+        <f>F36/ABS(E18)</f>
+        <v/>
+      </c>
+      <c r="H36" s="84">
+        <f>IF(G36&lt;1,"TRADE","review")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="84" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>KWSW5 Curncy</t>
+        </is>
+      </c>
+      <c r="C37" s="9">
+        <f>BDP(B37,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D37" s="9">
+        <f>BDP(B37,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E37" s="90">
+        <f>(D37-C37)*100</f>
+        <v/>
+      </c>
+      <c r="F37" s="41">
+        <f>C19*1000000000*F19*(E37/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="G37" s="9">
+        <f>F37/ABS(E19)</f>
+        <v/>
+      </c>
+      <c r="H37" s="84">
+        <f>IF(G37&lt;1,"TRADE","review")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="84" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>KWSW10 Curncy</t>
+        </is>
+      </c>
+      <c r="C38" s="9">
+        <f>BDP(B38,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D38" s="9">
+        <f>BDP(B38,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E38" s="90">
+        <f>(D38-C38)*100</f>
+        <v/>
+      </c>
+      <c r="F38" s="41">
+        <f>C20*1000000000*F20*(E38/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="G38" s="9">
+        <f>F38/ABS(E20)</f>
+        <v/>
+      </c>
+      <c r="H38" s="84">
+        <f>IF(G38&lt;1,"TRADE","review")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="79" t="inlineStr">
+        <is>
+          <t>TOTAL cost</t>
+        </is>
+      </c>
+      <c r="F39" s="91">
+        <f>SUM(F35:F38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Break-even (bp) = cost / DV01: the adverse move that pays for the hedge. &lt;1bp -&gt; trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>For the 7Y split / sub-1Y dust, run the same row with KWSW7 / KWCDC — break-even blows out.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 'Hedge Cost Data Pull' sheet
Standalone bid/offer pull + cost calc for all six candidates (2Y/3Y/5Y/10Y
trades + 7Y split + sub-1Y dust). Self-contained: DV01 off Sheet1 buckets,
annuity via SUMIF on Bootstrap, notional solved inline, cost = notional x
annuity x half-spread, break-even = cost/DV01, verdict TRADE/SKIP. Skip
rationale annotated for the 7Y split and dust. BDP computes on the terminal.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -16,9 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD-v2" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD-v3" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hedge" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hedge Cost Data Pull" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +40,7 @@
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -208,6 +209,24 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -283,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -382,6 +401,17 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1003,6 +1033,455 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="92" t="inlineStr">
+        <is>
+          <t>Hedge Cost Data Pull</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Live bid/offer per tenor -&gt; crossing cost -&gt; break-even move. Self-contained: DV01 from Sheet1 buckets, annuity from the Bootstrap curve, notional solved inline. BDP computes on the terminal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="50" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B4" s="50" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C4" s="50" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="D4" s="50" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="E4" s="50" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="F4" s="50" t="inlineStr">
+        <is>
+          <t>Spread (bp)</t>
+        </is>
+      </c>
+      <c r="G4" s="50" t="inlineStr">
+        <is>
+          <t>Group DV01 (KRW/bp)</t>
+        </is>
+      </c>
+      <c r="H4" s="50" t="inlineStr">
+        <is>
+          <t>Annuity</t>
+        </is>
+      </c>
+      <c r="I4" s="50" t="inlineStr">
+        <is>
+          <t>Notional (bn)</t>
+        </is>
+      </c>
+      <c r="J4" s="50" t="inlineStr">
+        <is>
+          <t>Cost (KRW)</t>
+        </is>
+      </c>
+      <c r="K4" s="50" t="inlineStr">
+        <is>
+          <t>Break-even (bp)</t>
+        </is>
+      </c>
+      <c r="L4" s="50" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="84" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>KWSW2 Curncy</t>
+        </is>
+      </c>
+      <c r="D5" s="9">
+        <f>BDP(C5,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E5" s="9">
+        <f>BDP(C5,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F5" s="90">
+        <f>(E5-D5)*100</f>
+        <v/>
+      </c>
+      <c r="G5" s="41">
+        <f>Sheet1!B9+Sheet1!B10</f>
+        <v/>
+      </c>
+      <c r="H5" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B5,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I5" s="93">
+        <f>ABS(G5/(H5*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J5" s="41">
+        <f>I5*1000000000*H5*(F5/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K5" s="9">
+        <f>J5/ABS(G5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="94">
+        <f>IF(K5&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="84" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>KWSW3 Curncy</t>
+        </is>
+      </c>
+      <c r="D6" s="9">
+        <f>BDP(C6,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E6" s="9">
+        <f>BDP(C6,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F6" s="90">
+        <f>(E6-D6)*100</f>
+        <v/>
+      </c>
+      <c r="G6" s="41">
+        <f>Sheet1!B11</f>
+        <v/>
+      </c>
+      <c r="H6" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B6,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I6" s="93">
+        <f>ABS(G6/(H6*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J6" s="41">
+        <f>I6*1000000000*H6*(F6/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K6" s="9">
+        <f>J6/ABS(G6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="94">
+        <f>IF(K6&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="84" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>KWSW5 Curncy</t>
+        </is>
+      </c>
+      <c r="D7" s="9">
+        <f>BDP(C7,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E7" s="9">
+        <f>BDP(C7,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F7" s="90">
+        <f>(E7-D7)*100</f>
+        <v/>
+      </c>
+      <c r="G7" s="41">
+        <f>Sheet1!B12+Sheet1!B13</f>
+        <v/>
+      </c>
+      <c r="H7" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B7,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I7" s="93">
+        <f>ABS(G7/(H7*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J7" s="41">
+        <f>I7*1000000000*H7*(F7/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K7" s="9">
+        <f>J7/ABS(G7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="94">
+        <f>IF(K7&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="84" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>KWSW10 Curncy</t>
+        </is>
+      </c>
+      <c r="D8" s="9">
+        <f>BDP(C8,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E8" s="9">
+        <f>BDP(C8,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F8" s="90">
+        <f>(E8-D8)*100</f>
+        <v/>
+      </c>
+      <c r="G8" s="41">
+        <f>Sheet1!B14+Sheet1!B15</f>
+        <v/>
+      </c>
+      <c r="H8" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B8,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I8" s="93">
+        <f>ABS(G8/(H8*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J8" s="41">
+        <f>I8*1000000000*H8*(F8/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K8" s="9">
+        <f>J8/ABS(G8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="94">
+        <f>IF(K8&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="95" t="inlineStr">
+        <is>
+          <t>7Y split</t>
+        </is>
+      </c>
+      <c r="B9" s="96" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="96" t="inlineStr">
+        <is>
+          <t>KWSW7 Curncy</t>
+        </is>
+      </c>
+      <c r="D9" s="97">
+        <f>BDP(C9,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E9" s="97">
+        <f>BDP(C9,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F9" s="98">
+        <f>(E9-D9)*100</f>
+        <v/>
+      </c>
+      <c r="G9" s="99">
+        <f>Sheet1!B14</f>
+        <v/>
+      </c>
+      <c r="H9" s="100">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B9,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I9" s="101">
+        <f>ABS(G9/(H9*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J9" s="99">
+        <f>I9*1000000000*H9*(F9/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K9" s="97">
+        <f>J9/ABS(G9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="102">
+        <f>IF(K9&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="95" t="inlineStr">
+        <is>
+          <t>Dust 3-9M</t>
+        </is>
+      </c>
+      <c r="B10" s="96" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="96" t="inlineStr">
+        <is>
+          <t>KWCDC Curncy</t>
+        </is>
+      </c>
+      <c r="D10" s="97">
+        <f>BDP(C10,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E10" s="97">
+        <f>BDP(C10,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F10" s="98">
+        <f>(E10-D10)*100</f>
+        <v/>
+      </c>
+      <c r="G10" s="99">
+        <f>Sheet1!B6+Sheet1!B7+Sheet1!B8</f>
+        <v/>
+      </c>
+      <c r="H10" s="100">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B10,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I10" s="101">
+        <f>ABS(G10/(H10*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J10" s="99">
+        <f>I10*1000000000*H10*(F10/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K10" s="97">
+        <f>J10/ABS(G10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="102">
+        <f>IF(K10&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="79" t="inlineStr">
+        <is>
+          <t>TOTAL cost (4 trades)</t>
+        </is>
+      </c>
+      <c r="J11" s="91">
+        <f>SUM(J5:J8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Break-even (bp) = cost / DV01 ≈ half the bid/offer: the adverse move that pays for the hedge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>7Y split: most 7Y risk is already absorbed by the 10Y hedge, so the marginal risk removed is small vs a full bid/offer — skip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Dust: ~10k/bp total and below a sensible minimum ticket — operationally not worth a trade regardless of break-even.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Confirm each ticker with &lt;ticker&gt; DES / ALLQ before relying on the pull.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5743,7 +6222,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6703,7 +7182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Hedge Cost Analysis: real KWSWNI tickers + liquidity (per BBG Help Desk)
Rebuild the cost sheet with the correct offshore KRW IRS root (KWSWNI<n>
BGN Curncy, confirm on GC S205 > Table), editable ticker cells, live
bid/ask, 1-month avg spread via BDH, crossing cost, break-even, and a
manual SDRV volume column as the liquidity cross-check. DV01 off KRD-v3,
annuity via SUMIF on Bootstrap. Commands block documents GC S205 / SDRV / SDR.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -40,7 +40,7 @@
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="35">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -227,6 +227,15 @@
       <color rgb="009C0006"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -302,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -412,6 +421,10 @@
     <xf numFmtId="170" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="32" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1033,441 +1046,593 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="92" t="inlineStr">
         <is>
-          <t>Hedge Cost Data Pull</t>
+          <t>Hedge Cost Analysis — offshore KRW IRS (vs 91D CD)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Live bid/offer per tenor -&gt; crossing cost -&gt; break-even move. Self-contained: DV01 from Sheet1 buckets, annuity from the Bootstrap curve, notional solved inline. BDP computes on the terminal.</t>
+          <t>Tickers per Bloomberg Help Desk: root KWSWNI&lt;n&gt; BGN Curncy, confirm each on GC S205 &lt;GO&gt; &gt; Table. Bid/offer -&gt; crossing cost -&gt; break-even; volume from SDRV is the liquidity check.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>Bloomberg commands</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="n"/>
+      <c r="C4" s="31" t="n"/>
+      <c r="D4" s="31" t="n"/>
+      <c r="E4" s="31" t="n"/>
+      <c r="F4" s="31" t="n"/>
+      <c r="G4" s="31" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="79" t="inlineStr">
+        <is>
+          <t>Tickers / curve</t>
+        </is>
+      </c>
+      <c r="B5" s="103" t="inlineStr">
+        <is>
+          <t>GC S205 &lt;GO&gt;  &gt;  click Table  (offshore KRW vs 91D CD, members per tenor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>Bid / Ask (Excel)</t>
+        </is>
+      </c>
+      <c r="B6" s="103">
+        <f>BDP("KWSWNI5 BGN Curncy","PX_ASK")   /   "PX_BID"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="79" t="inlineStr">
+        <is>
+          <t>1-month history</t>
+        </is>
+      </c>
+      <c r="B7" s="103">
+        <f>BDH("KWSWNI5 BGN Curncy","PX_ASK","20260624","20260724")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="79" t="inlineStr">
+        <is>
+          <t>Liquidity / volume</t>
+        </is>
+      </c>
+      <c r="B8" s="103" t="inlineStr">
+        <is>
+          <t>SDRV &lt;GO&gt; &gt; Rates tab &gt; IRS/FRA view &gt; Currency=KRW &gt; volume &amp; trade count by tenor (USDmm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="79" t="inlineStr">
+        <is>
+          <t>Drill to trades</t>
+        </is>
+      </c>
+      <c r="B9" s="103" t="inlineStr">
+        <is>
+          <t>click a tenor &gt; SDR &lt;GO&gt; for the individual trades behind the total</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Cost + liquidity by tenor</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="n"/>
+      <c r="C11" s="31" t="n"/>
+      <c r="D11" s="31" t="n"/>
+      <c r="E11" s="31" t="n"/>
+      <c r="F11" s="31" t="n"/>
+      <c r="G11" s="31" t="n"/>
+      <c r="H11" s="31" t="n"/>
+      <c r="I11" s="31" t="n"/>
+      <c r="J11" s="31" t="n"/>
+      <c r="K11" s="31" t="n"/>
+      <c r="L11" s="31" t="n"/>
+      <c r="M11" s="31" t="n"/>
+      <c r="N11" s="31" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="50" t="inlineStr">
         <is>
           <t>Tenor</t>
         </is>
       </c>
-      <c r="B4" s="50" t="inlineStr">
+      <c r="B12" s="50" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="C4" s="50" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="D4" s="50" t="inlineStr">
+      <c r="C12" s="50" t="inlineStr">
+        <is>
+          <t>Ticker (edit)</t>
+        </is>
+      </c>
+      <c r="D12" s="50" t="inlineStr">
         <is>
           <t>Bid</t>
         </is>
       </c>
-      <c r="E4" s="50" t="inlineStr">
+      <c r="E12" s="50" t="inlineStr">
         <is>
           <t>Ask</t>
         </is>
       </c>
-      <c r="F4" s="50" t="inlineStr">
+      <c r="F12" s="50" t="inlineStr">
         <is>
           <t>Spread (bp)</t>
         </is>
       </c>
-      <c r="G4" s="50" t="inlineStr">
+      <c r="G12" s="50" t="inlineStr">
+        <is>
+          <t>Avg spr 1M (bp)</t>
+        </is>
+      </c>
+      <c r="H12" s="50" t="inlineStr">
         <is>
           <t>Group DV01 (KRW/bp)</t>
         </is>
       </c>
-      <c r="H4" s="50" t="inlineStr">
+      <c r="I12" s="50" t="inlineStr">
         <is>
           <t>Annuity</t>
         </is>
       </c>
-      <c r="I4" s="50" t="inlineStr">
+      <c r="J12" s="50" t="inlineStr">
         <is>
           <t>Notional (bn)</t>
         </is>
       </c>
-      <c r="J4" s="50" t="inlineStr">
+      <c r="K12" s="50" t="inlineStr">
         <is>
           <t>Cost (KRW)</t>
         </is>
       </c>
-      <c r="K4" s="50" t="inlineStr">
+      <c r="L12" s="50" t="inlineStr">
         <is>
           <t>Break-even (bp)</t>
         </is>
       </c>
-      <c r="L4" s="50" t="inlineStr">
+      <c r="M12" s="50" t="inlineStr">
+        <is>
+          <t>Vol USDmm (SDRV)</t>
+        </is>
+      </c>
+      <c r="N12" s="50" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="84" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="84" t="inlineStr">
         <is>
           <t>2Y</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>KWSW2 Curncy</t>
-        </is>
-      </c>
-      <c r="D5" s="9">
-        <f>BDP(C5,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E5" s="9">
-        <f>BDP(C5,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F5" s="90">
-        <f>(E5-D5)*100</f>
-        <v/>
-      </c>
-      <c r="G5" s="41">
-        <f>Sheet1!B9+Sheet1!B10</f>
-        <v/>
-      </c>
-      <c r="H5" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B5,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I5" s="93">
-        <f>ABS(G5/(H5*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J5" s="41">
-        <f>I5*1000000000*H5*(F5/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="K5" s="9">
-        <f>J5/ABS(G5)</f>
-        <v/>
-      </c>
-      <c r="L5" s="94">
-        <f>IF(K5&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="84" t="inlineStr">
+      <c r="C13" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI2 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="D13" s="9">
+        <f>BDP(C13,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E13" s="9">
+        <f>BDP(C13,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F13" s="6">
+        <f>(E13-D13)*100</f>
+        <v/>
+      </c>
+      <c r="G13" s="6">
+        <f>(AVERAGE(BDH(C13,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C13,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="H13" s="41">
+        <f>'KRD-v3'!B15+'KRD-v3'!B16</f>
+        <v/>
+      </c>
+      <c r="I13" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B13,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="J13" s="93">
+        <f>ABS(H13/(I13*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="K13" s="41">
+        <f>J13*1000000000*I13*(F13/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>K13/ABS(H13)</f>
+        <v/>
+      </c>
+      <c r="M13" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="94">
+        <f>IF(L13&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="84" t="inlineStr">
         <is>
           <t>3Y</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>KWSW3 Curncy</t>
-        </is>
-      </c>
-      <c r="D6" s="9">
-        <f>BDP(C6,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E6" s="9">
-        <f>BDP(C6,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F6" s="90">
-        <f>(E6-D6)*100</f>
-        <v/>
-      </c>
-      <c r="G6" s="41">
-        <f>Sheet1!B11</f>
-        <v/>
-      </c>
-      <c r="H6" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B6,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I6" s="93">
-        <f>ABS(G6/(H6*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J6" s="41">
-        <f>I6*1000000000*H6*(F6/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="K6" s="9">
-        <f>J6/ABS(G6)</f>
-        <v/>
-      </c>
-      <c r="L6" s="94">
-        <f>IF(K6&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="84" t="inlineStr">
+      <c r="C14" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI3 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="D14" s="9">
+        <f>BDP(C14,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E14" s="9">
+        <f>BDP(C14,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F14" s="6">
+        <f>(E14-D14)*100</f>
+        <v/>
+      </c>
+      <c r="G14" s="6">
+        <f>(AVERAGE(BDH(C14,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C14,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="H14" s="41">
+        <f>'KRD-v3'!B17</f>
+        <v/>
+      </c>
+      <c r="I14" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B14,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="J14" s="93">
+        <f>ABS(H14/(I14*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="K14" s="41">
+        <f>J14*1000000000*I14*(F14/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="L14" s="6">
+        <f>K14/ABS(H14)</f>
+        <v/>
+      </c>
+      <c r="M14" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="94">
+        <f>IF(L14&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="84" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B15" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>KWSW5 Curncy</t>
-        </is>
-      </c>
-      <c r="D7" s="9">
-        <f>BDP(C7,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E7" s="9">
-        <f>BDP(C7,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F7" s="90">
-        <f>(E7-D7)*100</f>
-        <v/>
-      </c>
-      <c r="G7" s="41">
-        <f>Sheet1!B12+Sheet1!B13</f>
-        <v/>
-      </c>
-      <c r="H7" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B7,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I7" s="93">
-        <f>ABS(G7/(H7*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J7" s="41">
-        <f>I7*1000000000*H7*(F7/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="K7" s="9">
-        <f>J7/ABS(G7)</f>
-        <v/>
-      </c>
-      <c r="L7" s="94">
-        <f>IF(K7&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="84" t="inlineStr">
+      <c r="C15" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI5 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="D15" s="9">
+        <f>BDP(C15,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E15" s="9">
+        <f>BDP(C15,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F15" s="6">
+        <f>(E15-D15)*100</f>
+        <v/>
+      </c>
+      <c r="G15" s="6">
+        <f>(AVERAGE(BDH(C15,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C15,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="H15" s="41">
+        <f>'KRD-v3'!B18+'KRD-v3'!B19</f>
+        <v/>
+      </c>
+      <c r="I15" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B15,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="J15" s="93">
+        <f>ABS(H15/(I15*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="K15" s="41">
+        <f>J15*1000000000*I15*(F15/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="L15" s="6">
+        <f>K15/ABS(H15)</f>
+        <v/>
+      </c>
+      <c r="M15" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="94">
+        <f>IF(L15&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="84" t="inlineStr">
         <is>
           <t>10Y</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B16" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>KWSW10 Curncy</t>
-        </is>
-      </c>
-      <c r="D8" s="9">
-        <f>BDP(C8,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E8" s="9">
-        <f>BDP(C8,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F8" s="90">
-        <f>(E8-D8)*100</f>
-        <v/>
-      </c>
-      <c r="G8" s="41">
-        <f>Sheet1!B14+Sheet1!B15</f>
-        <v/>
-      </c>
-      <c r="H8" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B8,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I8" s="93">
-        <f>ABS(G8/(H8*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J8" s="41">
-        <f>I8*1000000000*H8*(F8/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="K8" s="9">
-        <f>J8/ABS(G8)</f>
-        <v/>
-      </c>
-      <c r="L8" s="94">
-        <f>IF(K8&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="95" t="inlineStr">
+      <c r="C16" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI10 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="D16" s="9">
+        <f>BDP(C16,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E16" s="9">
+        <f>BDP(C16,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>(E16-D16)*100</f>
+        <v/>
+      </c>
+      <c r="G16" s="6">
+        <f>(AVERAGE(BDH(C16,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C16,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="H16" s="41">
+        <f>'KRD-v3'!B20+'KRD-v3'!B21</f>
+        <v/>
+      </c>
+      <c r="I16" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B16,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="J16" s="93">
+        <f>ABS(H16/(I16*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="K16" s="41">
+        <f>J16*1000000000*I16*(F16/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="L16" s="6">
+        <f>K16/ABS(H16)</f>
+        <v/>
+      </c>
+      <c r="M16" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="94">
+        <f>IF(L16&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="95" t="inlineStr">
         <is>
           <t>7Y split</t>
         </is>
       </c>
-      <c r="B9" s="96" t="n">
+      <c r="B17" s="96" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="96" t="inlineStr">
-        <is>
-          <t>KWSW7 Curncy</t>
-        </is>
-      </c>
-      <c r="D9" s="97">
-        <f>BDP(C9,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E9" s="97">
-        <f>BDP(C9,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F9" s="98">
-        <f>(E9-D9)*100</f>
-        <v/>
-      </c>
-      <c r="G9" s="99">
-        <f>Sheet1!B14</f>
-        <v/>
-      </c>
-      <c r="H9" s="100">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B9,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I9" s="101">
-        <f>ABS(G9/(H9*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J9" s="99">
-        <f>I9*1000000000*H9*(F9/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="K9" s="97">
-        <f>J9/ABS(G9)</f>
-        <v/>
-      </c>
-      <c r="L9" s="102">
-        <f>IF(K9&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="95" t="inlineStr">
+      <c r="C17" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI7 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="D17" s="97">
+        <f>BDP(C17,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E17" s="97">
+        <f>BDP(C17,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F17" s="105">
+        <f>(E17-D17)*100</f>
+        <v/>
+      </c>
+      <c r="G17" s="105">
+        <f>(AVERAGE(BDH(C17,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C17,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="H17" s="99">
+        <f>'KRD-v3'!B20</f>
+        <v/>
+      </c>
+      <c r="I17" s="100">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B17,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="J17" s="101">
+        <f>ABS(H17/(I17*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="K17" s="99">
+        <f>J17*1000000000*I17*(F17/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="L17" s="105">
+        <f>K17/ABS(H17)</f>
+        <v/>
+      </c>
+      <c r="M17" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="102">
+        <f>IF(L17&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="95" t="inlineStr">
         <is>
           <t>Dust 3-9M</t>
         </is>
       </c>
-      <c r="B10" s="96" t="n">
+      <c r="B18" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="96" t="inlineStr">
-        <is>
-          <t>KWCDC Curncy</t>
-        </is>
-      </c>
-      <c r="D10" s="97">
-        <f>BDP(C10,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E10" s="97">
-        <f>BDP(C10,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F10" s="98">
-        <f>(E10-D10)*100</f>
-        <v/>
-      </c>
-      <c r="G10" s="99">
-        <f>Sheet1!B6+Sheet1!B7+Sheet1!B8</f>
-        <v/>
-      </c>
-      <c r="H10" s="100">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B10,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I10" s="101">
-        <f>ABS(G10/(H10*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J10" s="99">
-        <f>I10*1000000000*H10*(F10/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="K10" s="97">
-        <f>J10/ABS(G10)</f>
-        <v/>
-      </c>
-      <c r="L10" s="102">
-        <f>IF(K10&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="79" t="inlineStr">
+      <c r="C18" s="104" t="inlineStr">
+        <is>
+          <t>(front = CD/FRA, see GC S205)</t>
+        </is>
+      </c>
+      <c r="D18" s="97">
+        <f>BDP(C18,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="E18" s="97">
+        <f>BDP(C18,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="F18" s="105">
+        <f>(E18-D18)*100</f>
+        <v/>
+      </c>
+      <c r="G18" s="105">
+        <f>(AVERAGE(BDH(C18,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C18,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="H18" s="99">
+        <f>'KRD-v3'!B12+'KRD-v3'!B13+'KRD-v3'!B14</f>
+        <v/>
+      </c>
+      <c r="I18" s="100">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B18,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="J18" s="101">
+        <f>ABS(H18/(I18*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="K18" s="99">
+        <f>J18*1000000000*I18*(F18/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="L18" s="105">
+        <f>K18/ABS(H18)</f>
+        <v/>
+      </c>
+      <c r="M18" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="102">
+        <f>IF(L18&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="79" t="inlineStr">
         <is>
           <t>TOTAL cost (4 trades)</t>
         </is>
       </c>
-      <c r="J11" s="91">
-        <f>SUM(J5:J8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Break-even (bp) = cost / DV01 ≈ half the bid/offer: the adverse move that pays for the hedge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>7Y split: most 7Y risk is already absorbed by the 10Y hedge, so the marginal risk removed is small vs a full bid/offer — skip.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Dust: ~10k/bp total and below a sensible minimum ticket — operationally not worth a trade regardless of break-even.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Confirm each ticker with &lt;ticker&gt; DES / ALLQ before relying on the pull.</t>
+      <c r="K19" s="91">
+        <f>SUM(K13:K16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Yellow = inputs: paste the exact ticker from GC S205 &gt; Table, and the SDRV volume (USDmm) per tenor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Break-even (bp) = cost / DV01 ≈ half the bid/offer: the adverse move that pays for the hedge. &lt;1bp -&gt; trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Cross-check with SDRV volume: tight break-even AND high volume = liquid, trade. Wide + thin = skip (7Y).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>7Y split: 10Y already absorbs most 7Y; marginal risk removed &lt; a full bid/offer. Dust: below min ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>DV01 pulled from KRD-v3 (folded buckets); annuity via SUMIF on Bootstrap. BDP/BDH compute on the terminal.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hedge: move cost & liquidity analysis inline, right under the trades
Rebuild Hedge in order: risk, strategy, trades, cost & liquidity, residual,
optional. Cost rows pull each line's DV01 straight from the blotter above,
add KWSWNI bid/ask + 1M avg spread + crossing cost + break-even + SDRV
volume + verdict. Delete the standalone 'Hedge Cost Data Pull' sheet;
commands (GC S205 / SDRV / SDR) noted inline.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -16,10 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD-v2" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD-v3" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hedge" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hedge Cost Data Pull" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -311,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -425,6 +424,11 @@
     <xf numFmtId="0" fontId="34" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="34" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="32" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="31" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="31" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1046,607 +1050,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="92" t="inlineStr">
-        <is>
-          <t>Hedge Cost Analysis — offshore KRW IRS (vs 91D CD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Tickers per Bloomberg Help Desk: root KWSWNI&lt;n&gt; BGN Curncy, confirm each on GC S205 &lt;GO&gt; &gt; Table. Bid/offer -&gt; crossing cost -&gt; break-even; volume from SDRV is the liquidity check.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="30" t="inlineStr">
-        <is>
-          <t>Bloomberg commands</t>
-        </is>
-      </c>
-      <c r="B4" s="31" t="n"/>
-      <c r="C4" s="31" t="n"/>
-      <c r="D4" s="31" t="n"/>
-      <c r="E4" s="31" t="n"/>
-      <c r="F4" s="31" t="n"/>
-      <c r="G4" s="31" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="79" t="inlineStr">
-        <is>
-          <t>Tickers / curve</t>
-        </is>
-      </c>
-      <c r="B5" s="103" t="inlineStr">
-        <is>
-          <t>GC S205 &lt;GO&gt;  &gt;  click Table  (offshore KRW vs 91D CD, members per tenor)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="79" t="inlineStr">
-        <is>
-          <t>Bid / Ask (Excel)</t>
-        </is>
-      </c>
-      <c r="B6" s="103">
-        <f>BDP("KWSWNI5 BGN Curncy","PX_ASK")   /   "PX_BID"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="79" t="inlineStr">
-        <is>
-          <t>1-month history</t>
-        </is>
-      </c>
-      <c r="B7" s="103">
-        <f>BDH("KWSWNI5 BGN Curncy","PX_ASK","20260624","20260724")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="79" t="inlineStr">
-        <is>
-          <t>Liquidity / volume</t>
-        </is>
-      </c>
-      <c r="B8" s="103" t="inlineStr">
-        <is>
-          <t>SDRV &lt;GO&gt; &gt; Rates tab &gt; IRS/FRA view &gt; Currency=KRW &gt; volume &amp; trade count by tenor (USDmm)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="79" t="inlineStr">
-        <is>
-          <t>Drill to trades</t>
-        </is>
-      </c>
-      <c r="B9" s="103" t="inlineStr">
-        <is>
-          <t>click a tenor &gt; SDR &lt;GO&gt; for the individual trades behind the total</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>Cost + liquidity by tenor</t>
-        </is>
-      </c>
-      <c r="B11" s="31" t="n"/>
-      <c r="C11" s="31" t="n"/>
-      <c r="D11" s="31" t="n"/>
-      <c r="E11" s="31" t="n"/>
-      <c r="F11" s="31" t="n"/>
-      <c r="G11" s="31" t="n"/>
-      <c r="H11" s="31" t="n"/>
-      <c r="I11" s="31" t="n"/>
-      <c r="J11" s="31" t="n"/>
-      <c r="K11" s="31" t="n"/>
-      <c r="L11" s="31" t="n"/>
-      <c r="M11" s="31" t="n"/>
-      <c r="N11" s="31" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="50" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B12" s="50" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="C12" s="50" t="inlineStr">
-        <is>
-          <t>Ticker (edit)</t>
-        </is>
-      </c>
-      <c r="D12" s="50" t="inlineStr">
-        <is>
-          <t>Bid</t>
-        </is>
-      </c>
-      <c r="E12" s="50" t="inlineStr">
-        <is>
-          <t>Ask</t>
-        </is>
-      </c>
-      <c r="F12" s="50" t="inlineStr">
-        <is>
-          <t>Spread (bp)</t>
-        </is>
-      </c>
-      <c r="G12" s="50" t="inlineStr">
-        <is>
-          <t>Avg spr 1M (bp)</t>
-        </is>
-      </c>
-      <c r="H12" s="50" t="inlineStr">
-        <is>
-          <t>Group DV01 (KRW/bp)</t>
-        </is>
-      </c>
-      <c r="I12" s="50" t="inlineStr">
-        <is>
-          <t>Annuity</t>
-        </is>
-      </c>
-      <c r="J12" s="50" t="inlineStr">
-        <is>
-          <t>Notional (bn)</t>
-        </is>
-      </c>
-      <c r="K12" s="50" t="inlineStr">
-        <is>
-          <t>Cost (KRW)</t>
-        </is>
-      </c>
-      <c r="L12" s="50" t="inlineStr">
-        <is>
-          <t>Break-even (bp)</t>
-        </is>
-      </c>
-      <c r="M12" s="50" t="inlineStr">
-        <is>
-          <t>Vol USDmm (SDRV)</t>
-        </is>
-      </c>
-      <c r="N12" s="50" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="84" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C13" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI2 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="D13" s="9">
-        <f>BDP(C13,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E13" s="9">
-        <f>BDP(C13,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F13" s="6">
-        <f>(E13-D13)*100</f>
-        <v/>
-      </c>
-      <c r="G13" s="6">
-        <f>(AVERAGE(BDH(C13,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C13,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
-        <v/>
-      </c>
-      <c r="H13" s="41">
-        <f>'KRD-v3'!B15+'KRD-v3'!B16</f>
-        <v/>
-      </c>
-      <c r="I13" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B13,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="J13" s="93">
-        <f>ABS(H13/(I13*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="K13" s="41">
-        <f>J13*1000000000*I13*(F13/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="L13" s="6">
-        <f>K13/ABS(H13)</f>
-        <v/>
-      </c>
-      <c r="M13" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="94">
-        <f>IF(L13&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="84" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI3 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="D14" s="9">
-        <f>BDP(C14,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E14" s="9">
-        <f>BDP(C14,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F14" s="6">
-        <f>(E14-D14)*100</f>
-        <v/>
-      </c>
-      <c r="G14" s="6">
-        <f>(AVERAGE(BDH(C14,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C14,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
-        <v/>
-      </c>
-      <c r="H14" s="41">
-        <f>'KRD-v3'!B17</f>
-        <v/>
-      </c>
-      <c r="I14" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B14,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="J14" s="93">
-        <f>ABS(H14/(I14*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="K14" s="41">
-        <f>J14*1000000000*I14*(F14/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="L14" s="6">
-        <f>K14/ABS(H14)</f>
-        <v/>
-      </c>
-      <c r="M14" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="94">
-        <f>IF(L14&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="84" t="inlineStr">
-        <is>
-          <t>5Y</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C15" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI5 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="D15" s="9">
-        <f>BDP(C15,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E15" s="9">
-        <f>BDP(C15,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F15" s="6">
-        <f>(E15-D15)*100</f>
-        <v/>
-      </c>
-      <c r="G15" s="6">
-        <f>(AVERAGE(BDH(C15,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C15,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
-        <v/>
-      </c>
-      <c r="H15" s="41">
-        <f>'KRD-v3'!B18+'KRD-v3'!B19</f>
-        <v/>
-      </c>
-      <c r="I15" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B15,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="J15" s="93">
-        <f>ABS(H15/(I15*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="K15" s="41">
-        <f>J15*1000000000*I15*(F15/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="L15" s="6">
-        <f>K15/ABS(H15)</f>
-        <v/>
-      </c>
-      <c r="M15" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="94">
-        <f>IF(L15&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="84" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="C16" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI10 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="D16" s="9">
-        <f>BDP(C16,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E16" s="9">
-        <f>BDP(C16,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F16" s="6">
-        <f>(E16-D16)*100</f>
-        <v/>
-      </c>
-      <c r="G16" s="6">
-        <f>(AVERAGE(BDH(C16,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C16,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
-        <v/>
-      </c>
-      <c r="H16" s="41">
-        <f>'KRD-v3'!B20+'KRD-v3'!B21</f>
-        <v/>
-      </c>
-      <c r="I16" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B16,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="J16" s="93">
-        <f>ABS(H16/(I16*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="K16" s="41">
-        <f>J16*1000000000*I16*(F16/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="L16" s="6">
-        <f>K16/ABS(H16)</f>
-        <v/>
-      </c>
-      <c r="M16" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="94">
-        <f>IF(L16&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="95" t="inlineStr">
-        <is>
-          <t>7Y split</t>
-        </is>
-      </c>
-      <c r="B17" s="96" t="n">
-        <v>7</v>
-      </c>
-      <c r="C17" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI7 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="D17" s="97">
-        <f>BDP(C17,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E17" s="97">
-        <f>BDP(C17,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F17" s="105">
-        <f>(E17-D17)*100</f>
-        <v/>
-      </c>
-      <c r="G17" s="105">
-        <f>(AVERAGE(BDH(C17,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C17,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
-        <v/>
-      </c>
-      <c r="H17" s="99">
-        <f>'KRD-v3'!B20</f>
-        <v/>
-      </c>
-      <c r="I17" s="100">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B17,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="J17" s="101">
-        <f>ABS(H17/(I17*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="K17" s="99">
-        <f>J17*1000000000*I17*(F17/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="L17" s="105">
-        <f>K17/ABS(H17)</f>
-        <v/>
-      </c>
-      <c r="M17" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="102">
-        <f>IF(L17&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="95" t="inlineStr">
-        <is>
-          <t>Dust 3-9M</t>
-        </is>
-      </c>
-      <c r="B18" s="96" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" s="104" t="inlineStr">
-        <is>
-          <t>(front = CD/FRA, see GC S205)</t>
-        </is>
-      </c>
-      <c r="D18" s="97">
-        <f>BDP(C18,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="E18" s="97">
-        <f>BDP(C18,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="F18" s="105">
-        <f>(E18-D18)*100</f>
-        <v/>
-      </c>
-      <c r="G18" s="105">
-        <f>(AVERAGE(BDH(C18,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(C18,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
-        <v/>
-      </c>
-      <c r="H18" s="99">
-        <f>'KRD-v3'!B12+'KRD-v3'!B13+'KRD-v3'!B14</f>
-        <v/>
-      </c>
-      <c r="I18" s="100">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;B18,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="J18" s="101">
-        <f>ABS(H18/(I18*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="K18" s="99">
-        <f>J18*1000000000*I18*(F18/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="L18" s="105">
-        <f>K18/ABS(H18)</f>
-        <v/>
-      </c>
-      <c r="M18" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="102">
-        <f>IF(L18&lt;1,"TRADE","SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="79" t="inlineStr">
-        <is>
-          <t>TOTAL cost (4 trades)</t>
-        </is>
-      </c>
-      <c r="K19" s="91">
-        <f>SUM(K13:K16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Yellow = inputs: paste the exact ticker from GC S205 &gt; Table, and the SDRV volume (USDmm) per tenor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Break-even (bp) = cost / DV01 ≈ half the bid/offer: the adverse move that pays for the hedge. &lt;1bp -&gt; trade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Cross-check with SDRV volume: tight break-even AND high volume = liquid, trade. Wide + thin = skip (7Y).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>7Y split: 10Y already absorbs most 7Y; marginal risk removed &lt; a full bid/offer. Dust: below min ticket.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>DV01 pulled from KRD-v3 (folded buckets); annuity via SUMIF on Bootstrap. BDP/BDH compute on the terminal.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6387,7 +5790,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7347,7 +6750,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -31119,19 +30522,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -31144,7 +30551,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Bucketed KRD (Sheet1) hedged at liquid benchmarks. Notional(T) = group DV01 / (annuity(T) x 1bp), sized live off the curve; direction from the bucket sign.</t>
+          <t>Bucketed KRD hedged at liquid benchmarks; cost analysis (live bid/offer + SDRV volume) sits under the trades.</t>
         </is>
       </c>
     </row>
@@ -31159,6 +30566,15 @@
       <c r="D4" s="31" t="n"/>
       <c r="E4" s="31" t="n"/>
       <c r="F4" s="31" t="n"/>
+      <c r="G4" s="31" t="n"/>
+      <c r="H4" s="31" t="n"/>
+      <c r="I4" s="31" t="n"/>
+      <c r="J4" s="31" t="n"/>
+      <c r="L4" s="79" t="inlineStr">
+        <is>
+          <t>Benchmark annuity</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="79" t="inlineStr">
@@ -31166,13 +30582,28 @@
           <t>Net DV01</t>
         </is>
       </c>
-      <c r="B5" s="80">
+      <c r="B5" s="107">
         <f>Sheet1!$B$21</f>
         <v/>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
           <t>KRW per bp — net receiver</t>
+        </is>
+      </c>
+      <c r="L5" s="51" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="M5" s="51" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="N5" s="51" t="inlineStr">
+        <is>
+          <t>Annuity</t>
         </is>
       </c>
     </row>
@@ -31182,14 +30613,26 @@
           <t>Front 1Y–3Y</t>
         </is>
       </c>
-      <c r="B6" s="81">
+      <c r="B6" s="108">
         <f>Sheet1!$B$9+Sheet1!$B$10+Sheet1!$B$11</f>
         <v/>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>long (positive) — pays if rates rise</t>
-        </is>
+          <t>long (positive)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M6,Bootstrap!$D$3:$D$122)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -31198,14 +30641,26 @@
           <t>Back 4Y–10Y</t>
         </is>
       </c>
-      <c r="B7" s="82">
+      <c r="B7" s="109">
         <f>Sheet1!$B$12+Sheet1!$B$13+Sheet1!$B$14+Sheet1!$B$15</f>
         <v/>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>short (negative) — concentrated at 10Y</t>
-        </is>
+          <t>short (negative), concentrated at 10Y</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M7,Bootstrap!$D$3:$D$122)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -31220,8 +30675,34 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>dust — leave unhedged</t>
-        </is>
+          <t>dust — leave</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M8,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>7</v>
+      </c>
+      <c r="N9" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M9,Bootstrap!$D$3:$D$122)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -31235,648 +30716,799 @@
       <c r="D10" s="31" t="n"/>
       <c r="E10" s="31" t="n"/>
       <c r="F10" s="31" t="n"/>
+      <c r="G10" s="31" t="n"/>
+      <c r="H10" s="31" t="n"/>
+      <c r="I10" s="31" t="n"/>
+      <c r="J10" s="31" t="n"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>10</v>
+      </c>
+      <c r="N10" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M10,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="83" t="inlineStr">
         <is>
-          <t>•  Hedge points, not buckets — trade the 4 liquid benchmarks (2Y/3Y/5Y/10Y), not all 10 nodes.</t>
+          <t>•  Hedge liquid benchmarks (2Y/3Y/5Y/10Y), not every bucket.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="83" t="inlineStr">
         <is>
-          <t>•  Fold orphans into the nearest benchmark: 1Y→2Y, 4Y→5Y, 7Y→10Y. Size to null the group DV01.</t>
+          <t>•  Fold orphans into the nearest benchmark: 1Y→2Y, 4Y→5Y, 7Y→10Y.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="83" t="inlineStr">
         <is>
-          <t>•  Skip the sub-1Y dust — its bid/offer costs more than the risk it removes.</t>
-        </is>
-      </c>
+          <t>•  Skip the sub-1Y dust — bid/offer &gt; risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>3 · The trades  (4 swaps)</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="31" t="n"/>
+      <c r="I14" s="31" t="n"/>
+      <c r="J14" s="31" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
-        <is>
-          <t>3 · The trades  (4 swaps)</t>
-        </is>
-      </c>
-      <c r="B15" s="31" t="n"/>
-      <c r="C15" s="31" t="n"/>
-      <c r="D15" s="31" t="n"/>
-      <c r="E15" s="31" t="n"/>
-      <c r="F15" s="31" t="n"/>
-      <c r="H15" s="79" t="inlineStr">
-        <is>
-          <t>Benchmark annuity (curve)</t>
+      <c r="A15" s="50" t="inlineStr">
+        <is>
+          <t>Swap</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C15" s="50" t="inlineStr">
+        <is>
+          <t>Notional (bn)</t>
+        </is>
+      </c>
+      <c r="D15" s="50" t="inlineStr">
+        <is>
+          <t>Absorbs</t>
+        </is>
+      </c>
+      <c r="E15" s="50" t="inlineStr">
+        <is>
+          <t>Group DV01 (KRW/bp)</t>
+        </is>
+      </c>
+      <c r="F15" s="50" t="inlineStr">
+        <is>
+          <t>Annuity</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="50" t="inlineStr">
-        <is>
-          <t>Swap</t>
-        </is>
-      </c>
-      <c r="B16" s="50" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C16" s="50" t="inlineStr">
-        <is>
-          <t>Notional (bn)</t>
-        </is>
-      </c>
-      <c r="D16" s="50" t="inlineStr">
-        <is>
-          <t>Absorbs</t>
-        </is>
-      </c>
-      <c r="E16" s="50" t="inlineStr">
-        <is>
-          <t>Group DV01 (KRW/bp)</t>
-        </is>
-      </c>
-      <c r="F16" s="50" t="inlineStr">
-        <is>
-          <t>Annuity</t>
-        </is>
-      </c>
-      <c r="H16" s="51" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="I16" s="51" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="J16" s="51" t="inlineStr">
-        <is>
-          <t>Annuity</t>
-        </is>
+      <c r="A16" s="84" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B16" s="84">
+        <f>IF(E16&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C16" s="110">
+        <f>ABS(E16/(F16*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>1Y + 2Y</t>
+        </is>
+      </c>
+      <c r="E16" s="41">
+        <f>Sheet1!$B$9+Sheet1!$B$10</f>
+        <v/>
+      </c>
+      <c r="F16" s="86">
+        <f>$N$6</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="84" t="inlineStr">
         <is>
-          <t>2Y</t>
+          <t>3Y</t>
         </is>
       </c>
       <c r="B17" s="84">
         <f>IF(E17&gt;0,"Receive fixed","Pay fixed")</f>
         <v/>
       </c>
-      <c r="C17" s="85">
+      <c r="C17" s="110">
         <f>ABS(E17/(F17*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>1Y + 2Y</t>
+          <t>3Y</t>
         </is>
       </c>
       <c r="E17" s="41">
-        <f>Sheet1!$B$9+Sheet1!$B$10</f>
+        <f>Sheet1!$B$11</f>
         <v/>
       </c>
       <c r="F17" s="86">
-        <f>$J$17</f>
-        <v/>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>2</v>
-      </c>
-      <c r="J17" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I17,Bootstrap!$D$3:$D$122)</f>
+        <f>$N$7</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="84" t="inlineStr">
         <is>
-          <t>3Y</t>
+          <t>5Y</t>
         </is>
       </c>
       <c r="B18" s="84">
         <f>IF(E18&gt;0,"Receive fixed","Pay fixed")</f>
         <v/>
       </c>
-      <c r="C18" s="85">
+      <c r="C18" s="110">
         <f>ABS(E18/(F18*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>3Y</t>
+          <t>4Y + 5Y</t>
         </is>
       </c>
       <c r="E18" s="41">
-        <f>Sheet1!$B$11</f>
+        <f>Sheet1!$B$12+Sheet1!$B$13</f>
         <v/>
       </c>
       <c r="F18" s="86">
-        <f>$J$18</f>
-        <v/>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>3</v>
-      </c>
-      <c r="J18" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I18,Bootstrap!$D$3:$D$122)</f>
+        <f>$N$8</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="84" t="inlineStr">
         <is>
-          <t>5Y</t>
+          <t>10Y</t>
         </is>
       </c>
       <c r="B19" s="84">
         <f>IF(E19&gt;0,"Receive fixed","Pay fixed")</f>
         <v/>
       </c>
-      <c r="C19" s="85">
+      <c r="C19" s="110">
         <f>ABS(E19/(F19*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>4Y + 5Y</t>
+          <t>7Y + 10Y</t>
         </is>
       </c>
       <c r="E19" s="41">
-        <f>Sheet1!$B$12+Sheet1!$B$13</f>
+        <f>Sheet1!$B$14+Sheet1!$B$15</f>
         <v/>
       </c>
       <c r="F19" s="86">
-        <f>$J$19</f>
-        <v/>
-      </c>
-      <c r="H19" t="inlineStr">
+        <f>$N$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>4 · Cost to hedge &amp; liquidity   (KWSWNI tickers — confirm on GC S205 &gt; Table)</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="n"/>
+      <c r="C21" s="31" t="n"/>
+      <c r="D21" s="31" t="n"/>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="31" t="n"/>
+      <c r="G21" s="31" t="n"/>
+      <c r="H21" s="31" t="n"/>
+      <c r="I21" s="31" t="n"/>
+      <c r="J21" s="31" t="n"/>
+      <c r="K21" s="31" t="n"/>
+      <c r="L21" s="31" t="n"/>
+      <c r="M21" s="31" t="n"/>
+      <c r="N21" s="31" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="50" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B22" s="50" t="inlineStr">
+        <is>
+          <t>Ticker (edit)</t>
+        </is>
+      </c>
+      <c r="C22" s="50" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="D22" s="50" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="E22" s="50" t="inlineStr">
+        <is>
+          <t>Spread (bp)</t>
+        </is>
+      </c>
+      <c r="F22" s="50" t="inlineStr">
+        <is>
+          <t>Avg spr 1M (bp)</t>
+        </is>
+      </c>
+      <c r="G22" s="50" t="inlineStr">
+        <is>
+          <t>DV01 (KRW/bp)</t>
+        </is>
+      </c>
+      <c r="H22" s="50" t="inlineStr">
+        <is>
+          <t>Annuity</t>
+        </is>
+      </c>
+      <c r="I22" s="50" t="inlineStr">
+        <is>
+          <t>Notl (bn)</t>
+        </is>
+      </c>
+      <c r="J22" s="50" t="inlineStr">
+        <is>
+          <t>Cost (KRW)</t>
+        </is>
+      </c>
+      <c r="K22" s="50" t="inlineStr">
+        <is>
+          <t>Break-even (bp)</t>
+        </is>
+      </c>
+      <c r="L22" s="50" t="inlineStr">
+        <is>
+          <t>Vol USDmm</t>
+        </is>
+      </c>
+      <c r="M22" s="50" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="84" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B23" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI2 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C23" s="9">
+        <f>BDP(B23,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D23" s="9">
+        <f>BDP(B23,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E23" s="6">
+        <f>(D23-C23)*100</f>
+        <v/>
+      </c>
+      <c r="F23" s="6">
+        <f>(AVERAGE(BDH(B23,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B23,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="G23" s="41">
+        <f>E16</f>
+        <v/>
+      </c>
+      <c r="H23" s="86">
+        <f>F16</f>
+        <v/>
+      </c>
+      <c r="I23" s="93">
+        <f>C16</f>
+        <v/>
+      </c>
+      <c r="J23" s="41">
+        <f>I23*1000000000*H23*(E23/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K23" s="6">
+        <f>J23/ABS(G23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="94">
+        <f>IF(K23&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="84" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B24" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI3 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C24" s="9">
+        <f>BDP(B24,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D24" s="9">
+        <f>BDP(B24,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E24" s="6">
+        <f>(D24-C24)*100</f>
+        <v/>
+      </c>
+      <c r="F24" s="6">
+        <f>(AVERAGE(BDH(B24,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B24,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="G24" s="41">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="H24" s="86">
+        <f>F17</f>
+        <v/>
+      </c>
+      <c r="I24" s="93">
+        <f>C17</f>
+        <v/>
+      </c>
+      <c r="J24" s="41">
+        <f>I24*1000000000*H24*(E24/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K24" s="6">
+        <f>J24/ABS(G24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="94">
+        <f>IF(K24&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="84" t="inlineStr">
         <is>
           <t>5Y</t>
         </is>
       </c>
-      <c r="I19" t="n">
-        <v>5</v>
-      </c>
-      <c r="J19" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I19,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="84" t="inlineStr">
+      <c r="B25" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI5 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C25" s="9">
+        <f>BDP(B25,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D25" s="9">
+        <f>BDP(B25,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E25" s="6">
+        <f>(D25-C25)*100</f>
+        <v/>
+      </c>
+      <c r="F25" s="6">
+        <f>(AVERAGE(BDH(B25,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B25,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="G25" s="41">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="H25" s="86">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="I25" s="93">
+        <f>C18</f>
+        <v/>
+      </c>
+      <c r="J25" s="41">
+        <f>I25*1000000000*H25*(E25/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K25" s="6">
+        <f>J25/ABS(G25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="94">
+        <f>IF(K25&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="84" t="inlineStr">
         <is>
           <t>10Y</t>
         </is>
       </c>
-      <c r="B20" s="84">
-        <f>IF(E20&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-      <c r="C20" s="85">
-        <f>ABS(E20/(F20*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>7Y + 10Y</t>
-        </is>
-      </c>
-      <c r="E20" s="41">
-        <f>Sheet1!$B$14+Sheet1!$B$15</f>
-        <v/>
-      </c>
-      <c r="F20" s="86">
-        <f>$J$21</f>
-        <v/>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>7Y</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>7</v>
-      </c>
-      <c r="J20" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I20,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>10</v>
-      </c>
-      <c r="J21" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I21,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>4 · After the hedge</t>
-        </is>
-      </c>
-      <c r="B22" s="31" t="n"/>
-      <c r="C22" s="31" t="n"/>
-      <c r="D22" s="31" t="n"/>
-      <c r="E22" s="31" t="n"/>
-      <c r="F22" s="31" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="79" t="inlineStr">
-        <is>
-          <t>Grouped buckets 2Y/3Y/5Y/10Y</t>
-        </is>
-      </c>
-      <c r="C23" s="83" t="inlineStr">
-        <is>
-          <t>neutralized to 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="79" t="inlineStr">
-        <is>
-          <t>Residual DV01</t>
-        </is>
-      </c>
-      <c r="C24" s="87">
+      <c r="B26" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI10 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C26" s="9">
+        <f>BDP(B26,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D26" s="9">
+        <f>BDP(B26,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E26" s="6">
+        <f>(D26-C26)*100</f>
+        <v/>
+      </c>
+      <c r="F26" s="6">
+        <f>(AVERAGE(BDH(B26,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B26,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="G26" s="41">
+        <f>E19</f>
+        <v/>
+      </c>
+      <c r="H26" s="86">
+        <f>F19</f>
+        <v/>
+      </c>
+      <c r="I26" s="93">
+        <f>C19</f>
+        <v/>
+      </c>
+      <c r="J26" s="41">
+        <f>I26*1000000000*H26*(E26/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K26" s="6">
+        <f>J26/ABS(G26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="94">
+        <f>IF(K26&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="95" t="inlineStr">
+        <is>
+          <t>7Y split</t>
+        </is>
+      </c>
+      <c r="B27" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI7 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C27" s="97">
+        <f>BDP(B27,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D27" s="97">
+        <f>BDP(B27,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E27" s="105">
+        <f>(D27-C27)*100</f>
+        <v/>
+      </c>
+      <c r="F27" s="105">
+        <f>(AVERAGE(BDH(B27,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B27,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="G27" s="99">
+        <f>Sheet1!$B$14</f>
+        <v/>
+      </c>
+      <c r="H27" s="100">
+        <f>$N$9</f>
+        <v/>
+      </c>
+      <c r="I27" s="101">
+        <f>ABS(G27/(H27*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J27" s="99">
+        <f>I27*1000000000*H27*(E27/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K27" s="105">
+        <f>J27/ABS(G27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="102">
+        <f>IF(K27&lt;1,"TRADE","SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="95" t="inlineStr">
+        <is>
+          <t>Dust 3-9M</t>
+        </is>
+      </c>
+      <c r="B28" s="104" t="inlineStr">
+        <is>
+          <t>(front=CD/FRA, GC S205)</t>
+        </is>
+      </c>
+      <c r="C28" s="97">
+        <f>BDP(B28,"PX_BID")</f>
+        <v/>
+      </c>
+      <c r="D28" s="97">
+        <f>BDP(B28,"PX_ASK")</f>
+        <v/>
+      </c>
+      <c r="E28" s="105">
+        <f>(D28-C28)*100</f>
+        <v/>
+      </c>
+      <c r="F28" s="105">
+        <f>(AVERAGE(BDH(B28,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B28,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <v/>
+      </c>
+      <c r="G28" s="99">
         <f>Sheet1!$B$6+Sheet1!$B$7+Sheet1!$B$8</f>
         <v/>
       </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>sub-1Y dust only</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="79" t="inlineStr">
-        <is>
-          <t>Curve residual</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>small 7s10s (7Y folded into 10Y) — see option below</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="30" t="inlineStr">
-        <is>
-          <t>5 · Optional — split 7Y out (kills the 7s10s residual, +1 ticket)</t>
-        </is>
-      </c>
-      <c r="B27" s="31" t="n"/>
-      <c r="C27" s="31" t="n"/>
-      <c r="D27" s="31" t="n"/>
-      <c r="E27" s="31" t="n"/>
-      <c r="F27" s="31" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="50" t="inlineStr">
-        <is>
-          <t>Swap</t>
-        </is>
-      </c>
-      <c r="B28" s="50" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C28" s="50" t="inlineStr">
-        <is>
-          <t>Notional (bn)</t>
-        </is>
-      </c>
-      <c r="D28" s="50" t="inlineStr">
-        <is>
-          <t>Absorbs</t>
-        </is>
-      </c>
-      <c r="E28" s="50" t="inlineStr">
-        <is>
-          <t>Group DV01 (KRW/bp)</t>
-        </is>
-      </c>
-      <c r="F28" s="50" t="inlineStr">
-        <is>
-          <t>Annuity</t>
-        </is>
+      <c r="H28" s="100">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;1,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I28" s="101">
+        <f>ABS(G28/(H28*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J28" s="99">
+        <f>I28*1000000000*H28*(E28/2)*0.0001</f>
+        <v/>
+      </c>
+      <c r="K28" s="105">
+        <f>J28/ABS(G28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="102">
+        <f>IF(K28&lt;1,"TRADE","SKIP")</f>
+        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="84" t="inlineStr">
-        <is>
-          <t>7Y</t>
-        </is>
-      </c>
-      <c r="B29" s="84">
-        <f>IF(E29&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-      <c r="C29" s="88">
-        <f>ABS(E29/(F29*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>7Y</t>
-        </is>
-      </c>
-      <c r="E29" s="41">
-        <f>Sheet1!$B$14</f>
-        <v/>
-      </c>
-      <c r="F29" s="86">
-        <f>$J$20</f>
+      <c r="A29" s="79" t="inlineStr">
+        <is>
+          <t>TOTAL cost (4 trades)</t>
+        </is>
+      </c>
+      <c r="J29" s="91">
+        <f>SUM(J23:J26)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="84" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="B30" s="84">
-        <f>IF(E30&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-      <c r="C30" s="88">
-        <f>ABS(E30/(F30*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="E30" s="41">
-        <f>Sheet1!$B$15</f>
-        <v/>
-      </c>
-      <c r="F30" s="86">
-        <f>$J$21</f>
-        <v/>
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Yellow = inputs: exact ticker from GC S205 &gt; Table, and SDRV volume (USDmm) per tenor.</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Wired to Sheet1 (1Y=B9 … 10Y=B15). Drops into the master as-is; confirm Bootstrap!B3:B122/D3:D122 match.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>6 · Cost to hedge  (live bid/offer — computes on the terminal)</t>
-        </is>
-      </c>
-      <c r="B33" s="31" t="n"/>
-      <c r="C33" s="31" t="n"/>
-      <c r="D33" s="31" t="n"/>
-      <c r="E33" s="31" t="n"/>
-      <c r="F33" s="31" t="n"/>
-      <c r="G33" s="31" t="n"/>
-      <c r="H33" s="31" t="n"/>
+          <t>Break-even (bp) = cost / DV01 ≈ half the bid/offer. &lt;1bp -&gt; TRADE. Cross-check with SDRV volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="103" t="inlineStr">
+        <is>
+          <t>Commands:  GC S205 &lt;GO&gt; (tickers/curve) · SDRV &lt;GO&gt; Rates&gt;IRS/FRA&gt;KRW (volume) · SDR &lt;GO&gt; (trade drill).</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="50" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B34" s="50" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="C34" s="50" t="inlineStr">
-        <is>
-          <t>Bid</t>
-        </is>
-      </c>
-      <c r="D34" s="50" t="inlineStr">
-        <is>
-          <t>Ask</t>
-        </is>
-      </c>
-      <c r="E34" s="50" t="inlineStr">
-        <is>
-          <t>Spread (bp)</t>
-        </is>
-      </c>
-      <c r="F34" s="50" t="inlineStr">
-        <is>
-          <t>Cost (KRW)</t>
-        </is>
-      </c>
-      <c r="G34" s="50" t="inlineStr">
-        <is>
-          <t>Break-even (bp)</t>
-        </is>
-      </c>
-      <c r="H34" s="50" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>5 · After the hedge</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="n"/>
+      <c r="C34" s="31" t="n"/>
+      <c r="D34" s="31" t="n"/>
+      <c r="E34" s="31" t="n"/>
+      <c r="F34" s="31" t="n"/>
+      <c r="G34" s="31" t="n"/>
+      <c r="H34" s="31" t="n"/>
+      <c r="I34" s="31" t="n"/>
+      <c r="J34" s="31" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="84" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>KWSW2 Curncy</t>
-        </is>
-      </c>
-      <c r="C35" s="9">
-        <f>BDP(B35,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="D35" s="9">
-        <f>BDP(B35,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="E35" s="90">
-        <f>(D35-C35)*100</f>
-        <v/>
-      </c>
-      <c r="F35" s="41">
-        <f>C17*1000000000*F17*(E35/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="G35" s="9">
-        <f>F35/ABS(E17)</f>
-        <v/>
-      </c>
-      <c r="H35" s="84">
-        <f>IF(G35&lt;1,"TRADE","review")</f>
-        <v/>
+      <c r="A35" s="79" t="inlineStr">
+        <is>
+          <t>Grouped buckets 2Y/3Y/5Y/10Y</t>
+        </is>
+      </c>
+      <c r="C35" s="83" t="inlineStr">
+        <is>
+          <t>neutralized to 0</t>
+        </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="84" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>KWSW3 Curncy</t>
-        </is>
-      </c>
-      <c r="C36" s="9">
-        <f>BDP(B36,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="D36" s="9">
-        <f>BDP(B36,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="E36" s="90">
-        <f>(D36-C36)*100</f>
-        <v/>
-      </c>
-      <c r="F36" s="41">
-        <f>C18*1000000000*F18*(E36/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="G36" s="9">
-        <f>F36/ABS(E18)</f>
-        <v/>
-      </c>
-      <c r="H36" s="84">
-        <f>IF(G36&lt;1,"TRADE","review")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="84" t="inlineStr">
-        <is>
-          <t>5Y</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>KWSW5 Curncy</t>
-        </is>
-      </c>
-      <c r="C37" s="9">
-        <f>BDP(B37,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="D37" s="9">
-        <f>BDP(B37,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="E37" s="90">
-        <f>(D37-C37)*100</f>
-        <v/>
-      </c>
-      <c r="F37" s="41">
-        <f>C19*1000000000*F19*(E37/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="G37" s="9">
-        <f>F37/ABS(E19)</f>
-        <v/>
-      </c>
-      <c r="H37" s="84">
-        <f>IF(G37&lt;1,"TRADE","review")</f>
-        <v/>
+      <c r="A36" s="79" t="inlineStr">
+        <is>
+          <t>Residual DV01</t>
+        </is>
+      </c>
+      <c r="C36" s="87">
+        <f>Sheet1!$B$6+Sheet1!$B$7+Sheet1!$B$8</f>
+        <v/>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>sub-1Y dust only</t>
+        </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="84" t="inlineStr">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>6 · Optional — split 7Y out (kills 7s10s residual, +1 ticket)</t>
+        </is>
+      </c>
+      <c r="B38" s="31" t="n"/>
+      <c r="C38" s="31" t="n"/>
+      <c r="D38" s="31" t="n"/>
+      <c r="E38" s="31" t="n"/>
+      <c r="F38" s="31" t="n"/>
+      <c r="G38" s="31" t="n"/>
+      <c r="H38" s="31" t="n"/>
+      <c r="I38" s="31" t="n"/>
+      <c r="J38" s="31" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="50" t="inlineStr">
+        <is>
+          <t>Swap</t>
+        </is>
+      </c>
+      <c r="B39" s="50" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C39" s="50" t="inlineStr">
+        <is>
+          <t>Notional (bn)</t>
+        </is>
+      </c>
+      <c r="D39" s="50" t="inlineStr">
+        <is>
+          <t>Absorbs</t>
+        </is>
+      </c>
+      <c r="E39" s="50" t="inlineStr">
+        <is>
+          <t>Group DV01 (KRW/bp)</t>
+        </is>
+      </c>
+      <c r="F39" s="50" t="inlineStr">
+        <is>
+          <t>Annuity</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="84" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="B40" s="84">
+        <f>IF(E40&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C40" s="111">
+        <f>ABS(E40/(F40*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="E40" s="41">
+        <f>Sheet1!$B$14</f>
+        <v/>
+      </c>
+      <c r="F40" s="86">
+        <f>$N$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="84" t="inlineStr">
         <is>
           <t>10Y</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>KWSW10 Curncy</t>
-        </is>
-      </c>
-      <c r="C38" s="9">
-        <f>BDP(B38,"PX_BID")</f>
-        <v/>
-      </c>
-      <c r="D38" s="9">
-        <f>BDP(B38,"PX_ASK")</f>
-        <v/>
-      </c>
-      <c r="E38" s="90">
-        <f>(D38-C38)*100</f>
-        <v/>
-      </c>
-      <c r="F38" s="41">
-        <f>C20*1000000000*F20*(E38/2)*0.0001</f>
-        <v/>
-      </c>
-      <c r="G38" s="9">
-        <f>F38/ABS(E20)</f>
-        <v/>
-      </c>
-      <c r="H38" s="84">
-        <f>IF(G38&lt;1,"TRADE","review")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="79" t="inlineStr">
-        <is>
-          <t>TOTAL cost</t>
-        </is>
-      </c>
-      <c r="F39" s="91">
-        <f>SUM(F35:F38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>Break-even (bp) = cost / DV01: the adverse move that pays for the hedge. &lt;1bp -&gt; trade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>For the 7Y split / sub-1Y dust, run the same row with KWSW7 / KWCDC — break-even blows out.</t>
-        </is>
+      <c r="B41" s="84">
+        <f>IF(E41&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C41" s="111">
+        <f>ABS(E41/(F41*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="E41" s="41">
+        <f>Sheet1!$B$15</f>
+        <v/>
+      </c>
+      <c r="F41" s="86">
+        <f>$N$10</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Hedge cost table: self-contained refs + BDH date fix
- DV01 now sourced from KRD-v3 with ABSOLUTE refs (survives copy-paste to
  the master regardless of where the block lands); annuity inline via SUMIF.
  Fixes the broken =E16-style relative refs that showed DV01=4 / #DIV/0.
- BDH gets Dts=H so AVERAGE sees only values, not the date column (was
  returning date serials like 46198 in Avg spr 1M).
- IFERROR-wrap BDP/BDH/cost so a bad ticker degrades to n/a, not #VALUE;
  dust verdict hardcoded SKIP.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -31013,46 +31013,46 @@
         </is>
       </c>
       <c r="C23" s="9">
-        <f>BDP(B23,"PX_BID")</f>
+        <f>IFERROR(BDP(B23,"PX_BID"),"n/a")</f>
         <v/>
       </c>
       <c r="D23" s="9">
-        <f>BDP(B23,"PX_ASK")</f>
+        <f>IFERROR(BDP(B23,"PX_ASK"),"n/a")</f>
         <v/>
       </c>
       <c r="E23" s="6">
-        <f>(D23-C23)*100</f>
+        <f>IFERROR((D23-C23)*100,"n/a")</f>
         <v/>
       </c>
       <c r="F23" s="6">
-        <f>(AVERAGE(BDH(B23,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B23,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <f>IFERROR((AVERAGE(BDH(B23,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B23,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
         <v/>
       </c>
       <c r="G23" s="41">
-        <f>E16</f>
+        <f>'KRD-v3'!$B$15+'KRD-v3'!$B$16</f>
         <v/>
       </c>
       <c r="H23" s="86">
-        <f>F16</f>
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;2,Bootstrap!$D$3:$D$122)</f>
         <v/>
       </c>
       <c r="I23" s="93">
-        <f>C16</f>
+        <f>ABS(G23/(H23*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="J23" s="41">
-        <f>I23*1000000000*H23*(E23/2)*0.0001</f>
+        <f>IFERROR(I23*1000000000*H23*(E23/2)*0.0001,"n/a")</f>
         <v/>
       </c>
       <c r="K23" s="6">
-        <f>J23/ABS(G23)</f>
+        <f>IFERROR(J23/ABS(G23),"n/a")</f>
         <v/>
       </c>
       <c r="L23" s="104" t="n">
         <v>0</v>
       </c>
       <c r="M23" s="94">
-        <f>IF(K23&lt;1,"TRADE","SKIP")</f>
+        <f>IFERROR(IF(K23&lt;1,"TRADE","SKIP"),"SKIP")</f>
         <v/>
       </c>
     </row>
@@ -31068,46 +31068,46 @@
         </is>
       </c>
       <c r="C24" s="9">
-        <f>BDP(B24,"PX_BID")</f>
+        <f>IFERROR(BDP(B24,"PX_BID"),"n/a")</f>
         <v/>
       </c>
       <c r="D24" s="9">
-        <f>BDP(B24,"PX_ASK")</f>
+        <f>IFERROR(BDP(B24,"PX_ASK"),"n/a")</f>
         <v/>
       </c>
       <c r="E24" s="6">
-        <f>(D24-C24)*100</f>
+        <f>IFERROR((D24-C24)*100,"n/a")</f>
         <v/>
       </c>
       <c r="F24" s="6">
-        <f>(AVERAGE(BDH(B24,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B24,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <f>IFERROR((AVERAGE(BDH(B24,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B24,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
         <v/>
       </c>
       <c r="G24" s="41">
-        <f>E17</f>
+        <f>'KRD-v3'!$B$17</f>
         <v/>
       </c>
       <c r="H24" s="86">
-        <f>F17</f>
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;3,Bootstrap!$D$3:$D$122)</f>
         <v/>
       </c>
       <c r="I24" s="93">
-        <f>C17</f>
+        <f>ABS(G24/(H24*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="J24" s="41">
-        <f>I24*1000000000*H24*(E24/2)*0.0001</f>
+        <f>IFERROR(I24*1000000000*H24*(E24/2)*0.0001,"n/a")</f>
         <v/>
       </c>
       <c r="K24" s="6">
-        <f>J24/ABS(G24)</f>
+        <f>IFERROR(J24/ABS(G24),"n/a")</f>
         <v/>
       </c>
       <c r="L24" s="104" t="n">
         <v>0</v>
       </c>
       <c r="M24" s="94">
-        <f>IF(K24&lt;1,"TRADE","SKIP")</f>
+        <f>IFERROR(IF(K24&lt;1,"TRADE","SKIP"),"SKIP")</f>
         <v/>
       </c>
     </row>
@@ -31123,46 +31123,46 @@
         </is>
       </c>
       <c r="C25" s="9">
-        <f>BDP(B25,"PX_BID")</f>
+        <f>IFERROR(BDP(B25,"PX_BID"),"n/a")</f>
         <v/>
       </c>
       <c r="D25" s="9">
-        <f>BDP(B25,"PX_ASK")</f>
+        <f>IFERROR(BDP(B25,"PX_ASK"),"n/a")</f>
         <v/>
       </c>
       <c r="E25" s="6">
-        <f>(D25-C25)*100</f>
+        <f>IFERROR((D25-C25)*100,"n/a")</f>
         <v/>
       </c>
       <c r="F25" s="6">
-        <f>(AVERAGE(BDH(B25,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B25,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <f>IFERROR((AVERAGE(BDH(B25,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B25,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
         <v/>
       </c>
       <c r="G25" s="41">
-        <f>E18</f>
+        <f>'KRD-v3'!$B$18+'KRD-v3'!$B$19</f>
         <v/>
       </c>
       <c r="H25" s="86">
-        <f>F18</f>
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;5,Bootstrap!$D$3:$D$122)</f>
         <v/>
       </c>
       <c r="I25" s="93">
-        <f>C18</f>
+        <f>ABS(G25/(H25*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="J25" s="41">
-        <f>I25*1000000000*H25*(E25/2)*0.0001</f>
+        <f>IFERROR(I25*1000000000*H25*(E25/2)*0.0001,"n/a")</f>
         <v/>
       </c>
       <c r="K25" s="6">
-        <f>J25/ABS(G25)</f>
+        <f>IFERROR(J25/ABS(G25),"n/a")</f>
         <v/>
       </c>
       <c r="L25" s="104" t="n">
         <v>0</v>
       </c>
       <c r="M25" s="94">
-        <f>IF(K25&lt;1,"TRADE","SKIP")</f>
+        <f>IFERROR(IF(K25&lt;1,"TRADE","SKIP"),"SKIP")</f>
         <v/>
       </c>
     </row>
@@ -31178,46 +31178,46 @@
         </is>
       </c>
       <c r="C26" s="9">
-        <f>BDP(B26,"PX_BID")</f>
+        <f>IFERROR(BDP(B26,"PX_BID"),"n/a")</f>
         <v/>
       </c>
       <c r="D26" s="9">
-        <f>BDP(B26,"PX_ASK")</f>
+        <f>IFERROR(BDP(B26,"PX_ASK"),"n/a")</f>
         <v/>
       </c>
       <c r="E26" s="6">
-        <f>(D26-C26)*100</f>
+        <f>IFERROR((D26-C26)*100,"n/a")</f>
         <v/>
       </c>
       <c r="F26" s="6">
-        <f>(AVERAGE(BDH(B26,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B26,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <f>IFERROR((AVERAGE(BDH(B26,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B26,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
         <v/>
       </c>
       <c r="G26" s="41">
-        <f>E19</f>
+        <f>'KRD-v3'!$B$20+'KRD-v3'!$B$21</f>
         <v/>
       </c>
       <c r="H26" s="86">
-        <f>F19</f>
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;10,Bootstrap!$D$3:$D$122)</f>
         <v/>
       </c>
       <c r="I26" s="93">
-        <f>C19</f>
+        <f>ABS(G26/(H26*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="J26" s="41">
-        <f>I26*1000000000*H26*(E26/2)*0.0001</f>
+        <f>IFERROR(I26*1000000000*H26*(E26/2)*0.0001,"n/a")</f>
         <v/>
       </c>
       <c r="K26" s="6">
-        <f>J26/ABS(G26)</f>
+        <f>IFERROR(J26/ABS(G26),"n/a")</f>
         <v/>
       </c>
       <c r="L26" s="104" t="n">
         <v>0</v>
       </c>
       <c r="M26" s="94">
-        <f>IF(K26&lt;1,"TRADE","SKIP")</f>
+        <f>IFERROR(IF(K26&lt;1,"TRADE","SKIP"),"SKIP")</f>
         <v/>
       </c>
     </row>
@@ -31233,27 +31233,27 @@
         </is>
       </c>
       <c r="C27" s="97">
-        <f>BDP(B27,"PX_BID")</f>
+        <f>IFERROR(BDP(B27,"PX_BID"),"n/a")</f>
         <v/>
       </c>
       <c r="D27" s="97">
-        <f>BDP(B27,"PX_ASK")</f>
+        <f>IFERROR(BDP(B27,"PX_ASK"),"n/a")</f>
         <v/>
       </c>
       <c r="E27" s="105">
-        <f>(D27-C27)*100</f>
+        <f>IFERROR((D27-C27)*100,"n/a")</f>
         <v/>
       </c>
       <c r="F27" s="105">
-        <f>(AVERAGE(BDH(B27,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B27,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <f>IFERROR((AVERAGE(BDH(B27,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B27,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
         <v/>
       </c>
       <c r="G27" s="99">
-        <f>Sheet1!$B$14</f>
+        <f>'KRD-v3'!$B$20</f>
         <v/>
       </c>
       <c r="H27" s="100">
-        <f>$N$9</f>
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;7,Bootstrap!$D$3:$D$122)</f>
         <v/>
       </c>
       <c r="I27" s="101">
@@ -31261,18 +31261,18 @@
         <v/>
       </c>
       <c r="J27" s="99">
-        <f>I27*1000000000*H27*(E27/2)*0.0001</f>
+        <f>IFERROR(I27*1000000000*H27*(E27/2)*0.0001,"n/a")</f>
         <v/>
       </c>
       <c r="K27" s="105">
-        <f>J27/ABS(G27)</f>
+        <f>IFERROR(J27/ABS(G27),"n/a")</f>
         <v/>
       </c>
       <c r="L27" s="104" t="n">
         <v>0</v>
       </c>
       <c r="M27" s="102">
-        <f>IF(K27&lt;1,"TRADE","SKIP")</f>
+        <f>IFERROR(IF(K27&lt;1,"TRADE","SKIP"),"SKIP")</f>
         <v/>
       </c>
     </row>
@@ -31288,23 +31288,23 @@
         </is>
       </c>
       <c r="C28" s="97">
-        <f>BDP(B28,"PX_BID")</f>
+        <f>IFERROR(BDP(B28,"PX_BID"),"n/a")</f>
         <v/>
       </c>
       <c r="D28" s="97">
-        <f>BDP(B28,"PX_ASK")</f>
+        <f>IFERROR(BDP(B28,"PX_ASK"),"n/a")</f>
         <v/>
       </c>
       <c r="E28" s="105">
-        <f>(D28-C28)*100</f>
+        <f>IFERROR((D28-C28)*100,"n/a")</f>
         <v/>
       </c>
       <c r="F28" s="105">
-        <f>(AVERAGE(BDH(B28,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd")))-AVERAGE(BDH(B28,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"))))*100</f>
+        <f>IFERROR((AVERAGE(BDH(B28,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B28,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
         <v/>
       </c>
       <c r="G28" s="99">
-        <f>Sheet1!$B$6+Sheet1!$B$7+Sheet1!$B$8</f>
+        <f>'KRD-v3'!$B$12+'KRD-v3'!$B$13+'KRD-v3'!$B$14</f>
         <v/>
       </c>
       <c r="H28" s="100">
@@ -31316,19 +31316,20 @@
         <v/>
       </c>
       <c r="J28" s="99">
-        <f>I28*1000000000*H28*(E28/2)*0.0001</f>
+        <f>IFERROR(I28*1000000000*H28*(E28/2)*0.0001,"n/a")</f>
         <v/>
       </c>
       <c r="K28" s="105">
-        <f>J28/ABS(G28)</f>
+        <f>IFERROR(J28/ABS(G28),"n/a")</f>
         <v/>
       </c>
       <c r="L28" s="104" t="n">
         <v>0</v>
       </c>
-      <c r="M28" s="102">
-        <f>IF(K28&lt;1,"TRADE","SKIP")</f>
-        <v/>
+      <c r="M28" s="102" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Hedge: rebuild to mirror master layout, cost aligned at rows 44-51
Delta table B4:B23, risk 27-31, strategy 33-36, trades 40-43, cost 46-51 —
matching the master. Blotter DV01 reads the on-sheet delta table (B11:B17);
cost reads the blotter (E/F/C $40:$43) via ABSOLUTE refs so the two halves
can't misalign again. Skips (7Y=B16, dust=B8:B10) self-source. In the master
(delta from KRD-v2 at the same cells) the refs resolve to the real numbers.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -310,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -429,6 +429,9 @@
     <xf numFmtId="3" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="31" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="31" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -30522,907 +30525,407 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="78" t="inlineStr">
-        <is>
-          <t>Hedge proposal — KRW amortising IRS (10Y, HSBC receives fixed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Bucketed KRD hedged at liquid benchmarks; cost analysis (live bid/offer + SDRV volume) sits under the trades.</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Hedging the trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="51" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B3" s="51" t="inlineStr">
+        <is>
+          <t>dv01</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2D</t>
+        </is>
+      </c>
+      <c r="B4" s="55">
+        <f>'KRD-v3'!B8</f>
+        <v/>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>y1 exposure</t>
+        </is>
+      </c>
+      <c r="F4" s="55">
+        <f>$B$8+$B$9+$B$10+$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="B5" s="55">
+        <f>'KRD-v3'!B9</f>
+        <v/>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>y4-y10 exposure</t>
+        </is>
+      </c>
+      <c r="F5" s="55">
+        <f>$B$14+$B$15+$B$16+$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="B6" s="55">
+        <f>'KRD-v3'!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
+      <c r="B7" s="55">
+        <f>'KRD-v3'!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="B8" s="55">
+        <f>'KRD-v3'!B12</f>
+        <v/>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Original Trade</t>
+        </is>
+      </c>
+      <c r="F8" s="79" t="inlineStr">
+        <is>
+          <t>HSBC pay Float 3m CD, Q/A365</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6M</t>
+        </is>
+      </c>
+      <c r="B9" s="55">
+        <f>'KRD-v3'!B13</f>
+        <v/>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>fixed leg -&gt; back-end risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>9M</t>
+        </is>
+      </c>
+      <c r="B10" s="55">
+        <f>'KRD-v3'!B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1Y</t>
+        </is>
+      </c>
+      <c r="B11" s="55">
+        <f>'KRD-v3'!B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B12" s="55">
+        <f>'KRD-v3'!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B13" s="55">
+        <f>'KRD-v3'!B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4Y</t>
+        </is>
+      </c>
+      <c r="B14" s="55">
+        <f>'KRD-v3'!B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B15" s="55">
+        <f>'KRD-v3'!B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="B16" s="55">
+        <f>'KRD-v3'!B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B17" s="55">
+        <f>'KRD-v3'!B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>12Y</t>
+        </is>
+      </c>
+      <c r="B18" s="55">
+        <f>'KRD-v3'!B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>15Y</t>
+        </is>
+      </c>
+      <c r="B19" s="55">
+        <f>'KRD-v3'!B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>20Y</t>
+        </is>
+      </c>
+      <c r="B20" s="55">
+        <f>'KRD-v3'!B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>25Y</t>
+        </is>
+      </c>
+      <c r="B21" s="55">
+        <f>'KRD-v3'!B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>30Y</t>
+        </is>
+      </c>
+      <c r="B22" s="55">
+        <f>'KRD-v3'!B26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="79" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B23" s="87">
+        <f>'KRD-v3'!B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="112" t="inlineStr">
         <is>
           <t>1 · The risk</t>
         </is>
       </c>
-      <c r="B4" s="31" t="n"/>
-      <c r="C4" s="31" t="n"/>
-      <c r="D4" s="31" t="n"/>
-      <c r="E4" s="31" t="n"/>
-      <c r="F4" s="31" t="n"/>
-      <c r="G4" s="31" t="n"/>
-      <c r="H4" s="31" t="n"/>
-      <c r="I4" s="31" t="n"/>
-      <c r="J4" s="31" t="n"/>
-      <c r="L4" s="79" t="inlineStr">
-        <is>
-          <t>Benchmark annuity</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="79" t="inlineStr">
+      <c r="B27" s="113" t="n"/>
+      <c r="C27" s="113" t="n"/>
+      <c r="D27" s="113" t="n"/>
+      <c r="E27" s="113" t="n"/>
+      <c r="F27" s="113" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="79" t="inlineStr">
         <is>
           <t>Net DV01</t>
         </is>
       </c>
-      <c r="B5" s="107">
-        <f>Sheet1!$B$21</f>
-        <v/>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>KRW per bp — net receiver</t>
-        </is>
-      </c>
-      <c r="L5" s="51" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="M5" s="51" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N5" s="51" t="inlineStr">
-        <is>
-          <t>Annuity</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="79" t="inlineStr">
-        <is>
-          <t>Front 1Y–3Y</t>
-        </is>
-      </c>
-      <c r="B6" s="108">
-        <f>Sheet1!$B$9+Sheet1!$B$10+Sheet1!$B$11</f>
-        <v/>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>long (positive)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M6,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="79" t="inlineStr">
-        <is>
-          <t>Back 4Y–10Y</t>
-        </is>
-      </c>
-      <c r="B7" s="109">
-        <f>Sheet1!$B$12+Sheet1!$B$13+Sheet1!$B$14+Sheet1!$B$15</f>
-        <v/>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>short (negative), concentrated at 10Y</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M7,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="79" t="inlineStr">
-        <is>
-          <t>Sub-1Y (3M/6M/9M)</t>
-        </is>
-      </c>
-      <c r="B8" s="74">
-        <f>Sheet1!$B$6+Sheet1!$B$7+Sheet1!$B$8</f>
-        <v/>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>dust — leave</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>5Y</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N8" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M8,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>7Y</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
-        <v>7</v>
-      </c>
-      <c r="N9" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M9,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>2 · Strategy</t>
-        </is>
-      </c>
-      <c r="B10" s="31" t="n"/>
-      <c r="C10" s="31" t="n"/>
-      <c r="D10" s="31" t="n"/>
-      <c r="E10" s="31" t="n"/>
-      <c r="F10" s="31" t="n"/>
-      <c r="G10" s="31" t="n"/>
-      <c r="H10" s="31" t="n"/>
-      <c r="I10" s="31" t="n"/>
-      <c r="J10" s="31" t="n"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
-        <v>10</v>
-      </c>
-      <c r="N10" s="75">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;M10,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="83" t="inlineStr">
-        <is>
-          <t>•  Hedge liquid benchmarks (2Y/3Y/5Y/10Y), not every bucket.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="83" t="inlineStr">
-        <is>
-          <t>•  Fold orphans into the nearest benchmark: 1Y→2Y, 4Y→5Y, 7Y→10Y.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="83" t="inlineStr">
-        <is>
-          <t>•  Skip the sub-1Y dust — bid/offer &gt; risk.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>3 · The trades  (4 swaps)</t>
-        </is>
-      </c>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="31" t="n"/>
-      <c r="E14" s="31" t="n"/>
-      <c r="F14" s="31" t="n"/>
-      <c r="G14" s="31" t="n"/>
-      <c r="H14" s="31" t="n"/>
-      <c r="I14" s="31" t="n"/>
-      <c r="J14" s="31" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="50" t="inlineStr">
-        <is>
-          <t>Swap</t>
-        </is>
-      </c>
-      <c r="B15" s="50" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C15" s="50" t="inlineStr">
-        <is>
-          <t>Notional (bn)</t>
-        </is>
-      </c>
-      <c r="D15" s="50" t="inlineStr">
-        <is>
-          <t>Absorbs</t>
-        </is>
-      </c>
-      <c r="E15" s="50" t="inlineStr">
-        <is>
-          <t>Group DV01 (KRW/bp)</t>
-        </is>
-      </c>
-      <c r="F15" s="50" t="inlineStr">
-        <is>
-          <t>Annuity</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="84" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="B16" s="84">
-        <f>IF(E16&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-      <c r="C16" s="110">
-        <f>ABS(E16/(F16*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>1Y + 2Y</t>
-        </is>
-      </c>
-      <c r="E16" s="41">
-        <f>Sheet1!$B$9+Sheet1!$B$10</f>
-        <v/>
-      </c>
-      <c r="F16" s="86">
-        <f>$N$6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="84" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="B17" s="84">
-        <f>IF(E17&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-      <c r="C17" s="110">
-        <f>ABS(E17/(F17*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="E17" s="41">
-        <f>Sheet1!$B$11</f>
-        <v/>
-      </c>
-      <c r="F17" s="86">
-        <f>$N$7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="84" t="inlineStr">
-        <is>
-          <t>5Y</t>
-        </is>
-      </c>
-      <c r="B18" s="84">
-        <f>IF(E18&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-      <c r="C18" s="110">
-        <f>ABS(E18/(F18*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>4Y + 5Y</t>
-        </is>
-      </c>
-      <c r="E18" s="41">
-        <f>Sheet1!$B$12+Sheet1!$B$13</f>
-        <v/>
-      </c>
-      <c r="F18" s="86">
-        <f>$N$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="84" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="B19" s="84">
-        <f>IF(E19&gt;0,"Receive fixed","Pay fixed")</f>
-        <v/>
-      </c>
-      <c r="C19" s="110">
-        <f>ABS(E19/(F19*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>7Y + 10Y</t>
-        </is>
-      </c>
-      <c r="E19" s="41">
-        <f>Sheet1!$B$14+Sheet1!$B$15</f>
-        <v/>
-      </c>
-      <c r="F19" s="86">
-        <f>$N$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="30" t="inlineStr">
-        <is>
-          <t>4 · Cost to hedge &amp; liquidity   (KWSWNI tickers — confirm on GC S205 &gt; Table)</t>
-        </is>
-      </c>
-      <c r="B21" s="31" t="n"/>
-      <c r="C21" s="31" t="n"/>
-      <c r="D21" s="31" t="n"/>
-      <c r="E21" s="31" t="n"/>
-      <c r="F21" s="31" t="n"/>
-      <c r="G21" s="31" t="n"/>
-      <c r="H21" s="31" t="n"/>
-      <c r="I21" s="31" t="n"/>
-      <c r="J21" s="31" t="n"/>
-      <c r="K21" s="31" t="n"/>
-      <c r="L21" s="31" t="n"/>
-      <c r="M21" s="31" t="n"/>
-      <c r="N21" s="31" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="50" t="inlineStr">
-        <is>
-          <t>Tenor</t>
-        </is>
-      </c>
-      <c r="B22" s="50" t="inlineStr">
-        <is>
-          <t>Ticker (edit)</t>
-        </is>
-      </c>
-      <c r="C22" s="50" t="inlineStr">
-        <is>
-          <t>Bid</t>
-        </is>
-      </c>
-      <c r="D22" s="50" t="inlineStr">
-        <is>
-          <t>Ask</t>
-        </is>
-      </c>
-      <c r="E22" s="50" t="inlineStr">
-        <is>
-          <t>Spread (bp)</t>
-        </is>
-      </c>
-      <c r="F22" s="50" t="inlineStr">
-        <is>
-          <t>Avg spr 1M (bp)</t>
-        </is>
-      </c>
-      <c r="G22" s="50" t="inlineStr">
-        <is>
-          <t>DV01 (KRW/bp)</t>
-        </is>
-      </c>
-      <c r="H22" s="50" t="inlineStr">
-        <is>
-          <t>Annuity</t>
-        </is>
-      </c>
-      <c r="I22" s="50" t="inlineStr">
-        <is>
-          <t>Notl (bn)</t>
-        </is>
-      </c>
-      <c r="J22" s="50" t="inlineStr">
-        <is>
-          <t>Cost (KRW)</t>
-        </is>
-      </c>
-      <c r="K22" s="50" t="inlineStr">
-        <is>
-          <t>Break-even (bp)</t>
-        </is>
-      </c>
-      <c r="L22" s="50" t="inlineStr">
-        <is>
-          <t>Vol USDmm</t>
-        </is>
-      </c>
-      <c r="M22" s="50" t="inlineStr">
-        <is>
-          <t>Verdict</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="84" t="inlineStr">
-        <is>
-          <t>2Y</t>
-        </is>
-      </c>
-      <c r="B23" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI2 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="C23" s="9">
-        <f>IFERROR(BDP(B23,"PX_BID"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D23" s="9">
-        <f>IFERROR(BDP(B23,"PX_ASK"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E23" s="6">
-        <f>IFERROR((D23-C23)*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F23" s="6">
-        <f>IFERROR((AVERAGE(BDH(B23,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B23,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G23" s="41">
-        <f>'KRD-v3'!$B$15+'KRD-v3'!$B$16</f>
-        <v/>
-      </c>
-      <c r="H23" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;2,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I23" s="93">
-        <f>ABS(G23/(H23*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J23" s="41">
-        <f>IFERROR(I23*1000000000*H23*(E23/2)*0.0001,"n/a")</f>
-        <v/>
-      </c>
-      <c r="K23" s="6">
-        <f>IFERROR(J23/ABS(G23),"n/a")</f>
-        <v/>
-      </c>
-      <c r="L23" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="94">
-        <f>IFERROR(IF(K23&lt;1,"TRADE","SKIP"),"SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="84" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
-      <c r="B24" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI3 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="C24" s="9">
-        <f>IFERROR(BDP(B24,"PX_BID"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D24" s="9">
-        <f>IFERROR(BDP(B24,"PX_ASK"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E24" s="6">
-        <f>IFERROR((D24-C24)*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F24" s="6">
-        <f>IFERROR((AVERAGE(BDH(B24,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B24,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G24" s="41">
-        <f>'KRD-v3'!$B$17</f>
-        <v/>
-      </c>
-      <c r="H24" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;3,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I24" s="93">
-        <f>ABS(G24/(H24*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J24" s="41">
-        <f>IFERROR(I24*1000000000*H24*(E24/2)*0.0001,"n/a")</f>
-        <v/>
-      </c>
-      <c r="K24" s="6">
-        <f>IFERROR(J24/ABS(G24),"n/a")</f>
-        <v/>
-      </c>
-      <c r="L24" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="94">
-        <f>IFERROR(IF(K24&lt;1,"TRADE","SKIP"),"SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="84" t="inlineStr">
-        <is>
-          <t>5Y</t>
-        </is>
-      </c>
-      <c r="B25" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI5 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="C25" s="9">
-        <f>IFERROR(BDP(B25,"PX_BID"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D25" s="9">
-        <f>IFERROR(BDP(B25,"PX_ASK"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E25" s="6">
-        <f>IFERROR((D25-C25)*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F25" s="6">
-        <f>IFERROR((AVERAGE(BDH(B25,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B25,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G25" s="41">
-        <f>'KRD-v3'!$B$18+'KRD-v3'!$B$19</f>
-        <v/>
-      </c>
-      <c r="H25" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;5,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I25" s="93">
-        <f>ABS(G25/(H25*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J25" s="41">
-        <f>IFERROR(I25*1000000000*H25*(E25/2)*0.0001,"n/a")</f>
-        <v/>
-      </c>
-      <c r="K25" s="6">
-        <f>IFERROR(J25/ABS(G25),"n/a")</f>
-        <v/>
-      </c>
-      <c r="L25" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="94">
-        <f>IFERROR(IF(K25&lt;1,"TRADE","SKIP"),"SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="84" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
-      <c r="B26" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI10 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="C26" s="9">
-        <f>IFERROR(BDP(B26,"PX_BID"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D26" s="9">
-        <f>IFERROR(BDP(B26,"PX_ASK"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E26" s="6">
-        <f>IFERROR((D26-C26)*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F26" s="6">
-        <f>IFERROR((AVERAGE(BDH(B26,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B26,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G26" s="41">
-        <f>'KRD-v3'!$B$20+'KRD-v3'!$B$21</f>
-        <v/>
-      </c>
-      <c r="H26" s="86">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;10,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I26" s="93">
-        <f>ABS(G26/(H26*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J26" s="41">
-        <f>IFERROR(I26*1000000000*H26*(E26/2)*0.0001,"n/a")</f>
-        <v/>
-      </c>
-      <c r="K26" s="6">
-        <f>IFERROR(J26/ABS(G26),"n/a")</f>
-        <v/>
-      </c>
-      <c r="L26" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="94">
-        <f>IFERROR(IF(K26&lt;1,"TRADE","SKIP"),"SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="95" t="inlineStr">
-        <is>
-          <t>7Y split</t>
-        </is>
-      </c>
-      <c r="B27" s="104" t="inlineStr">
-        <is>
-          <t>KWSWNI7 BGN Curncy</t>
-        </is>
-      </c>
-      <c r="C27" s="97">
-        <f>IFERROR(BDP(B27,"PX_BID"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D27" s="97">
-        <f>IFERROR(BDP(B27,"PX_ASK"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E27" s="105">
-        <f>IFERROR((D27-C27)*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F27" s="105">
-        <f>IFERROR((AVERAGE(BDH(B27,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B27,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G27" s="99">
-        <f>'KRD-v3'!$B$20</f>
-        <v/>
-      </c>
-      <c r="H27" s="100">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;7,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I27" s="101">
-        <f>ABS(G27/(H27*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J27" s="99">
-        <f>IFERROR(I27*1000000000*H27*(E27/2)*0.0001,"n/a")</f>
-        <v/>
-      </c>
-      <c r="K27" s="105">
-        <f>IFERROR(J27/ABS(G27),"n/a")</f>
-        <v/>
-      </c>
-      <c r="L27" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="102">
-        <f>IFERROR(IF(K27&lt;1,"TRADE","SKIP"),"SKIP")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="95" t="inlineStr">
-        <is>
-          <t>Dust 3-9M</t>
-        </is>
-      </c>
-      <c r="B28" s="104" t="inlineStr">
-        <is>
-          <t>(front=CD/FRA, GC S205)</t>
-        </is>
-      </c>
-      <c r="C28" s="97">
-        <f>IFERROR(BDP(B28,"PX_BID"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="D28" s="97">
-        <f>IFERROR(BDP(B28,"PX_ASK"),"n/a")</f>
-        <v/>
-      </c>
-      <c r="E28" s="105">
-        <f>IFERROR((D28-C28)*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="F28" s="105">
-        <f>IFERROR((AVERAGE(BDH(B28,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B28,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
-        <v/>
-      </c>
-      <c r="G28" s="99">
-        <f>'KRD-v3'!$B$12+'KRD-v3'!$B$13+'KRD-v3'!$B$14</f>
-        <v/>
-      </c>
-      <c r="H28" s="100">
-        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;1,Bootstrap!$D$3:$D$122)</f>
-        <v/>
-      </c>
-      <c r="I28" s="101">
-        <f>ABS(G28/(H28*0.0001))/1000000000</f>
-        <v/>
-      </c>
-      <c r="J28" s="99">
-        <f>IFERROR(I28*1000000000*H28*(E28/2)*0.0001,"n/a")</f>
-        <v/>
-      </c>
-      <c r="K28" s="105">
-        <f>IFERROR(J28/ABS(G28),"n/a")</f>
-        <v/>
-      </c>
-      <c r="L28" s="104" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="102" t="inlineStr">
-        <is>
-          <t>SKIP</t>
+      <c r="B28" s="107">
+        <f>$B$23</f>
+        <v/>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>KRW per bp, net receiver</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="79" t="inlineStr">
         <is>
-          <t>TOTAL cost (4 trades)</t>
-        </is>
-      </c>
-      <c r="J29" s="91">
-        <f>SUM(J23:J26)</f>
-        <v/>
+          <t>Front 1Y–3Y</t>
+        </is>
+      </c>
+      <c r="B29" s="108">
+        <f>$B$11+$B$12+$B$13</f>
+        <v/>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>long (positive), pays if rates rise</t>
+        </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Yellow = inputs: exact ticker from GC S205 &gt; Table, and SDRV volume (USDmm) per tenor.</t>
+      <c r="A30" s="79" t="inlineStr">
+        <is>
+          <t>Back 4Y–10Y</t>
+        </is>
+      </c>
+      <c r="B30" s="109">
+        <f>$B$14+$B$15+$B$16+$B$17</f>
+        <v/>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>short (negative), concentrated at 10Y</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>Break-even (bp) = cost / DV01 ≈ half the bid/offer. &lt;1bp -&gt; TRADE. Cross-check with SDRV volume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="103" t="inlineStr">
-        <is>
-          <t>Commands:  GC S205 &lt;GO&gt; (tickers/curve) · SDRV &lt;GO&gt; Rates&gt;IRS/FRA&gt;KRW (volume) · SDR &lt;GO&gt; (trade drill).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="30" t="inlineStr">
-        <is>
-          <t>5 · After the hedge</t>
-        </is>
-      </c>
-      <c r="B34" s="31" t="n"/>
-      <c r="C34" s="31" t="n"/>
-      <c r="D34" s="31" t="n"/>
-      <c r="E34" s="31" t="n"/>
-      <c r="F34" s="31" t="n"/>
-      <c r="G34" s="31" t="n"/>
-      <c r="H34" s="31" t="n"/>
-      <c r="I34" s="31" t="n"/>
-      <c r="J34" s="31" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="79" t="inlineStr">
-        <is>
-          <t>Grouped buckets 2Y/3Y/5Y/10Y</t>
-        </is>
-      </c>
-      <c r="C35" s="83" t="inlineStr">
-        <is>
-          <t>neutralized to 0</t>
-        </is>
-      </c>
+      <c r="A31" s="79" t="inlineStr">
+        <is>
+          <t>Sub-1Y (3M/6M/9M)</t>
+        </is>
+      </c>
+      <c r="B31" s="74">
+        <f>$B$8+$B$9+$B$10</f>
+        <v/>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>miniscule</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="112" t="inlineStr">
+        <is>
+          <t>2 · Strategy</t>
+        </is>
+      </c>
+      <c r="B33" s="113" t="n"/>
+      <c r="C33" s="113" t="n"/>
+      <c r="D33" s="113" t="n"/>
+      <c r="E33" s="113" t="n"/>
+      <c r="F33" s="113" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="79" t="inlineStr">
-        <is>
-          <t>Residual DV01</t>
-        </is>
-      </c>
-      <c r="C36" s="87">
-        <f>Sheet1!$B$6+Sheet1!$B$7+Sheet1!$B$8</f>
-        <v/>
-      </c>
-      <c r="D36" s="7" t="inlineStr">
-        <is>
-          <t>sub-1Y dust only</t>
+      <c r="A36" s="83" t="inlineStr">
+        <is>
+          <t>Receive fixed front-end; Pay Fixed for long end; Short-end not worth hedging — doesn't even cover b/a</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="30" t="inlineStr">
-        <is>
-          <t>6 · Optional — split 7Y out (kills 7s10s residual, +1 ticket)</t>
-        </is>
-      </c>
-      <c r="B38" s="31" t="n"/>
-      <c r="C38" s="31" t="n"/>
-      <c r="D38" s="31" t="n"/>
-      <c r="E38" s="31" t="n"/>
-      <c r="F38" s="31" t="n"/>
-      <c r="G38" s="31" t="n"/>
-      <c r="H38" s="31" t="n"/>
-      <c r="I38" s="31" t="n"/>
-      <c r="J38" s="31" t="n"/>
+      <c r="A38" s="112" t="inlineStr">
+        <is>
+          <t>3 · The trades  --&gt;  4 swaps?</t>
+        </is>
+      </c>
+      <c r="B38" s="113" t="n"/>
+      <c r="C38" s="113" t="n"/>
+      <c r="D38" s="113" t="n"/>
+      <c r="E38" s="113" t="n"/>
+      <c r="F38" s="113" t="n"/>
+      <c r="H38" s="79" t="inlineStr">
+        <is>
+          <t>Benchmark annuity (curve)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="50" t="inlineStr">
@@ -31447,10 +30950,25 @@
       </c>
       <c r="E39" s="50" t="inlineStr">
         <is>
-          <t>Group DV01 (KRW/bp)</t>
+          <t>Group DV01 (KRW)</t>
         </is>
       </c>
       <c r="F39" s="50" t="inlineStr">
+        <is>
+          <t>Annuity SUM(DF*Tau)</t>
+        </is>
+      </c>
+      <c r="H39" s="51" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="I39" s="51" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="J39" s="51" t="inlineStr">
         <is>
           <t>Annuity</t>
         </is>
@@ -31459,57 +30977,601 @@
     <row r="40">
       <c r="A40" s="84" t="inlineStr">
         <is>
-          <t>7Y</t>
+          <t>2Y</t>
         </is>
       </c>
       <c r="B40" s="84">
         <f>IF(E40&gt;0,"Receive fixed","Pay fixed")</f>
         <v/>
       </c>
-      <c r="C40" s="111">
+      <c r="C40" s="110">
         <f>ABS(E40/(F40*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>7Y</t>
+          <t>1Y + 2Y</t>
         </is>
       </c>
       <c r="E40" s="41">
-        <f>Sheet1!$B$14</f>
+        <f>$B$11+$B$12</f>
         <v/>
       </c>
       <c r="F40" s="86">
-        <f>$N$9</f>
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;2,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I40,Bootstrap!$D$3:$D$122)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="84" t="inlineStr">
         <is>
-          <t>10Y</t>
+          <t>3Y</t>
         </is>
       </c>
       <c r="B41" s="84">
         <f>IF(E41&gt;0,"Receive fixed","Pay fixed")</f>
         <v/>
       </c>
-      <c r="C41" s="111">
+      <c r="C41" s="110">
         <f>ABS(E41/(F41*0.0001))/1000000000</f>
         <v/>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="E41" s="41">
+        <f>$B$13</f>
+        <v/>
+      </c>
+      <c r="F41" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;3,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>3</v>
+      </c>
+      <c r="J41" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I41,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="84" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B42" s="84">
+        <f>IF(E42&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C42" s="110">
+        <f>ABS(E42/(F42*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>4Y + 5Y</t>
+        </is>
+      </c>
+      <c r="E42" s="41">
+        <f>$B$14+$B$15</f>
+        <v/>
+      </c>
+      <c r="F42" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;5,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>5</v>
+      </c>
+      <c r="J42" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I42,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="84" t="inlineStr">
+        <is>
           <t>10Y</t>
         </is>
       </c>
-      <c r="E41" s="41">
-        <f>Sheet1!$B$15</f>
-        <v/>
-      </c>
-      <c r="F41" s="86">
-        <f>$N$10</f>
-        <v/>
+      <c r="B43" s="84">
+        <f>IF(E43&gt;0,"Receive fixed","Pay fixed")</f>
+        <v/>
+      </c>
+      <c r="C43" s="110">
+        <f>ABS(E43/(F43*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>7Y + 10Y</t>
+        </is>
+      </c>
+      <c r="E43" s="41">
+        <f>$B$16+$B$17</f>
+        <v/>
+      </c>
+      <c r="F43" s="86">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;10,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>7Y</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>7</v>
+      </c>
+      <c r="J43" s="75">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I43,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="112" t="inlineStr">
+        <is>
+          <t>4 · Hedge Cost Analysis</t>
+        </is>
+      </c>
+      <c r="B44" s="113" t="n"/>
+      <c r="C44" s="113" t="n"/>
+      <c r="D44" s="113" t="n"/>
+      <c r="E44" s="113" t="n"/>
+      <c r="F44" s="113" t="n"/>
+      <c r="G44" s="113" t="n"/>
+      <c r="H44" s="113" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="I44" s="113" t="n">
+        <v>10</v>
+      </c>
+      <c r="J44" s="114">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;I44,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="K44" s="113" t="n"/>
+      <c r="L44" s="113" t="n"/>
+      <c r="M44" s="113" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="50" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B45" s="50" t="inlineStr">
+        <is>
+          <t>Ticker (edit)</t>
+        </is>
+      </c>
+      <c r="C45" s="50" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="D45" s="50" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="E45" s="50" t="inlineStr">
+        <is>
+          <t>Spread (bp)</t>
+        </is>
+      </c>
+      <c r="F45" s="50" t="inlineStr">
+        <is>
+          <t>Avg spr 1M (bp)</t>
+        </is>
+      </c>
+      <c r="G45" s="50" t="inlineStr">
+        <is>
+          <t>DV01 (KRW)</t>
+        </is>
+      </c>
+      <c r="H45" s="50" t="inlineStr">
+        <is>
+          <t>Annuity</t>
+        </is>
+      </c>
+      <c r="I45" s="50" t="inlineStr">
+        <is>
+          <t>Notl (bn)</t>
+        </is>
+      </c>
+      <c r="J45" s="50" t="inlineStr">
+        <is>
+          <t>Cost (KRW)</t>
+        </is>
+      </c>
+      <c r="K45" s="50" t="inlineStr">
+        <is>
+          <t>Break-even (bp)</t>
+        </is>
+      </c>
+      <c r="L45" s="50" t="inlineStr">
+        <is>
+          <t>Vol USDmm</t>
+        </is>
+      </c>
+      <c r="M45" s="50" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="84" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B46" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI2 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C46" s="9">
+        <f>IFERROR(BDP(B46,"PX_BID"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D46" s="9">
+        <f>IFERROR(BDP(B46,"PX_ASK"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E46" s="6">
+        <f>IFERROR((D46-C46)*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F46" s="6">
+        <f>IFERROR((AVERAGE(BDH(B46,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B46,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G46" s="41">
+        <f>$E$40</f>
+        <v/>
+      </c>
+      <c r="H46" s="86">
+        <f>$F$40</f>
+        <v/>
+      </c>
+      <c r="I46" s="93">
+        <f>$C$40</f>
+        <v/>
+      </c>
+      <c r="J46" s="41">
+        <f>IFERROR(I46*1000000000*H46*(E46/2)*0.0001,"n/a")</f>
+        <v/>
+      </c>
+      <c r="K46" s="6">
+        <f>IFERROR(J46/ABS(G46),"n/a")</f>
+        <v/>
+      </c>
+      <c r="L46" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" s="94">
+        <f>IFERROR(IF(K46&lt;1,"TRADE","SKIP"),"SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="84" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B47" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI3 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C47" s="9">
+        <f>IFERROR(BDP(B47,"PX_BID"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D47" s="9">
+        <f>IFERROR(BDP(B47,"PX_ASK"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E47" s="6">
+        <f>IFERROR((D47-C47)*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F47" s="6">
+        <f>IFERROR((AVERAGE(BDH(B47,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B47,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G47" s="41">
+        <f>$E$41</f>
+        <v/>
+      </c>
+      <c r="H47" s="86">
+        <f>$F$41</f>
+        <v/>
+      </c>
+      <c r="I47" s="93">
+        <f>$C$41</f>
+        <v/>
+      </c>
+      <c r="J47" s="41">
+        <f>IFERROR(I47*1000000000*H47*(E47/2)*0.0001,"n/a")</f>
+        <v/>
+      </c>
+      <c r="K47" s="6">
+        <f>IFERROR(J47/ABS(G47),"n/a")</f>
+        <v/>
+      </c>
+      <c r="L47" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="94">
+        <f>IFERROR(IF(K47&lt;1,"TRADE","SKIP"),"SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="84" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B48" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI5 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C48" s="9">
+        <f>IFERROR(BDP(B48,"PX_BID"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D48" s="9">
+        <f>IFERROR(BDP(B48,"PX_ASK"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E48" s="6">
+        <f>IFERROR((D48-C48)*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F48" s="6">
+        <f>IFERROR((AVERAGE(BDH(B48,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B48,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G48" s="41">
+        <f>$E$42</f>
+        <v/>
+      </c>
+      <c r="H48" s="86">
+        <f>$F$42</f>
+        <v/>
+      </c>
+      <c r="I48" s="93">
+        <f>$C$42</f>
+        <v/>
+      </c>
+      <c r="J48" s="41">
+        <f>IFERROR(I48*1000000000*H48*(E48/2)*0.0001,"n/a")</f>
+        <v/>
+      </c>
+      <c r="K48" s="6">
+        <f>IFERROR(J48/ABS(G48),"n/a")</f>
+        <v/>
+      </c>
+      <c r="L48" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="94">
+        <f>IFERROR(IF(K48&lt;1,"TRADE","SKIP"),"SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="84" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B49" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI10 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C49" s="9">
+        <f>IFERROR(BDP(B49,"PX_BID"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D49" s="9">
+        <f>IFERROR(BDP(B49,"PX_ASK"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E49" s="6">
+        <f>IFERROR((D49-C49)*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F49" s="6">
+        <f>IFERROR((AVERAGE(BDH(B49,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B49,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G49" s="41">
+        <f>$E$43</f>
+        <v/>
+      </c>
+      <c r="H49" s="86">
+        <f>$F$43</f>
+        <v/>
+      </c>
+      <c r="I49" s="93">
+        <f>$C$43</f>
+        <v/>
+      </c>
+      <c r="J49" s="41">
+        <f>IFERROR(I49*1000000000*H49*(E49/2)*0.0001,"n/a")</f>
+        <v/>
+      </c>
+      <c r="K49" s="6">
+        <f>IFERROR(J49/ABS(G49),"n/a")</f>
+        <v/>
+      </c>
+      <c r="L49" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="94">
+        <f>IFERROR(IF(K49&lt;1,"TRADE","SKIP"),"SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="95" t="inlineStr">
+        <is>
+          <t>7Y split</t>
+        </is>
+      </c>
+      <c r="B50" s="104" t="inlineStr">
+        <is>
+          <t>KWSWNI7 BGN Curncy</t>
+        </is>
+      </c>
+      <c r="C50" s="97">
+        <f>IFERROR(BDP(B50,"PX_BID"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D50" s="97">
+        <f>IFERROR(BDP(B50,"PX_ASK"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E50" s="105">
+        <f>IFERROR((D50-C50)*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F50" s="105">
+        <f>IFERROR((AVERAGE(BDH(B50,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B50,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G50" s="99">
+        <f>$B$16</f>
+        <v/>
+      </c>
+      <c r="H50" s="100">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;7,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I50" s="101">
+        <f>ABS(G50/(H50*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J50" s="99">
+        <f>IFERROR(I50*1000000000*H50*(E50/2)*0.0001,"n/a")</f>
+        <v/>
+      </c>
+      <c r="K50" s="105">
+        <f>IFERROR(J50/ABS(G50),"n/a")</f>
+        <v/>
+      </c>
+      <c r="L50" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" s="102">
+        <f>IFERROR(IF(K50&lt;1,"TRADE","SKIP"),"SKIP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="95" t="inlineStr">
+        <is>
+          <t>Dust 3-9M</t>
+        </is>
+      </c>
+      <c r="B51" s="104" t="inlineStr">
+        <is>
+          <t>(front=CD/FRA, GC S205)</t>
+        </is>
+      </c>
+      <c r="C51" s="97">
+        <f>IFERROR(BDP(B51,"PX_BID"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D51" s="97">
+        <f>IFERROR(BDP(B51,"PX_ASK"),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E51" s="105">
+        <f>IFERROR((D51-C51)*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="F51" s="105">
+        <f>IFERROR((AVERAGE(BDH(B51,"PX_ASK",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H"))-AVERAGE(BDH(B51,"PX_BID",TEXT(TODAY()-30,"yyyymmdd"),TEXT(TODAY(),"yyyymmdd"),"Dts=H")))*100,"n/a")</f>
+        <v/>
+      </c>
+      <c r="G51" s="99">
+        <f>$B$8+$B$9+$B$10</f>
+        <v/>
+      </c>
+      <c r="H51" s="100">
+        <f>Quotes!$B$2*SUMIF(Bootstrap!$B$3:$B$122,"&lt;="&amp;1,Bootstrap!$D$3:$D$122)</f>
+        <v/>
+      </c>
+      <c r="I51" s="101">
+        <f>ABS(G51/(H51*0.0001))/1000000000</f>
+        <v/>
+      </c>
+      <c r="J51" s="99">
+        <f>IFERROR(I51*1000000000*H51*(E51/2)*0.0001,"n/a")</f>
+        <v/>
+      </c>
+      <c r="K51" s="105">
+        <f>IFERROR(J51/ABS(G51),"n/a")</f>
+        <v/>
+      </c>
+      <c r="L51" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="102" t="inlineStr">
+        <is>
+          <t>SKIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Break-even (bp) = cost / DV01 ≈ half the bid/offer. &lt;1bp -&gt; TRADE. Cross-check SDRV volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="103" t="inlineStr">
+        <is>
+          <t>Commands: GC S205 &lt;GO&gt; (tickers) · SDRV &lt;GO&gt; Rates&gt;IRS/FRA&gt;KRW (volume) · SDR &lt;GO&gt; (trades).</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add live Client Pricing sheet (par + hedge cost + margin -> client rate)
Mid par references Amort-Set-up!B12 (full-curve notional-weighted par, the
accurate 4.27% figure) not a 4-point recompute. Client DV01 = tau x
SUMPRODUCT(notional, DF) x 1bp. Hedge cost pulled live from Hedge!J46:J49
(BDP); FX via BDP(USDKRW); revenue a blue input. Outputs the two client
rates: par + hedge-cost-bp, and + target-revenue-bp.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -16,9 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD-v2" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KRD-v3" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hedge" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Pricing" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWPM" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Swap_Check" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +40,7 @@
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="36">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -235,6 +236,12 @@
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -310,7 +317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -432,6 +439,9 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="34" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="35" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1053,6 +1063,192 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="3" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="92" t="inlineStr">
+        <is>
+          <t>Client Pricing — fixed rate to show the client</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Client PAYS fixed, so mark UP from mid: par + hedging cost + target margin. Live off the curve, Hedge cost table, and BDP FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>Inputs (live)</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="n"/>
+      <c r="C4" s="31" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="79" t="inlineStr">
+        <is>
+          <t>Mid par — amortiser (full curve)</t>
+        </is>
+      </c>
+      <c r="C5" s="115">
+        <f>'Amort-Set-up'!$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>Client DV01 (KRW / bp)</t>
+        </is>
+      </c>
+      <c r="C6" s="55">
+        <f>Quotes!$B$2*SUMPRODUCT('Amort-Set-up'!$E$20:$E$59,'Amort-Set-up'!$D$20:$D$59)*0.0001</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="79" t="inlineStr">
+        <is>
+          <t>Hedge cost (KRW) — from Hedge sheet</t>
+        </is>
+      </c>
+      <c r="C7" s="55">
+        <f>SUM(Hedge!$J$46:$J$49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="79" t="inlineStr">
+        <is>
+          <t>USD / KRW  (BDP live)</t>
+        </is>
+      </c>
+      <c r="C8" s="70">
+        <f>BDP("USDKRW BGN Curncy","PX_LAST")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="79" t="inlineStr">
+        <is>
+          <t>Target revenue (USD)</t>
+        </is>
+      </c>
+      <c r="C9" s="116" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Conversion to bp</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="n"/>
+      <c r="C11" s="31" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="79" t="inlineStr">
+        <is>
+          <t>Hedging cost (bp)</t>
+        </is>
+      </c>
+      <c r="C12" s="70">
+        <f>C7/C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="79" t="inlineStr">
+        <is>
+          <t>Target revenue (bp)</t>
+        </is>
+      </c>
+      <c r="C13" s="70">
+        <f>(C9*C8)/C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Rate to show the client</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="79" t="inlineStr">
+        <is>
+          <t>(a) after hedging cost</t>
+        </is>
+      </c>
+      <c r="C16" s="117">
+        <f>C5+C12*0.0001</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="79" t="inlineStr">
+        <is>
+          <t>(b) after hedging cost + target revenue</t>
+        </is>
+      </c>
+      <c r="C17" s="117">
+        <f>C5+(C12+C13)*0.0001</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Client pays fixed -&gt; both rates sit ABOVE mid par (you charge the hedge slippage + your spread).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Hedge cost is HALF the bid/offer (cross once, hold to maturity). For full round-trip, double it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Par accuracy = the Quotes sheet. For a live par, wire Quotes rates to BDP (KWSWNI tickers) so the bootstrap flows current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="103" t="inlineStr">
+        <is>
+          <t>FX ticker: confirm "USDKRW BGN Curncy" on DES; 300k-&gt;bp scales with it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5793,7 +5989,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6753,7 +6949,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Client Pricing: quote table as input, linked to Hedge/Amort-Set-up
Kevin's two-way quotes are editable inputs (yellow); mid/spread/hedge-cost
compute per tenor from them x the linked hedge notional/annuity (Hedge!C40:F43).
Par links to Amort-Set-up!B12, DV01 to the amort notionals x DF. Outputs the
two client rates = par + hedge-cost-bp and + revenue-bp. FX an input (or =BDP).
Computes fully offline; slip-in ready.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -317,7 +317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -442,6 +442,9 @@
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="34" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="35" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="34" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="26" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="34" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1063,12 +1066,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="3" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1081,160 +1089,344 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Client PAYS fixed, so mark UP from mid: par + hedging cost + target margin. Live off the curve, Hedge cost table, and BDP FX.</t>
+          <t>Paste Kevin's two-way quotes below (yellow). Notionals/annuity link to Hedge; par &amp; DV01 to Amort-Set-up. Client pays fixed -&gt; mark up from mid.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="30" t="inlineStr">
         <is>
-          <t>Inputs (live)</t>
+          <t>1 · Market quotes  (input — paste Kevin's two-way)</t>
         </is>
       </c>
       <c r="B4" s="31" t="n"/>
       <c r="C4" s="31" t="n"/>
+      <c r="D4" s="31" t="n"/>
+      <c r="E4" s="31" t="n"/>
+      <c r="F4" s="31" t="n"/>
+      <c r="G4" s="31" t="n"/>
+      <c r="H4" s="31" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="79" t="inlineStr">
-        <is>
-          <t>Mid par — amortiser (full curve)</t>
-        </is>
-      </c>
-      <c r="C5" s="115">
-        <f>'Amort-Set-up'!$B$12</f>
-        <v/>
+      <c r="A5" s="50" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B5" s="50" t="inlineStr">
+        <is>
+          <t>Pay (offer)</t>
+        </is>
+      </c>
+      <c r="C5" s="50" t="inlineStr">
+        <is>
+          <t>Receive (bid)</t>
+        </is>
+      </c>
+      <c r="D5" s="50" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E5" s="50" t="inlineStr">
+        <is>
+          <t>Spread (bp)</t>
+        </is>
+      </c>
+      <c r="F5" s="50" t="inlineStr">
+        <is>
+          <t>Hedge notl (bn)</t>
+        </is>
+      </c>
+      <c r="G5" s="50" t="inlineStr">
+        <is>
+          <t>Annuity</t>
+        </is>
+      </c>
+      <c r="H5" s="50" t="inlineStr">
+        <is>
+          <t>Hedge cost (KRW)</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="79" t="inlineStr">
-        <is>
-          <t>Client DV01 (KRW / bp)</t>
-        </is>
-      </c>
-      <c r="C6" s="55">
-        <f>Quotes!$B$2*SUMPRODUCT('Amort-Set-up'!$E$20:$E$59,'Amort-Set-up'!$D$20:$D$59)*0.0001</f>
+      <c r="A6" s="84" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B6" s="118" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="C6" s="118" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="D6" s="9">
+        <f>(B6+C6)/2</f>
+        <v/>
+      </c>
+      <c r="E6" s="6">
+        <f>(B6-C6)*100</f>
+        <v/>
+      </c>
+      <c r="F6" s="90">
+        <f>Hedge!C40</f>
+        <v/>
+      </c>
+      <c r="G6" s="86">
+        <f>Hedge!F40</f>
+        <v/>
+      </c>
+      <c r="H6" s="41">
+        <f>F6*1000000000*G6*(E6/2)*0.0001</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="79" t="inlineStr">
-        <is>
-          <t>Hedge cost (KRW) — from Hedge sheet</t>
-        </is>
-      </c>
-      <c r="C7" s="55">
-        <f>SUM(Hedge!$J$46:$J$49)</f>
+      <c r="A7" s="84" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B7" s="118" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="C7" s="118" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="D7" s="9">
+        <f>(B7+C7)/2</f>
+        <v/>
+      </c>
+      <c r="E7" s="6">
+        <f>(B7-C7)*100</f>
+        <v/>
+      </c>
+      <c r="F7" s="90">
+        <f>Hedge!C41</f>
+        <v/>
+      </c>
+      <c r="G7" s="86">
+        <f>Hedge!F41</f>
+        <v/>
+      </c>
+      <c r="H7" s="41">
+        <f>F7*1000000000*G7*(E7/2)*0.0001</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="79" t="inlineStr">
-        <is>
-          <t>USD / KRW  (BDP live)</t>
-        </is>
-      </c>
-      <c r="C8" s="70">
-        <f>BDP("USDKRW BGN Curncy","PX_LAST")</f>
+      <c r="A8" s="84" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B8" s="118" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="C8" s="118" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="D8" s="9">
+        <f>(B8+C8)/2</f>
+        <v/>
+      </c>
+      <c r="E8" s="6">
+        <f>(B8-C8)*100</f>
+        <v/>
+      </c>
+      <c r="F8" s="90">
+        <f>Hedge!C42</f>
+        <v/>
+      </c>
+      <c r="G8" s="86">
+        <f>Hedge!F42</f>
+        <v/>
+      </c>
+      <c r="H8" s="41">
+        <f>F8*1000000000*G8*(E8/2)*0.0001</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="79" t="inlineStr">
-        <is>
-          <t>Target revenue (USD)</t>
-        </is>
-      </c>
-      <c r="C9" s="116" t="n">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>Conversion to bp</t>
-        </is>
-      </c>
-      <c r="B11" s="31" t="n"/>
-      <c r="C11" s="31" t="n"/>
+      <c r="A9" s="84" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B9" s="118" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="C9" s="118" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="D9" s="9">
+        <f>(B9+C9)/2</f>
+        <v/>
+      </c>
+      <c r="E9" s="6">
+        <f>(B9-C9)*100</f>
+        <v/>
+      </c>
+      <c r="F9" s="90">
+        <f>Hedge!C43</f>
+        <v/>
+      </c>
+      <c r="G9" s="86">
+        <f>Hedge!F43</f>
+        <v/>
+      </c>
+      <c r="H9" s="41">
+        <f>F9*1000000000*G9*(E9/2)*0.0001</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="79" t="inlineStr">
+        <is>
+          <t>TOTAL hedge cost</t>
+        </is>
+      </c>
+      <c r="H10" s="119">
+        <f>SUM(H6:H9)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="79" t="inlineStr">
-        <is>
-          <t>Hedging cost (bp)</t>
-        </is>
-      </c>
-      <c r="C12" s="70">
-        <f>C7/C6</f>
-        <v/>
-      </c>
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>2 · Pricing inputs  (linked)</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="31" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="79" t="inlineStr">
         <is>
-          <t>Target revenue (bp)</t>
-        </is>
-      </c>
-      <c r="C13" s="70">
-        <f>(C9*C8)/C6</f>
+          <t>Mid par — amortiser (full curve)</t>
+        </is>
+      </c>
+      <c r="C13" s="115">
+        <f>'Amort-Set-up'!$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="79" t="inlineStr">
+        <is>
+          <t>Client DV01 (KRW / bp)</t>
+        </is>
+      </c>
+      <c r="C14" s="55">
+        <f>Quotes!$B$2*SUMPRODUCT('Amort-Set-up'!$E$20:$E$59,'Amort-Set-up'!$D$20:$D$59)*0.0001</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
-        <is>
-          <t>Rate to show the client</t>
-        </is>
-      </c>
-      <c r="B15" s="31" t="n"/>
-      <c r="C15" s="31" t="n"/>
+      <c r="A15" s="79" t="inlineStr">
+        <is>
+          <t>Total hedge cost (KRW)</t>
+        </is>
+      </c>
+      <c r="C15" s="55">
+        <f>H10</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="79" t="inlineStr">
         <is>
-          <t>(a) after hedging cost</t>
-        </is>
-      </c>
-      <c r="C16" s="117">
-        <f>C5+C12*0.0001</f>
-        <v/>
+          <t>USD / KRW   (input, or =BDP)</t>
+        </is>
+      </c>
+      <c r="C16" s="120" t="n">
+        <v>1380</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="79" t="inlineStr">
         <is>
+          <t>Target revenue (USD)</t>
+        </is>
+      </c>
+      <c r="C17" s="116" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>3 · Conversion to bp</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="n"/>
+      <c r="C19" s="31" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="79" t="inlineStr">
+        <is>
+          <t>Hedging cost (bp)</t>
+        </is>
+      </c>
+      <c r="C20" s="70">
+        <f>C15/C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="79" t="inlineStr">
+        <is>
+          <t>Target revenue (bp)</t>
+        </is>
+      </c>
+      <c r="C21" s="70">
+        <f>(C17*C16)/C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>4 · Rate to show the client</t>
+        </is>
+      </c>
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="31" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="79" t="inlineStr">
+        <is>
+          <t>(a) after hedging cost</t>
+        </is>
+      </c>
+      <c r="C24" s="117">
+        <f>C13+C20*0.0001</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="79" t="inlineStr">
+        <is>
           <t>(b) after hedging cost + target revenue</t>
         </is>
       </c>
-      <c r="C17" s="117">
-        <f>C5+(C12+C13)*0.0001</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Client pays fixed -&gt; both rates sit ABOVE mid par (you charge the hedge slippage + your spread).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Hedge cost is HALF the bid/offer (cross once, hold to maturity). For full round-trip, double it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Par accuracy = the Quotes sheet. For a live par, wire Quotes rates to BDP (KWSWNI tickers) so the bootstrap flows current.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="103" t="inlineStr">
-        <is>
-          <t>FX ticker: confirm "USDKRW BGN Curncy" on DES; 300k-&gt;bp scales with it.</t>
+      <c r="C25" s="117">
+        <f>C13+(C20+C21)*0.0001</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Yellow = inputs. Client pays fixed, so both rates are ABOVE mid. Cost uses HALF the bid/offer (cross once).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="103" t="inlineStr">
+        <is>
+          <t>Links: notional/annuity &lt;- Hedge!C40:F43 · par &lt;- Amort-Set-up!B12 · DV01 &lt;- Amort-Set-up notionals x DF. FX: set =BDP("USDKRW BGN Curncy","PX_LAST").</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Client Pricing: expand to full working
Six visible sections: (1) quotes with hedge direction + executed side, (2)
hedge cost with every factor (notional x annuity x half-spread), (3) DV01
built from the annuity, (4) mid par, (5) cost->bp conversion with intermediate
KRW, (6) rate build-up waterfall. Inputs yellow; notionals/annuity/dir link to
Hedge, par/DV01 to Amort-Set-up. Computes offline.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
+++ b/bloomberg/KRW_IRS_Bootstrap_Book1.xlsx
@@ -40,7 +40,7 @@
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="38">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -242,6 +242,18 @@
       <color rgb="00006100"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -317,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -445,6 +457,13 @@
     <xf numFmtId="165" fontId="34" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="26" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="34" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="37" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1066,30 +1085,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="92" t="inlineStr">
         <is>
-          <t>Client Pricing — fixed rate to show the client</t>
+          <t>Client Pricing — fixed rate to show the client  (full working)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Paste Kevin's two-way quotes below (yellow). Notionals/annuity link to Hedge; par &amp; DV01 to Amort-Set-up. Client pays fixed -&gt; mark up from mid.</t>
+          <t>Client PAYS fixed -&gt; rate = mid par + hedging cost + margin. Quotes (yellow) are inputs; notionals/annuity/par/DV01 link to Hedge &amp; Amort-Set-up.</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1123,6 @@
       <c r="E4" s="31" t="n"/>
       <c r="F4" s="31" t="n"/>
       <c r="G4" s="31" t="n"/>
-      <c r="H4" s="31" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="50" t="inlineStr">
@@ -1135,17 +1152,12 @@
       </c>
       <c r="F5" s="50" t="inlineStr">
         <is>
-          <t>Hedge notl (bn)</t>
+          <t>Hedge dir</t>
         </is>
       </c>
       <c r="G5" s="50" t="inlineStr">
         <is>
-          <t>Annuity</t>
-        </is>
-      </c>
-      <c r="H5" s="50" t="inlineStr">
-        <is>
-          <t>Hedge cost (KRW)</t>
+          <t>You execute at</t>
         </is>
       </c>
     </row>
@@ -1169,16 +1181,12 @@
         <f>(B6-C6)*100</f>
         <v/>
       </c>
-      <c r="F6" s="90">
-        <f>Hedge!C40</f>
-        <v/>
-      </c>
-      <c r="G6" s="86">
-        <f>Hedge!F40</f>
-        <v/>
-      </c>
-      <c r="H6" s="41">
-        <f>F6*1000000000*G6*(E6/2)*0.0001</f>
+      <c r="F6" s="4">
+        <f>Hedge!B40</f>
+        <v/>
+      </c>
+      <c r="G6" s="9">
+        <f>IF(F6="Receive fixed",C6,B6)</f>
         <v/>
       </c>
     </row>
@@ -1202,16 +1210,12 @@
         <f>(B7-C7)*100</f>
         <v/>
       </c>
-      <c r="F7" s="90">
-        <f>Hedge!C41</f>
-        <v/>
-      </c>
-      <c r="G7" s="86">
-        <f>Hedge!F41</f>
-        <v/>
-      </c>
-      <c r="H7" s="41">
-        <f>F7*1000000000*G7*(E7/2)*0.0001</f>
+      <c r="F7" s="4">
+        <f>Hedge!B41</f>
+        <v/>
+      </c>
+      <c r="G7" s="9">
+        <f>IF(F7="Receive fixed",C7,B7)</f>
         <v/>
       </c>
     </row>
@@ -1235,16 +1239,12 @@
         <f>(B8-C8)*100</f>
         <v/>
       </c>
-      <c r="F8" s="90">
-        <f>Hedge!C42</f>
-        <v/>
-      </c>
-      <c r="G8" s="86">
-        <f>Hedge!F42</f>
-        <v/>
-      </c>
-      <c r="H8" s="41">
-        <f>F8*1000000000*G8*(E8/2)*0.0001</f>
+      <c r="F8" s="4">
+        <f>Hedge!B42</f>
+        <v/>
+      </c>
+      <c r="G8" s="9">
+        <f>IF(F8="Receive fixed",C8,B8)</f>
         <v/>
       </c>
     </row>
@@ -1268,165 +1268,418 @@
         <f>(B9-C9)*100</f>
         <v/>
       </c>
-      <c r="F9" s="90">
-        <f>Hedge!C43</f>
-        <v/>
-      </c>
-      <c r="G9" s="86">
-        <f>Hedge!F43</f>
-        <v/>
-      </c>
-      <c r="H9" s="41">
-        <f>F9*1000000000*G9*(E9/2)*0.0001</f>
+      <c r="F9" s="4">
+        <f>Hedge!B43</f>
+        <v/>
+      </c>
+      <c r="G9" s="9">
+        <f>IF(F9="Receive fixed",C9,B9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="79" t="inlineStr">
-        <is>
-          <t>TOTAL hedge cost</t>
-        </is>
-      </c>
-      <c r="H10" s="119">
-        <f>SUM(H6:H9)</f>
-        <v/>
+      <c r="A10" s="121" t="inlineStr">
+        <is>
+          <t>You cross HALF the bid/offer from mid: receive the bid on 2Y/3Y, pay the offer on 5Y/10Y.</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="30" t="inlineStr">
         <is>
-          <t>2 · Pricing inputs  (linked)</t>
+          <t>2 · Hedging cost  =  notional  x  annuity  x  ½·spread</t>
         </is>
       </c>
       <c r="B12" s="31" t="n"/>
       <c r="C12" s="31" t="n"/>
+      <c r="D12" s="31" t="n"/>
+      <c r="E12" s="31" t="n"/>
+      <c r="F12" s="31" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="79" t="inlineStr">
-        <is>
-          <t>Mid par — amortiser (full curve)</t>
-        </is>
-      </c>
-      <c r="C13" s="115">
-        <f>'Amort-Set-up'!$B$12</f>
-        <v/>
+      <c r="A13" s="50" t="inlineStr">
+        <is>
+          <t>Tenor</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="inlineStr">
+        <is>
+          <t>Notional (bn)</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="inlineStr">
+        <is>
+          <t>Annuity</t>
+        </is>
+      </c>
+      <c r="D13" s="50" t="inlineStr">
+        <is>
+          <t>½ spread (bp)</t>
+        </is>
+      </c>
+      <c r="E13" s="50" t="inlineStr">
+        <is>
+          <t>½ spread (dec)</t>
+        </is>
+      </c>
+      <c r="F13" s="50" t="inlineStr">
+        <is>
+          <t>Cost (KRW)</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="79" t="inlineStr">
-        <is>
-          <t>Client DV01 (KRW / bp)</t>
-        </is>
-      </c>
-      <c r="C14" s="55">
-        <f>Quotes!$B$2*SUMPRODUCT('Amort-Set-up'!$E$20:$E$59,'Amort-Set-up'!$D$20:$D$59)*0.0001</f>
+      <c r="A14" s="84" t="inlineStr">
+        <is>
+          <t>2Y</t>
+        </is>
+      </c>
+      <c r="B14" s="90">
+        <f>Hedge!C40</f>
+        <v/>
+      </c>
+      <c r="C14" s="86">
+        <f>Hedge!F40</f>
+        <v/>
+      </c>
+      <c r="D14" s="6">
+        <f>E6/2</f>
+        <v/>
+      </c>
+      <c r="E14" s="25">
+        <f>D14*0.0001</f>
+        <v/>
+      </c>
+      <c r="F14" s="41">
+        <f>B14*1000000000*C14*E14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="79" t="inlineStr">
-        <is>
-          <t>Total hedge cost (KRW)</t>
-        </is>
-      </c>
-      <c r="C15" s="55">
-        <f>H10</f>
+      <c r="A15" s="84" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
+      <c r="B15" s="90">
+        <f>Hedge!C41</f>
+        <v/>
+      </c>
+      <c r="C15" s="86">
+        <f>Hedge!F41</f>
+        <v/>
+      </c>
+      <c r="D15" s="6">
+        <f>E7/2</f>
+        <v/>
+      </c>
+      <c r="E15" s="25">
+        <f>D15*0.0001</f>
+        <v/>
+      </c>
+      <c r="F15" s="41">
+        <f>B15*1000000000*C15*E15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="79" t="inlineStr">
-        <is>
-          <t>USD / KRW   (input, or =BDP)</t>
-        </is>
-      </c>
-      <c r="C16" s="120" t="n">
-        <v>1380</v>
+      <c r="A16" s="84" t="inlineStr">
+        <is>
+          <t>5Y</t>
+        </is>
+      </c>
+      <c r="B16" s="90">
+        <f>Hedge!C42</f>
+        <v/>
+      </c>
+      <c r="C16" s="86">
+        <f>Hedge!F42</f>
+        <v/>
+      </c>
+      <c r="D16" s="6">
+        <f>E8/2</f>
+        <v/>
+      </c>
+      <c r="E16" s="25">
+        <f>D16*0.0001</f>
+        <v/>
+      </c>
+      <c r="F16" s="41">
+        <f>B16*1000000000*C16*E16</f>
+        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="79" t="inlineStr">
-        <is>
-          <t>Target revenue (USD)</t>
-        </is>
-      </c>
-      <c r="C17" s="116" t="n">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30" t="inlineStr">
-        <is>
-          <t>3 · Conversion to bp</t>
-        </is>
-      </c>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="31" t="n"/>
+      <c r="A17" s="84" t="inlineStr">
+        <is>
+          <t>10Y</t>
+        </is>
+      </c>
+      <c r="B17" s="90">
+        <f>Hedge!C43</f>
+        <v/>
+      </c>
+      <c r="C17" s="86">
+        <f>Hedge!F43</f>
+        <v/>
+      </c>
+      <c r="D17" s="6">
+        <f>E9/2</f>
+        <v/>
+      </c>
+      <c r="E17" s="25">
+        <f>D17*0.0001</f>
+        <v/>
+      </c>
+      <c r="F17" s="41">
+        <f>B17*1000000000*C17*E17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="79" t="inlineStr">
+        <is>
+          <t>TOTAL hedge cost</t>
+        </is>
+      </c>
+      <c r="F18" s="119">
+        <f>SUM(F14:F17)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="79" t="inlineStr">
-        <is>
-          <t>Hedging cost (bp)</t>
-        </is>
-      </c>
-      <c r="C20" s="70">
-        <f>C15/C14</f>
-        <v/>
-      </c>
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>3 · Client swap DV01  =  annuity  x  1bp</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="31" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="79" t="inlineStr">
         <is>
-          <t>Target revenue (bp)</t>
-        </is>
-      </c>
-      <c r="C21" s="70">
-        <f>(C17*C16)/C14</f>
-        <v/>
+          <t>Annuity (money) = Σ N × τ × DF</t>
+        </is>
+      </c>
+      <c r="C21" s="55">
+        <f>Quotes!$B$2*SUMPRODUCT('Amort-Set-up'!$E$20:$E$59,'Amort-Set-up'!$D$20:$D$59)</f>
+        <v/>
+      </c>
+      <c r="E21" s="121" t="inlineStr">
+        <is>
+          <t>τ = Quotes!B2 (0.25); N,DF from Amort-Set-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="79" t="inlineStr">
+        <is>
+          <t>DV01 = Annuity × 0.0001</t>
+        </is>
+      </c>
+      <c r="C22" s="122">
+        <f>C21*0.0001</f>
+        <v/>
+      </c>
+      <c r="E22" s="121" t="inlineStr">
+        <is>
+          <t>KRW of P&amp;L per 1bp on the client fixed rate</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="30" t="inlineStr">
         <is>
-          <t>4 · Rate to show the client</t>
+          <t>4 · Fair (mid) par — amortiser (full curve)</t>
         </is>
       </c>
       <c r="B23" s="31" t="n"/>
       <c r="C23" s="31" t="n"/>
+      <c r="D23" s="31" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="79" t="inlineStr">
         <is>
-          <t>(a) after hedging cost</t>
-        </is>
-      </c>
-      <c r="C24" s="117">
-        <f>C13+C20*0.0001</f>
+          <t>Mid par = SUMPRODUCT(N,fwd,DF) / SUMPRODUCT(N,DF)</t>
+        </is>
+      </c>
+      <c r="C24" s="123">
+        <f>'Amort-Set-up'!$B$12</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="79" t="inlineStr">
-        <is>
-          <t>(b) after hedging cost + target revenue</t>
-        </is>
-      </c>
-      <c r="C25" s="117">
-        <f>C13+(C20+C21)*0.0001</f>
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>5 · Convert costs to bp   (÷ DV01)</t>
+        </is>
+      </c>
+      <c r="B25" s="31" t="n"/>
+      <c r="C25" s="31" t="n"/>
+      <c r="D25" s="31" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="79" t="inlineStr">
+        <is>
+          <t>Total hedge cost (KRW)</t>
+        </is>
+      </c>
+      <c r="C26" s="55">
+        <f>F18</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Yellow = inputs. Client pays fixed, so both rates are ABOVE mid. Cost uses HALF the bid/offer (cross once).</t>
-        </is>
+      <c r="A27" s="79" t="inlineStr">
+        <is>
+          <t>→ Hedging cost (bp) = cost ÷ DV01</t>
+        </is>
+      </c>
+      <c r="C27" s="124">
+        <f>C26/C22</f>
+        <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="103" t="inlineStr">
-        <is>
-          <t>Links: notional/annuity &lt;- Hedge!C40:F43 · par &lt;- Amort-Set-up!B12 · DV01 &lt;- Amort-Set-up notionals x DF. FX: set =BDP("USDKRW BGN Curncy","PX_LAST").</t>
+      <c r="A28" s="79" t="inlineStr">
+        <is>
+          <t>Target revenue (USD)</t>
+        </is>
+      </c>
+      <c r="C28" s="116" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="79" t="inlineStr">
+        <is>
+          <t>USD / KRW   (input, or =BDP)</t>
+        </is>
+      </c>
+      <c r="C29" s="120" t="n">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="79" t="inlineStr">
+        <is>
+          <t>Revenue (KRW) = USD × FX</t>
+        </is>
+      </c>
+      <c r="C30" s="55">
+        <f>C28*C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="79" t="inlineStr">
+        <is>
+          <t>→ Revenue (bp) = KRW ÷ DV01</t>
+        </is>
+      </c>
+      <c r="C31" s="124">
+        <f>C30/C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>6 · Rate to show the client  (build-up)</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="n"/>
+      <c r="C33" s="31" t="n"/>
+      <c r="D33" s="31" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="50" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B34" s="50" t="inlineStr">
+        <is>
+          <t>+ bp</t>
+        </is>
+      </c>
+      <c r="C34" s="50" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="125" t="inlineStr">
+        <is>
+          <t>Mid par</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="126">
+        <f>C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="125" t="inlineStr">
+        <is>
+          <t>+ Hedging cost</t>
+        </is>
+      </c>
+      <c r="B36" s="6">
+        <f>C27</f>
+        <v/>
+      </c>
+      <c r="C36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="84">
+        <f> (a) after hedging cost</f>
+        <v/>
+      </c>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="127">
+        <f>C24+C27*0.0001</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="125" t="inlineStr">
+        <is>
+          <t>+ Target revenue</t>
+        </is>
+      </c>
+      <c r="B38" s="6">
+        <f>C31</f>
+        <v/>
+      </c>
+      <c r="C38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="84">
+        <f> (b) after cost + revenue</f>
+        <v/>
+      </c>
+      <c r="B39" s="4" t="n"/>
+      <c r="C39" s="127">
+        <f>C24+(C27+C31)*0.0001</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Client pays fixed -&gt; both rates sit ABOVE mid. Yellow = inputs. Links: Hedge (notl/annuity/dir), Amort-Set-up (par, DV01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="103" t="inlineStr">
+        <is>
+          <t>FX live: set C29 = BDP("USDKRW BGN Curncy","PX_LAST").  Full round-trip bid/offer: drop the /2 in section 2.</t>
         </is>
       </c>
     </row>

</xml_diff>